<commit_message>
Update fee collection and reports with new transactions
Added new fee payment records for multiple students in the 2024-25 and 2025-26 daywise collection CSVs, updated fee payment and due amounts in fees_collection.csv, and appended a new transaction in fee_transcation_atom_report.csv. Also, updated related Excel and Power BI files, removed an obsolete atom_report.xlsx, and moved atom_report.csv to the source_data directory.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL55"/>
+  <dimension ref="A1:AL60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8423,7 +8423,9 @@
       <c r="D53" t="n">
         <v>11350</v>
       </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="n">
+        <v>11350</v>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>18-Nov-2025 10:28:43</t>
@@ -8490,7 +8492,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W53" t="inlineStr">
@@ -8513,15 +8515,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA53" t="inlineStr"/>
-      <c r="AB53" t="inlineStr"/>
+      <c r="AA53" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB53" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC53" t="n">
         <v>0</v>
       </c>
       <c r="AD53" t="n">
         <v>0</v>
       </c>
-      <c r="AE53" t="inlineStr"/>
+      <c r="AE53" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF53" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -8563,13 +8571,19 @@
       <c r="D54" t="n">
         <v>16700</v>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="n">
+        <v>16700</v>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>18-Nov-2025 11:39:14</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>19-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -8630,7 +8644,7 @@
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W54" t="inlineStr">
@@ -8653,15 +8667,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA54" t="inlineStr"/>
-      <c r="AB54" t="inlineStr"/>
+      <c r="AA54" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB54" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC54" t="n">
         <v>0</v>
       </c>
       <c r="AD54" t="n">
         <v>0</v>
       </c>
-      <c r="AE54" t="inlineStr"/>
+      <c r="AE54" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF54" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -8703,13 +8723,19 @@
       <c r="D55" t="n">
         <v>8350</v>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="n">
+        <v>8350</v>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>18-Nov-2025 16:41:50</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>19-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -8770,7 +8796,7 @@
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W55" t="inlineStr">
@@ -8793,15 +8819,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA55" t="inlineStr"/>
-      <c r="AB55" t="inlineStr"/>
+      <c r="AA55" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB55" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC55" t="n">
         <v>0</v>
       </c>
       <c r="AD55" t="n">
         <v>0</v>
       </c>
-      <c r="AE55" t="inlineStr"/>
+      <c r="AE55" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF55" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -8827,6 +8859,718 @@
         </is>
       </c>
       <c r="AL55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>16507</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>POTNURU YELEENA</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>8374132397</v>
+      </c>
+      <c r="D56" t="n">
+        <v>8250</v>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>19-Nov-2025 09:11:28</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>eight thousand two hundred fifty</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O56" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P56" t="n">
+        <v>11000317376987</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>1763523653</v>
+      </c>
+      <c r="R56" t="n">
+        <v>704101659740</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr"/>
+      <c r="AC56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE56" t="inlineStr"/>
+      <c r="AF56" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG56" t="inlineStr"/>
+      <c r="AH56" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI56" t="n">
+        <v>18352</v>
+      </c>
+      <c r="AJ56" t="inlineStr">
+        <is>
+          <t>262241,263682</t>
+        </is>
+      </c>
+      <c r="AK56" t="inlineStr">
+        <is>
+          <t>2037,2040</t>
+        </is>
+      </c>
+      <c r="AL56" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>16754</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>BARLA VENKATA JOSHYA</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>7993557118</v>
+      </c>
+      <c r="D57" t="n">
+        <v>8250</v>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>19-Nov-2025 13:15:22</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>eight thousand two hundred fifty</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O57" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P57" t="n">
+        <v>11000317420497</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>1763538218</v>
+      </c>
+      <c r="R57" t="n">
+        <v>532374231246</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr"/>
+      <c r="AB57" t="inlineStr"/>
+      <c r="AC57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE57" t="inlineStr"/>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr"/>
+      <c r="AH57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI57" t="n">
+        <v>18267</v>
+      </c>
+      <c r="AJ57" t="inlineStr">
+        <is>
+          <t>262050,263641</t>
+        </is>
+      </c>
+      <c r="AK57" t="inlineStr">
+        <is>
+          <t>2037,2040</t>
+        </is>
+      </c>
+      <c r="AL57" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>17305</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>TUPAKULA DIA CHARLIE</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>9014136332</v>
+      </c>
+      <c r="D58" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>19-Nov-2025 15:31:01</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O58" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P58" t="n">
+        <v>11000317441689</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>1763546306</v>
+      </c>
+      <c r="R58" t="n">
+        <v>108599052932</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr"/>
+      <c r="AB58" t="inlineStr"/>
+      <c r="AC58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE58" t="inlineStr"/>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG58" t="inlineStr"/>
+      <c r="AH58" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI58" t="n">
+        <v>20014</v>
+      </c>
+      <c r="AJ58" t="inlineStr">
+        <is>
+          <t>263375</t>
+        </is>
+      </c>
+      <c r="AK58" t="inlineStr">
+        <is>
+          <t>2039</t>
+        </is>
+      </c>
+      <c r="AL58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>15855</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>GANGADA MOKSHITH</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>6305803494</v>
+      </c>
+      <c r="D59" t="n">
+        <v>8550</v>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>19-Nov-2025 16:38:21</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>eight thousand five hundred fifty</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O59" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P59" t="n">
+        <v>11000317451362</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>1763550487</v>
+      </c>
+      <c r="R59" t="n">
+        <v>355970292562</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr"/>
+      <c r="AB59" t="inlineStr"/>
+      <c r="AC59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE59" t="inlineStr"/>
+      <c r="AF59" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG59" t="inlineStr"/>
+      <c r="AH59" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI59" t="n">
+        <v>18628</v>
+      </c>
+      <c r="AJ59" t="inlineStr">
+        <is>
+          <t>262471,264025</t>
+        </is>
+      </c>
+      <c r="AK59" t="inlineStr">
+        <is>
+          <t>2037,2041</t>
+        </is>
+      </c>
+      <c r="AL59" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>17197</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>KONADA YASHASWINI</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>9881234227</v>
+      </c>
+      <c r="D60" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>19-Nov-2025 21:01:26</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O60" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P60" t="n">
+        <v>11000317484251</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>1763566147</v>
+      </c>
+      <c r="R60" t="n">
+        <v>108601056706</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr"/>
+      <c r="AB60" t="inlineStr"/>
+      <c r="AC60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE60" t="inlineStr"/>
+      <c r="AF60" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG60" t="inlineStr"/>
+      <c r="AH60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI60" t="n">
+        <v>19911</v>
+      </c>
+      <c r="AJ60" t="inlineStr">
+        <is>
+          <t>265070</t>
+        </is>
+      </c>
+      <c r="AK60" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL60" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update daywise fees collection data for Nov 2025
Added new fee collection records for various classes and dates in November 2025 across multiple CSV files. Also included new data files for online and annual fee collections for 2024-25 and 2025-26. These updates ensure the latest transactions are reflected in the output datasets.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL70"/>
+  <dimension ref="A1:AL77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9482,25 +9482,25 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>17197</v>
+        <v>15595</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>KONADA YASHASWINI</t>
+          <t>BHODEEP PEETALA</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>9881234227</v>
+        <v>9985727557</v>
       </c>
       <c r="D60" t="n">
-        <v>6750</v>
+        <v>9150</v>
       </c>
       <c r="E60" t="n">
-        <v>6750</v>
+        <v>9150</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>19-Nov-2025 21:01:26</t>
+          <t>19-Nov-2025 18:16:25</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -9510,7 +9510,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TRANSACTION IS SUCCESSFUL</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -9520,12 +9520,12 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>PREKGUKG</t>
+          <t>Multi</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>six thousand seven hundred fifty</t>
+          <t>nine thousand one hundred fifty</t>
         </is>
       </c>
       <c r="L60" t="n">
@@ -9543,13 +9543,13 @@
         <v>1234</v>
       </c>
       <c r="P60" t="n">
-        <v>11000317484251</v>
+        <v>11000317463739</v>
       </c>
       <c r="Q60" t="n">
-        <v>1763566147</v>
+        <v>1763555959</v>
       </c>
       <c r="R60" t="n">
-        <v>108601056706</v>
+        <v>1.01202532371806e+17</v>
       </c>
       <c r="S60" t="inlineStr">
         <is>
@@ -9563,17 +9563,17 @@
       </c>
       <c r="U60" t="inlineStr">
         <is>
-          <t>ICICI UPI QR</t>
+          <t>BANK OF BARODA FSS</t>
         </is>
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>SIBL0000899</t>
+          <t>IFSC0000000</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
@@ -9583,7 +9583,7 @@
       </c>
       <c r="Y60" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>DC</t>
         </is>
       </c>
       <c r="Z60" t="inlineStr">
@@ -9606,11 +9606,7 @@
       <c r="AE60" t="n">
         <v>5.9</v>
       </c>
-      <c r="AF60" t="inlineStr">
-        <is>
-          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
-        </is>
-      </c>
+      <c r="AF60" t="inlineStr"/>
       <c r="AG60" t="inlineStr"/>
       <c r="AH60" t="inlineStr">
         <is>
@@ -9618,42 +9614,48 @@
         </is>
       </c>
       <c r="AI60" t="n">
-        <v>19911</v>
+        <v>19130</v>
       </c>
       <c r="AJ60" t="inlineStr">
         <is>
-          <t>265070</t>
+          <t>262998,264501</t>
         </is>
       </c>
       <c r="AK60" t="inlineStr">
         <is>
-          <t>2047</t>
+          <t>2037,2043</t>
         </is>
       </c>
       <c r="AL60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>17290</v>
+        <v>17197</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PATNALA YOSHINI</t>
+          <t>KONADA YASHASWINI</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>9985244439</v>
+        <v>9881234227</v>
       </c>
       <c r="D61" t="n">
-        <v>8050</v>
-      </c>
-      <c r="E61" t="inlineStr"/>
+        <v>6750</v>
+      </c>
+      <c r="E61" t="n">
+        <v>6750</v>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>20-Nov-2025 08:47:32</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
+          <t>19-Nov-2025 21:01:26</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>20-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -9666,12 +9668,12 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>lVl</t>
+          <t>PREKGUKG</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>eight thousand fifty</t>
+          <t>six thousand seven hundred fifty</t>
         </is>
       </c>
       <c r="L61" t="n">
@@ -9689,13 +9691,13 @@
         <v>1234</v>
       </c>
       <c r="P61" t="n">
-        <v>11000317511572</v>
+        <v>11000317484251</v>
       </c>
       <c r="Q61" t="n">
-        <v>1763608577</v>
+        <v>1763566147</v>
       </c>
       <c r="R61" t="n">
-        <v>472308202173</v>
+        <v>108601056706</v>
       </c>
       <c r="S61" t="inlineStr">
         <is>
@@ -9714,7 +9716,7 @@
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W61" t="inlineStr">
@@ -9737,18 +9739,24 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA61" t="inlineStr"/>
-      <c r="AB61" t="inlineStr"/>
+      <c r="AA61" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB61" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC61" t="n">
         <v>0</v>
       </c>
       <c r="AD61" t="n">
         <v>0</v>
       </c>
-      <c r="AE61" t="inlineStr"/>
+      <c r="AE61" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF61" t="inlineStr">
         <is>
-          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
         </is>
       </c>
       <c r="AG61" t="inlineStr"/>
@@ -9758,46 +9766,48 @@
         </is>
       </c>
       <c r="AI61" t="n">
-        <v>20000</v>
+        <v>19911</v>
       </c>
       <c r="AJ61" t="inlineStr">
         <is>
-          <t>265468</t>
+          <t>265070</t>
         </is>
       </c>
       <c r="AK61" t="inlineStr">
         <is>
-          <t>2049</t>
-        </is>
-      </c>
-      <c r="AL61" t="inlineStr">
-        <is>
-          <t>UPI INTENT</t>
-        </is>
-      </c>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>17289</v>
+        <v>17290</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PATNALA DHARVIK</t>
+          <t>PATNALA YOSHINI</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>9985244439</v>
       </c>
       <c r="D62" t="n">
-        <v>7750</v>
-      </c>
-      <c r="E62" t="inlineStr"/>
+        <v>8050</v>
+      </c>
+      <c r="E62" t="n">
+        <v>8050</v>
+      </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>20-Nov-2025 08:49:38</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr"/>
+          <t>20-Nov-2025 08:47:32</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -9815,7 +9825,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>seven thousand seven hundred fifty</t>
+          <t>eight thousand fifty</t>
         </is>
       </c>
       <c r="L62" t="n">
@@ -9833,13 +9843,13 @@
         <v>1234</v>
       </c>
       <c r="P62" t="n">
-        <v>11000317511641</v>
+        <v>11000317511572</v>
       </c>
       <c r="Q62" t="n">
-        <v>1763608739</v>
+        <v>1763608577</v>
       </c>
       <c r="R62" t="n">
-        <v>962022877628</v>
+        <v>472308202173</v>
       </c>
       <c r="S62" t="inlineStr">
         <is>
@@ -9858,7 +9868,7 @@
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W62" t="inlineStr">
@@ -9881,15 +9891,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA62" t="inlineStr"/>
-      <c r="AB62" t="inlineStr"/>
+      <c r="AA62" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB62" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC62" t="n">
         <v>0</v>
       </c>
       <c r="AD62" t="n">
         <v>0</v>
       </c>
-      <c r="AE62" t="inlineStr"/>
+      <c r="AE62" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF62" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -9902,16 +9918,16 @@
         </is>
       </c>
       <c r="AI62" t="n">
-        <v>19999</v>
+        <v>20000</v>
       </c>
       <c r="AJ62" t="inlineStr">
         <is>
-          <t>265256</t>
+          <t>265468</t>
         </is>
       </c>
       <c r="AK62" t="inlineStr">
         <is>
-          <t>2048</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="AL62" t="inlineStr">
@@ -9922,26 +9938,32 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>15945</v>
+        <v>17289</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LEKSHITA LAASYA POTNURU</t>
+          <t>PATNALA DHARVIK</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>8801573949</v>
+        <v>9985244439</v>
       </c>
       <c r="D63" t="n">
-        <v>8850</v>
-      </c>
-      <c r="E63" t="inlineStr"/>
+        <v>7750</v>
+      </c>
+      <c r="E63" t="n">
+        <v>7750</v>
+      </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>20-Nov-2025 11:46:10</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr"/>
+          <t>20-Nov-2025 08:49:38</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -9959,7 +9981,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>eight thousand eight hundred fifty</t>
+          <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
       <c r="L63" t="n">
@@ -9977,13 +9999,13 @@
         <v>1234</v>
       </c>
       <c r="P63" t="n">
-        <v>11000317537894</v>
+        <v>11000317511641</v>
       </c>
       <c r="Q63" t="n">
-        <v>1763619330</v>
+        <v>1763608739</v>
       </c>
       <c r="R63" t="n">
-        <v>881654640858</v>
+        <v>962022877628</v>
       </c>
       <c r="S63" t="inlineStr">
         <is>
@@ -10002,7 +10024,7 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W63" t="inlineStr">
@@ -10025,15 +10047,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA63" t="inlineStr"/>
-      <c r="AB63" t="inlineStr"/>
+      <c r="AA63" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB63" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC63" t="n">
         <v>0</v>
       </c>
       <c r="AD63" t="n">
         <v>0</v>
       </c>
-      <c r="AE63" t="inlineStr"/>
+      <c r="AE63" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF63" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -10046,16 +10074,16 @@
         </is>
       </c>
       <c r="AI63" t="n">
-        <v>18833</v>
+        <v>19999</v>
       </c>
       <c r="AJ63" t="inlineStr">
         <is>
-          <t>262775,264278</t>
+          <t>265256</t>
         </is>
       </c>
       <c r="AK63" t="inlineStr">
         <is>
-          <t>2037,2042</t>
+          <t>2048</t>
         </is>
       </c>
       <c r="AL63" t="inlineStr">
@@ -10066,26 +10094,32 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>17277</v>
+        <v>15945</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EDUBILLI MAHASWIN</t>
+          <t>LEKSHITA LAASYA POTNURU</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>9618641662</v>
+        <v>8801573949</v>
       </c>
       <c r="D64" t="n">
-        <v>6750</v>
-      </c>
-      <c r="E64" t="inlineStr"/>
+        <v>8850</v>
+      </c>
+      <c r="E64" t="n">
+        <v>8850</v>
+      </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>20-Nov-2025 13:47:57</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr"/>
+          <t>20-Nov-2025 11:46:10</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -10098,12 +10132,12 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>PREKGUKG</t>
+          <t>lVl</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>six thousand seven hundred fifty</t>
+          <t>eight thousand eight hundred fifty</t>
         </is>
       </c>
       <c r="L64" t="n">
@@ -10121,13 +10155,13 @@
         <v>1234</v>
       </c>
       <c r="P64" t="n">
-        <v>11000317559740</v>
+        <v>11000317537894</v>
       </c>
       <c r="Q64" t="n">
-        <v>1763626601</v>
+        <v>1763619330</v>
       </c>
       <c r="R64" t="n">
-        <v>108604250147</v>
+        <v>881654640858</v>
       </c>
       <c r="S64" t="inlineStr">
         <is>
@@ -10146,7 +10180,7 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W64" t="inlineStr">
@@ -10169,18 +10203,24 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA64" t="inlineStr"/>
-      <c r="AB64" t="inlineStr"/>
+      <c r="AA64" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB64" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC64" t="n">
         <v>0</v>
       </c>
       <c r="AD64" t="n">
         <v>0</v>
       </c>
-      <c r="AE64" t="inlineStr"/>
+      <c r="AE64" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF64" t="inlineStr">
         <is>
-          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
         </is>
       </c>
       <c r="AG64" t="inlineStr"/>
@@ -10190,42 +10230,52 @@
         </is>
       </c>
       <c r="AI64" t="n">
-        <v>19988</v>
+        <v>18833</v>
       </c>
       <c r="AJ64" t="inlineStr">
         <is>
-          <t>263475</t>
+          <t>262775,264278</t>
         </is>
       </c>
       <c r="AK64" t="inlineStr">
         <is>
-          <t>2039</t>
-        </is>
-      </c>
-      <c r="AL64" t="inlineStr"/>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="AL64" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>14888</v>
+        <v>17277</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SHAIK GOUSIA NASRIN</t>
+          <t>EDUBILLI MAHASWIN</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>7207749584</v>
+        <v>9618641662</v>
       </c>
       <c r="D65" t="n">
-        <v>11250</v>
-      </c>
-      <c r="E65" t="inlineStr"/>
+        <v>6750</v>
+      </c>
+      <c r="E65" t="n">
+        <v>6750</v>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>20-Nov-2025 14:40:36</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr"/>
+          <t>20-Nov-2025 13:47:57</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -10238,12 +10288,12 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Multi</t>
+          <t>PREKGUKG</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>eleven thousand two hundred fifty</t>
+          <t>six thousand seven hundred fifty</t>
         </is>
       </c>
       <c r="L65" t="n">
@@ -10261,13 +10311,13 @@
         <v>1234</v>
       </c>
       <c r="P65" t="n">
-        <v>11000317567806</v>
+        <v>11000317559740</v>
       </c>
       <c r="Q65" t="n">
-        <v>1763629785</v>
+        <v>1763626601</v>
       </c>
       <c r="R65" t="n">
-        <v>108604632984</v>
+        <v>108604250147</v>
       </c>
       <c r="S65" t="inlineStr">
         <is>
@@ -10286,12 +10336,12 @@
       </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>IFSC0000000</t>
+          <t>SIBL0000899</t>
         </is>
       </c>
       <c r="X65" t="inlineStr">
@@ -10309,16 +10359,26 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA65" t="inlineStr"/>
-      <c r="AB65" t="inlineStr"/>
+      <c r="AA65" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB65" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC65" t="n">
         <v>0</v>
       </c>
       <c r="AD65" t="n">
         <v>0</v>
       </c>
-      <c r="AE65" t="inlineStr"/>
-      <c r="AF65" t="inlineStr"/>
+      <c r="AE65" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
       <c r="AG65" t="inlineStr"/>
       <c r="AH65" t="inlineStr">
         <is>
@@ -10326,42 +10386,48 @@
         </is>
       </c>
       <c r="AI65" t="n">
-        <v>19200</v>
+        <v>19988</v>
       </c>
       <c r="AJ65" t="inlineStr">
         <is>
-          <t>263115,264618</t>
+          <t>263475</t>
         </is>
       </c>
       <c r="AK65" t="inlineStr">
         <is>
-          <t>2037,2044</t>
+          <t>2039</t>
         </is>
       </c>
       <c r="AL65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>16983</v>
+        <v>14888</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NITHYA EMERALD THOTA</t>
+          <t>SHAIK GOUSIA NASRIN</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>8919560551</v>
+        <v>7207749584</v>
       </c>
       <c r="D66" t="n">
-        <v>8550</v>
-      </c>
-      <c r="E66" t="inlineStr"/>
+        <v>11250</v>
+      </c>
+      <c r="E66" t="n">
+        <v>11250</v>
+      </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>20-Nov-2025 17:01:38</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr"/>
+          <t>20-Nov-2025 14:40:36</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -10374,12 +10440,12 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>lVl</t>
+          <t>Multi</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>eight thousand five hundred fifty</t>
+          <t>eleven thousand two hundred fifty</t>
         </is>
       </c>
       <c r="L66" t="n">
@@ -10397,13 +10463,13 @@
         <v>1234</v>
       </c>
       <c r="P66" t="n">
-        <v>11000317588170</v>
+        <v>11000317567806</v>
       </c>
       <c r="Q66" t="n">
-        <v>1763636615</v>
+        <v>1763629785</v>
       </c>
       <c r="R66" t="n">
-        <v>108605493967</v>
+        <v>108604632984</v>
       </c>
       <c r="S66" t="inlineStr">
         <is>
@@ -10422,12 +10488,12 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>SIBL0000899</t>
+          <t>IFSC0000000</t>
         </is>
       </c>
       <c r="X66" t="inlineStr">
@@ -10445,20 +10511,22 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA66" t="inlineStr"/>
-      <c r="AB66" t="inlineStr"/>
+      <c r="AA66" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB66" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC66" t="n">
         <v>0</v>
       </c>
       <c r="AD66" t="n">
         <v>0</v>
       </c>
-      <c r="AE66" t="inlineStr"/>
-      <c r="AF66" t="inlineStr">
-        <is>
-          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
-        </is>
-      </c>
+      <c r="AE66" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF66" t="inlineStr"/>
       <c r="AG66" t="inlineStr"/>
       <c r="AH66" t="inlineStr">
         <is>
@@ -10466,42 +10534,48 @@
         </is>
       </c>
       <c r="AI66" t="n">
-        <v>18526</v>
+        <v>19200</v>
       </c>
       <c r="AJ66" t="inlineStr">
         <is>
-          <t>262171,263959</t>
+          <t>263115,264618</t>
         </is>
       </c>
       <c r="AK66" t="inlineStr">
         <is>
-          <t>2037,2041</t>
+          <t>2037,2044</t>
         </is>
       </c>
       <c r="AL66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>16580</v>
+        <v>16983</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CHANUKYA APPALACHARYULU MUNUBARTHI</t>
+          <t>NITHYA EMERALD THOTA</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>9908906244</v>
+        <v>8919560551</v>
       </c>
       <c r="D67" t="n">
-        <v>8850</v>
-      </c>
-      <c r="E67" t="inlineStr"/>
+        <v>8550</v>
+      </c>
+      <c r="E67" t="n">
+        <v>8550</v>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>20-Nov-2025 17:12:41</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr"/>
+          <t>20-Nov-2025 17:01:38</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -10519,7 +10593,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>eight thousand eight hundred fifty</t>
+          <t>eight thousand five hundred fifty</t>
         </is>
       </c>
       <c r="L67" t="n">
@@ -10537,13 +10611,13 @@
         <v>1234</v>
       </c>
       <c r="P67" t="n">
-        <v>11000317589448</v>
+        <v>11000317588170</v>
       </c>
       <c r="Q67" t="n">
-        <v>1763638742</v>
+        <v>1763636615</v>
       </c>
       <c r="R67" t="n">
-        <v>108605556686</v>
+        <v>108605493967</v>
       </c>
       <c r="S67" t="inlineStr">
         <is>
@@ -10562,7 +10636,7 @@
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W67" t="inlineStr">
@@ -10585,15 +10659,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA67" t="inlineStr"/>
-      <c r="AB67" t="inlineStr"/>
+      <c r="AA67" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB67" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC67" t="n">
         <v>0</v>
       </c>
       <c r="AD67" t="n">
         <v>0</v>
       </c>
-      <c r="AE67" t="inlineStr"/>
+      <c r="AE67" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF67" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -10606,42 +10686,48 @@
         </is>
       </c>
       <c r="AI67" t="n">
-        <v>18889</v>
+        <v>18526</v>
       </c>
       <c r="AJ67" t="inlineStr">
         <is>
-          <t>262808,264311</t>
+          <t>262171,263959</t>
         </is>
       </c>
       <c r="AK67" t="inlineStr">
         <is>
-          <t>2037,2042</t>
+          <t>2037,2041</t>
         </is>
       </c>
       <c r="AL67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>15795</v>
+        <v>16580</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YAAKSHITH CHETTI</t>
+          <t>CHANUKYA APPALACHARYULU MUNUBARTHI</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>9160018096</v>
+        <v>9908906244</v>
       </c>
       <c r="D68" t="n">
-        <v>500</v>
-      </c>
-      <c r="E68" t="inlineStr"/>
+        <v>8850</v>
+      </c>
+      <c r="E68" t="n">
+        <v>8850</v>
+      </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>20-Nov-2025 20:01:56</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr"/>
+          <t>20-Nov-2025 17:12:41</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H68" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -10659,7 +10745,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>five hundred</t>
+          <t>eight thousand eight hundred fifty</t>
         </is>
       </c>
       <c r="L68" t="n">
@@ -10677,13 +10763,13 @@
         <v>1234</v>
       </c>
       <c r="P68" t="n">
-        <v>11000317606868</v>
+        <v>11000317589448</v>
       </c>
       <c r="Q68" t="n">
-        <v>1763649005</v>
+        <v>1763638742</v>
       </c>
       <c r="R68" t="n">
-        <v>185561913245</v>
+        <v>108605556686</v>
       </c>
       <c r="S68" t="inlineStr">
         <is>
@@ -10702,7 +10788,7 @@
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W68" t="inlineStr">
@@ -10725,15 +10811,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA68" t="inlineStr"/>
-      <c r="AB68" t="inlineStr"/>
+      <c r="AA68" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB68" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC68" t="n">
         <v>0</v>
       </c>
       <c r="AD68" t="n">
         <v>0</v>
       </c>
-      <c r="AE68" t="inlineStr"/>
+      <c r="AE68" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF68" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -10746,46 +10838,48 @@
         </is>
       </c>
       <c r="AI68" t="n">
-        <v>19105</v>
+        <v>18889</v>
       </c>
       <c r="AJ68" t="inlineStr">
         <is>
-          <t>262986</t>
+          <t>262808,264311</t>
         </is>
       </c>
       <c r="AK68" t="inlineStr">
         <is>
-          <t>2037</t>
-        </is>
-      </c>
-      <c r="AL68" t="inlineStr">
-        <is>
-          <t>UPI INTENT</t>
-        </is>
-      </c>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="AL68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>16617</v>
+        <v>15795</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>THANU SREE BHOOMIREDDY</t>
+          <t>YAAKSHITH CHETTI</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>9573771080</v>
+        <v>9160018096</v>
       </c>
       <c r="D69" t="n">
-        <v>8050</v>
-      </c>
-      <c r="E69" t="inlineStr"/>
+        <v>500</v>
+      </c>
+      <c r="E69" t="n">
+        <v>500</v>
+      </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>20-Nov-2025 20:59:36</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr"/>
+          <t>20-Nov-2025 20:01:56</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -10803,7 +10897,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>eight thousand fifty</t>
+          <t>five hundred</t>
         </is>
       </c>
       <c r="L69" t="n">
@@ -10821,13 +10915,13 @@
         <v>1234</v>
       </c>
       <c r="P69" t="n">
-        <v>11000317615031</v>
+        <v>11000317606868</v>
       </c>
       <c r="Q69" t="n">
-        <v>1763652458</v>
+        <v>1763649005</v>
       </c>
       <c r="R69" t="n">
-        <v>108606865688</v>
+        <v>185561913245</v>
       </c>
       <c r="S69" t="inlineStr">
         <is>
@@ -10846,7 +10940,7 @@
       </c>
       <c r="V69" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W69" t="inlineStr">
@@ -10869,15 +10963,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA69" t="inlineStr"/>
-      <c r="AB69" t="inlineStr"/>
+      <c r="AA69" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB69" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC69" t="n">
         <v>0</v>
       </c>
       <c r="AD69" t="n">
         <v>0</v>
       </c>
-      <c r="AE69" t="inlineStr"/>
+      <c r="AE69" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF69" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -10890,42 +10990,52 @@
         </is>
       </c>
       <c r="AI69" t="n">
-        <v>18610</v>
+        <v>19105</v>
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>265580</t>
+          <t>262986</t>
         </is>
       </c>
       <c r="AK69" t="inlineStr">
         <is>
-          <t>2049</t>
-        </is>
-      </c>
-      <c r="AL69" t="inlineStr"/>
+          <t>2037</t>
+        </is>
+      </c>
+      <c r="AL69" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>17149</v>
+        <v>16617</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MELINDHA BADE</t>
+          <t>THANU SREE BHOOMIREDDY</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>9989075944</v>
+        <v>9573771080</v>
       </c>
       <c r="D70" t="n">
-        <v>9150</v>
-      </c>
-      <c r="E70" t="inlineStr"/>
+        <v>8050</v>
+      </c>
+      <c r="E70" t="n">
+        <v>8050</v>
+      </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>20-Nov-2025 21:49:09</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr"/>
+          <t>20-Nov-2025 20:59:36</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -10938,12 +11048,12 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Multi</t>
+          <t>lVl</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>nine thousand one hundred fifty</t>
+          <t>eight thousand fifty</t>
         </is>
       </c>
       <c r="L70" t="n">
@@ -10961,13 +11071,13 @@
         <v>1234</v>
       </c>
       <c r="P70" t="n">
-        <v>11000317619325</v>
+        <v>11000317615031</v>
       </c>
       <c r="Q70" t="n">
-        <v>1763655441</v>
+        <v>1763652458</v>
       </c>
       <c r="R70" t="n">
-        <v>108607082636</v>
+        <v>108606865688</v>
       </c>
       <c r="S70" t="inlineStr">
         <is>
@@ -10986,12 +11096,12 @@
       </c>
       <c r="V70" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W70" t="inlineStr">
         <is>
-          <t>IFSC0000000</t>
+          <t>SIBL0000899</t>
         </is>
       </c>
       <c r="X70" t="inlineStr">
@@ -11009,16 +11119,26 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA70" t="inlineStr"/>
-      <c r="AB70" t="inlineStr"/>
+      <c r="AA70" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB70" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC70" t="n">
         <v>0</v>
       </c>
       <c r="AD70" t="n">
         <v>0</v>
       </c>
-      <c r="AE70" t="inlineStr"/>
-      <c r="AF70" t="inlineStr"/>
+      <c r="AE70" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF70" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
       <c r="AG70" t="inlineStr"/>
       <c r="AH70" t="inlineStr">
         <is>
@@ -11026,19 +11146,1015 @@
         </is>
       </c>
       <c r="AI70" t="n">
+        <v>18610</v>
+      </c>
+      <c r="AJ70" t="inlineStr">
+        <is>
+          <t>265580</t>
+        </is>
+      </c>
+      <c r="AK70" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>17149</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>MELINDHA BADE</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>9989075944</v>
+      </c>
+      <c r="D71" t="n">
+        <v>9150</v>
+      </c>
+      <c r="E71" t="n">
+        <v>9150</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>20-Nov-2025 21:49:09</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>nine thousand one hundred fifty</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O71" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P71" t="n">
+        <v>11000317619325</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>1763655441</v>
+      </c>
+      <c r="R71" t="n">
+        <v>108607082636</v>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>IFSC0000000</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA71" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB71" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE71" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF71" t="inlineStr"/>
+      <c r="AG71" t="inlineStr"/>
+      <c r="AH71" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI71" t="n">
         <v>19852</v>
       </c>
-      <c r="AJ70" t="inlineStr">
+      <c r="AJ71" t="inlineStr">
         <is>
           <t>262887,264390</t>
         </is>
       </c>
-      <c r="AK70" t="inlineStr">
+      <c r="AK71" t="inlineStr">
         <is>
           <t>2037,2043</t>
         </is>
       </c>
-      <c r="AL70" t="inlineStr"/>
+      <c r="AL71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>16492</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ASHWATH ADITHYA MUNUBARTHI</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>9908906244</v>
+      </c>
+      <c r="D72" t="n">
+        <v>8550</v>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 07:11:30</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>eight thousand five hundred fifty</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O72" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P72" t="n">
+        <v>11000317632962</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>1763689095</v>
+      </c>
+      <c r="R72" t="n">
+        <v>108608167999</v>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr"/>
+      <c r="AB72" t="inlineStr"/>
+      <c r="AC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE72" t="inlineStr"/>
+      <c r="AF72" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG72" t="inlineStr"/>
+      <c r="AH72" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI72" t="n">
+        <v>18659</v>
+      </c>
+      <c r="AJ72" t="inlineStr">
+        <is>
+          <t>262404,264014</t>
+        </is>
+      </c>
+      <c r="AK72" t="inlineStr">
+        <is>
+          <t>2037,2041</t>
+        </is>
+      </c>
+      <c r="AL72" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>15898</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>MAHENDRA NAIDU VANJARI</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>9440280157</v>
+      </c>
+      <c r="D73" t="n">
+        <v>17800</v>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 09:13:00</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>seventeen thousand eight hundred</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O73" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P73" t="n">
+        <v>11000317644277</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>1763696190</v>
+      </c>
+      <c r="R73" t="n">
+        <v>122941457741</v>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>IFSC0000000</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA73" t="inlineStr"/>
+      <c r="AB73" t="inlineStr"/>
+      <c r="AC73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE73" t="inlineStr"/>
+      <c r="AF73" t="inlineStr"/>
+      <c r="AG73" t="inlineStr"/>
+      <c r="AH73" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI73" t="n">
+        <v>19009</v>
+      </c>
+      <c r="AJ73" t="inlineStr">
+        <is>
+          <t>262983,264486,266136</t>
+        </is>
+      </c>
+      <c r="AK73" t="inlineStr">
+        <is>
+          <t>2037,2043,2051</t>
+        </is>
+      </c>
+      <c r="AL73" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>15538</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>VENKATA VIGNESWARI SAI VINYA BOTTA</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>6303433178</v>
+      </c>
+      <c r="D74" t="n">
+        <v>8850</v>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 10:45:33</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>eight thousand eight hundred fifty</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N74" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O74" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P74" t="n">
+        <v>11000317657466</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>1763702116</v>
+      </c>
+      <c r="R74" t="n">
+        <v>404578383859</v>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA74" t="inlineStr"/>
+      <c r="AB74" t="inlineStr"/>
+      <c r="AC74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE74" t="inlineStr"/>
+      <c r="AF74" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG74" t="inlineStr"/>
+      <c r="AH74" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI74" t="n">
+        <v>18918</v>
+      </c>
+      <c r="AJ74" t="inlineStr">
+        <is>
+          <t>262741,264244</t>
+        </is>
+      </c>
+      <c r="AK74" t="inlineStr">
+        <is>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="AL74" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>14873</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>GNANA VIGNESWARI SAI CHANDRIKA BOTTA</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>6303433178</v>
+      </c>
+      <c r="D75" t="n">
+        <v>11250</v>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 10:46:49</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>eleven thousand two hundred fifty</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N75" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O75" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P75" t="n">
+        <v>11000317657543</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>1763702195</v>
+      </c>
+      <c r="R75" t="n">
+        <v>79146114128</v>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>IFSC0000000</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr"/>
+      <c r="AB75" t="inlineStr"/>
+      <c r="AC75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE75" t="inlineStr"/>
+      <c r="AF75" t="inlineStr"/>
+      <c r="AG75" t="inlineStr"/>
+      <c r="AH75" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI75" t="n">
+        <v>19244</v>
+      </c>
+      <c r="AJ75" t="inlineStr">
+        <is>
+          <t>263048,264551</t>
+        </is>
+      </c>
+      <c r="AK75" t="inlineStr">
+        <is>
+          <t>2037,2044</t>
+        </is>
+      </c>
+      <c r="AL75" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>15096</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>RAYASAM SRI VARNIKA</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>7382913422</v>
+      </c>
+      <c r="D76" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 14:41:57</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O76" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P76" t="n">
+        <v>11000317695213</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>1763715904</v>
+      </c>
+      <c r="R76" t="n">
+        <v>1.012025325918391e+17</v>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>BANK OF BARODA FSS</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr"/>
+      <c r="AB76" t="inlineStr"/>
+      <c r="AC76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE76" t="inlineStr"/>
+      <c r="AF76" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG76" t="inlineStr"/>
+      <c r="AH76" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI76" t="n">
+        <v>19483</v>
+      </c>
+      <c r="AJ76" t="inlineStr">
+        <is>
+          <t>264879</t>
+        </is>
+      </c>
+      <c r="AK76" t="inlineStr">
+        <is>
+          <t>2045</t>
+        </is>
+      </c>
+      <c r="AL76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>16992</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>GAUTAM MOOGI</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>7207505036</v>
+      </c>
+      <c r="D77" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>21-Nov-2025 17:59:17</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N77" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O77" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P77" t="n">
+        <v>11000317719673</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>1763728005</v>
+      </c>
+      <c r="R77" t="n">
+        <v>108611639217</v>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr"/>
+      <c r="AB77" t="inlineStr"/>
+      <c r="AC77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE77" t="inlineStr"/>
+      <c r="AF77" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG77" t="inlineStr"/>
+      <c r="AH77" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI77" t="n">
+        <v>18360</v>
+      </c>
+      <c r="AJ77" t="inlineStr">
+        <is>
+          <t>265368</t>
+        </is>
+      </c>
+      <c r="AK77" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="AL77" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update fee collection and reports with latest payments
Added new fee payment records for 2025-11-22 across multiple CSVs, updated student payment statuses and dues in fees_collection.csv and fees_report.csv, and appended new transactions in fee_transcation_atom_report.csv. Also updated Power BI dashboards and Excel reports to reflect the latest data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL77"/>
+  <dimension ref="A1:AL86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12156,6 +12156,1278 @@
       </c>
       <c r="AL77" t="inlineStr"/>
     </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>16353</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>HRIDAYANSH VICTOR RETOJI</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>9395553084</v>
+      </c>
+      <c r="D78" t="n">
+        <v>8550</v>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 07:12:07</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>eight thousand five hundred fifty</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N78" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O78" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P78" t="n">
+        <v>11000317752087</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>1763775572</v>
+      </c>
+      <c r="R78" t="n">
+        <v>108613908890</v>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr"/>
+      <c r="AB78" t="inlineStr"/>
+      <c r="AC78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE78" t="inlineStr"/>
+      <c r="AF78" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG78" t="inlineStr"/>
+      <c r="AH78" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI78" t="n">
+        <v>18469</v>
+      </c>
+      <c r="AJ78" t="inlineStr">
+        <is>
+          <t>262466,263884</t>
+        </is>
+      </c>
+      <c r="AK78" t="inlineStr">
+        <is>
+          <t>2037,2041</t>
+        </is>
+      </c>
+      <c r="AL78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>15824</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>GOLAGANI RITHIK NANDHAN</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>9393123464</v>
+      </c>
+      <c r="D79" t="n">
+        <v>8550</v>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 08:41:05</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>eight thousand five hundred fifty</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N79" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O79" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P79" t="n">
+        <v>11000317755959</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>1763781049</v>
+      </c>
+      <c r="R79" t="n">
+        <v>722776047390</v>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr"/>
+      <c r="AB79" t="inlineStr"/>
+      <c r="AC79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE79" t="inlineStr"/>
+      <c r="AF79" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG79" t="inlineStr"/>
+      <c r="AH79" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI79" t="n">
+        <v>18667</v>
+      </c>
+      <c r="AJ79" t="inlineStr">
+        <is>
+          <t>262441,264022</t>
+        </is>
+      </c>
+      <c r="AK79" t="inlineStr">
+        <is>
+          <t>2037,2041</t>
+        </is>
+      </c>
+      <c r="AL79" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>15009</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>GOLAGANI GEETHANJALI</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>9393123464</v>
+      </c>
+      <c r="D80" t="n">
+        <v>9150</v>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 08:44:37</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>nine thousand one hundred fifty</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O80" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P80" t="n">
+        <v>11000317756764</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>1763781250</v>
+      </c>
+      <c r="R80" t="n">
+        <v>387942566112</v>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>IFSC0000000</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr"/>
+      <c r="AB80" t="inlineStr"/>
+      <c r="AC80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE80" t="inlineStr"/>
+      <c r="AF80" t="inlineStr"/>
+      <c r="AG80" t="inlineStr"/>
+      <c r="AH80" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI80" t="n">
+        <v>19026</v>
+      </c>
+      <c r="AJ80" t="inlineStr">
+        <is>
+          <t>262897,264400</t>
+        </is>
+      </c>
+      <c r="AK80" t="inlineStr">
+        <is>
+          <t>2037,2043</t>
+        </is>
+      </c>
+      <c r="AL80" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>17316</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SUVVARI JAIDEEP</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>7386363690</v>
+      </c>
+      <c r="D81" t="n">
+        <v>8250</v>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 09:33:58</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>eight thousand two hundred fifty</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N81" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O81" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P81" t="n">
+        <v>11000317759875</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>1763783349</v>
+      </c>
+      <c r="R81" t="n">
+        <v>929606991918</v>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA81" t="inlineStr"/>
+      <c r="AB81" t="inlineStr"/>
+      <c r="AC81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE81" t="inlineStr"/>
+      <c r="AF81" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG81" t="inlineStr"/>
+      <c r="AH81" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI81" t="n">
+        <v>20024</v>
+      </c>
+      <c r="AJ81" t="inlineStr">
+        <is>
+          <t>262633,263603</t>
+        </is>
+      </c>
+      <c r="AK81" t="inlineStr">
+        <is>
+          <t>2037,2040</t>
+        </is>
+      </c>
+      <c r="AL81" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>16598</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>MANASHVI AKKIREDDY</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>8184888497</v>
+      </c>
+      <c r="D82" t="n">
+        <v>8250</v>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 09:56:00</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>eight thousand two hundred fifty</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O82" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P82" t="n">
+        <v>11000317762419</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>1763785456</v>
+      </c>
+      <c r="R82" t="n">
+        <v>108614534365</v>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr"/>
+      <c r="AB82" t="inlineStr"/>
+      <c r="AC82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE82" t="inlineStr"/>
+      <c r="AF82" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG82" t="inlineStr"/>
+      <c r="AH82" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI82" t="n">
+        <v>18346</v>
+      </c>
+      <c r="AJ82" t="inlineStr">
+        <is>
+          <t>262200,263672</t>
+        </is>
+      </c>
+      <c r="AK82" t="inlineStr">
+        <is>
+          <t>2037,2040</t>
+        </is>
+      </c>
+      <c r="AL82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>14944</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SRAVAN BHARGAV KADIRI</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>9701983320</v>
+      </c>
+      <c r="D83" t="n">
+        <v>11250</v>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 10:53:07</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>eleven thousand two hundred fifty</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O83" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P83" t="n">
+        <v>11000317774408</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>1763788955</v>
+      </c>
+      <c r="R83" t="n">
+        <v>108614807525</v>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>IFSC0000000</t>
+        </is>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr"/>
+      <c r="AB83" t="inlineStr"/>
+      <c r="AC83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE83" t="inlineStr"/>
+      <c r="AF83" t="inlineStr"/>
+      <c r="AG83" t="inlineStr"/>
+      <c r="AH83" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI83" t="n">
+        <v>19236</v>
+      </c>
+      <c r="AJ83" t="inlineStr">
+        <is>
+          <t>263139,264642</t>
+        </is>
+      </c>
+      <c r="AK83" t="inlineStr">
+        <is>
+          <t>2037,2044</t>
+        </is>
+      </c>
+      <c r="AL83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>17099</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>VINDYA SOWDALA</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>7075489300</v>
+      </c>
+      <c r="D84" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 12:23:46</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N84" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O84" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P84" t="n">
+        <v>11000317789451</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>1763794365</v>
+      </c>
+      <c r="R84" t="n">
+        <v>84407133536</v>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr"/>
+      <c r="AB84" t="inlineStr"/>
+      <c r="AC84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE84" t="inlineStr"/>
+      <c r="AF84" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG84" t="inlineStr"/>
+      <c r="AH84" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI84" t="n">
+        <v>18095</v>
+      </c>
+      <c r="AJ84" t="inlineStr">
+        <is>
+          <t>265111</t>
+        </is>
+      </c>
+      <c r="AK84" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL84" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>17100</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>BHAVIYSA SOWDALA</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>7075489300</v>
+      </c>
+      <c r="D85" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 12:26:26</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N85" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O85" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P85" t="n">
+        <v>11000317789617</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>1763794575</v>
+      </c>
+      <c r="R85" t="n">
+        <v>892395505599</v>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA85" t="inlineStr"/>
+      <c r="AB85" t="inlineStr"/>
+      <c r="AC85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE85" t="inlineStr"/>
+      <c r="AF85" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG85" t="inlineStr"/>
+      <c r="AH85" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI85" t="n">
+        <v>18638</v>
+      </c>
+      <c r="AJ85" t="inlineStr">
+        <is>
+          <t>265647</t>
+        </is>
+      </c>
+      <c r="AK85" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL85" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>16721</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>KURMAPU GAGANASHREE</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>9908361635</v>
+      </c>
+      <c r="D86" t="n">
+        <v>8250</v>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>22-Nov-2025 12:59:10</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>eight thousand two hundred fifty</t>
+        </is>
+      </c>
+      <c r="L86" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N86" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O86" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P86" t="n">
+        <v>11000317794411</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>1763796507</v>
+      </c>
+      <c r="R86" t="n">
+        <v>108615558861</v>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA86" t="inlineStr"/>
+      <c r="AB86" t="inlineStr"/>
+      <c r="AC86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE86" t="inlineStr"/>
+      <c r="AF86" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG86" t="inlineStr"/>
+      <c r="AH86" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI86" t="n">
+        <v>18114</v>
+      </c>
+      <c r="AJ86" t="inlineStr">
+        <is>
+          <t>262147,263524</t>
+        </is>
+      </c>
+      <c r="AK86" t="inlineStr">
+        <is>
+          <t>2037,2040</t>
+        </is>
+      </c>
+      <c r="AL86" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update fee collection and student data for Nov 2025
Added new fee collection records and updated student payment data for November 2025 across multiple CSV files. Also included new backup and updated Power BI dashboard and Excel reports. Removed obsolete atom_report.csv from source_data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL90"/>
+  <dimension ref="A1:AL96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12994,25 +12994,25 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>14944</v>
+        <v>17219</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SRAVAN BHARGAV KADIRI</t>
+          <t>VARTIKA KUMARI</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>9701983320</v>
+        <v>8369239788</v>
       </c>
       <c r="D83" t="n">
-        <v>11250</v>
+        <v>8250</v>
       </c>
       <c r="E83" t="n">
-        <v>11250</v>
+        <v>8250</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>22-Nov-2025 10:53:07</t>
+          <t>22-Nov-2025 10:44:52</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -13022,7 +13022,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>TRANSACTION IS SUCCESSFUL</t>
+          <t>TRANSACTION IS SUCCESS</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -13032,12 +13032,12 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Multi</t>
+          <t>lVl</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>eleven thousand two hundred fifty</t>
+          <t>eight thousand two hundred fifty</t>
         </is>
       </c>
       <c r="L83" t="n">
@@ -13055,13 +13055,13 @@
         <v>1234</v>
       </c>
       <c r="P83" t="n">
-        <v>11000317774408</v>
+        <v>11000317773361</v>
       </c>
       <c r="Q83" t="n">
-        <v>1763788955</v>
+        <v>1763788142</v>
       </c>
       <c r="R83" t="n">
-        <v>108614807525</v>
+        <v>104508217364</v>
       </c>
       <c r="S83" t="inlineStr">
         <is>
@@ -13080,12 +13080,12 @@
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W83" t="inlineStr">
         <is>
-          <t>IFSC0000000</t>
+          <t>SIBL0000899</t>
         </is>
       </c>
       <c r="X83" t="inlineStr">
@@ -13095,7 +13095,7 @@
       </c>
       <c r="Y83" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>QR_UPI</t>
         </is>
       </c>
       <c r="Z83" t="inlineStr">
@@ -13118,7 +13118,11 @@
       <c r="AE83" t="n">
         <v>5.9</v>
       </c>
-      <c r="AF83" t="inlineStr"/>
+      <c r="AF83" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
       <c r="AG83" t="inlineStr"/>
       <c r="AH83" t="inlineStr">
         <is>
@@ -13126,41 +13130,45 @@
         </is>
       </c>
       <c r="AI83" t="n">
-        <v>19236</v>
+        <v>19931</v>
       </c>
       <c r="AJ83" t="inlineStr">
         <is>
-          <t>263139,264642</t>
+          <t>262332,263555</t>
         </is>
       </c>
       <c r="AK83" t="inlineStr">
         <is>
-          <t>2037,2044</t>
-        </is>
-      </c>
-      <c r="AL83" t="inlineStr"/>
+          <t>2037,2040</t>
+        </is>
+      </c>
+      <c r="AL83" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>17099</v>
+        <v>14944</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>VINDYA SOWDALA</t>
+          <t>SRAVAN BHARGAV KADIRI</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>7075489300</v>
+        <v>9701983320</v>
       </c>
       <c r="D84" t="n">
-        <v>6750</v>
+        <v>11250</v>
       </c>
       <c r="E84" t="n">
-        <v>6750</v>
+        <v>11250</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>22-Nov-2025 12:23:46</t>
+          <t>22-Nov-2025 10:53:07</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -13180,12 +13188,12 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>PREKGUKG</t>
+          <t>Multi</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>six thousand seven hundred fifty</t>
+          <t>eleven thousand two hundred fifty</t>
         </is>
       </c>
       <c r="L84" t="n">
@@ -13203,13 +13211,13 @@
         <v>1234</v>
       </c>
       <c r="P84" t="n">
-        <v>11000317789451</v>
+        <v>11000317774408</v>
       </c>
       <c r="Q84" t="n">
-        <v>1763794365</v>
+        <v>1763788955</v>
       </c>
       <c r="R84" t="n">
-        <v>84407133536</v>
+        <v>108614807525</v>
       </c>
       <c r="S84" t="inlineStr">
         <is>
@@ -13228,12 +13236,12 @@
       </c>
       <c r="V84" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>SIBL0000899</t>
+          <t>IFSC0000000</t>
         </is>
       </c>
       <c r="X84" t="inlineStr">
@@ -13266,11 +13274,7 @@
       <c r="AE84" t="n">
         <v>5.9</v>
       </c>
-      <c r="AF84" t="inlineStr">
-        <is>
-          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
-        </is>
-      </c>
+      <c r="AF84" t="inlineStr"/>
       <c r="AG84" t="inlineStr"/>
       <c r="AH84" t="inlineStr">
         <is>
@@ -13278,45 +13282,41 @@
         </is>
       </c>
       <c r="AI84" t="n">
-        <v>18095</v>
+        <v>19236</v>
       </c>
       <c r="AJ84" t="inlineStr">
         <is>
-          <t>265111</t>
+          <t>263139,264642</t>
         </is>
       </c>
       <c r="AK84" t="inlineStr">
         <is>
-          <t>2047</t>
-        </is>
-      </c>
-      <c r="AL84" t="inlineStr">
-        <is>
-          <t>UPI INTENT</t>
-        </is>
-      </c>
+          <t>2037,2044</t>
+        </is>
+      </c>
+      <c r="AL84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>17100</v>
+        <v>17099</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>BHAVIYSA SOWDALA</t>
+          <t>VINDYA SOWDALA</t>
         </is>
       </c>
       <c r="C85" t="n">
         <v>7075489300</v>
       </c>
       <c r="D85" t="n">
-        <v>8050</v>
+        <v>6750</v>
       </c>
       <c r="E85" t="n">
-        <v>8050</v>
+        <v>6750</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>22-Nov-2025 12:26:26</t>
+          <t>22-Nov-2025 12:23:46</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -13336,12 +13336,12 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>lVl</t>
+          <t>PREKGUKG</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>eight thousand fifty</t>
+          <t>six thousand seven hundred fifty</t>
         </is>
       </c>
       <c r="L85" t="n">
@@ -13359,13 +13359,13 @@
         <v>1234</v>
       </c>
       <c r="P85" t="n">
-        <v>11000317789617</v>
+        <v>11000317789451</v>
       </c>
       <c r="Q85" t="n">
-        <v>1763794575</v>
+        <v>1763794365</v>
       </c>
       <c r="R85" t="n">
-        <v>892395505599</v>
+        <v>84407133536</v>
       </c>
       <c r="S85" t="inlineStr">
         <is>
@@ -13424,7 +13424,7 @@
       </c>
       <c r="AF85" t="inlineStr">
         <is>
-          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
         </is>
       </c>
       <c r="AG85" t="inlineStr"/>
@@ -13434,16 +13434,16 @@
         </is>
       </c>
       <c r="AI85" t="n">
-        <v>18638</v>
+        <v>18095</v>
       </c>
       <c r="AJ85" t="inlineStr">
         <is>
-          <t>265647</t>
+          <t>265111</t>
         </is>
       </c>
       <c r="AK85" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>2047</t>
         </is>
       </c>
       <c r="AL85" t="inlineStr">
@@ -13454,25 +13454,25 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>16721</v>
+        <v>17100</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>KURMAPU GAGANASHREE</t>
+          <t>BHAVIYSA SOWDALA</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>9908361635</v>
+        <v>7075489300</v>
       </c>
       <c r="D86" t="n">
-        <v>8250</v>
+        <v>8050</v>
       </c>
       <c r="E86" t="n">
-        <v>8250</v>
+        <v>8050</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>22-Nov-2025 12:59:10</t>
+          <t>22-Nov-2025 12:26:26</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -13497,7 +13497,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>eight thousand two hundred fifty</t>
+          <t>eight thousand fifty</t>
         </is>
       </c>
       <c r="L86" t="n">
@@ -13515,13 +13515,13 @@
         <v>1234</v>
       </c>
       <c r="P86" t="n">
-        <v>11000317794411</v>
+        <v>11000317789617</v>
       </c>
       <c r="Q86" t="n">
-        <v>1763796507</v>
+        <v>1763794575</v>
       </c>
       <c r="R86" t="n">
-        <v>108615558861</v>
+        <v>892395505599</v>
       </c>
       <c r="S86" t="inlineStr">
         <is>
@@ -13590,42 +13590,52 @@
         </is>
       </c>
       <c r="AI86" t="n">
-        <v>18114</v>
+        <v>18638</v>
       </c>
       <c r="AJ86" t="inlineStr">
         <is>
-          <t>262147,263524</t>
+          <t>265647</t>
         </is>
       </c>
       <c r="AK86" t="inlineStr">
         <is>
-          <t>2037,2040</t>
-        </is>
-      </c>
-      <c r="AL86" t="inlineStr"/>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL86" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>14160</v>
+        <v>16721</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>DHARMAVARAPU CHANDANA RAMYA</t>
+          <t>KURMAPU GAGANASHREE</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>8374970989</v>
+        <v>9908361635</v>
       </c>
       <c r="D87" t="n">
-        <v>11350</v>
-      </c>
-      <c r="E87" t="inlineStr"/>
+        <v>8250</v>
+      </c>
+      <c r="E87" t="n">
+        <v>8250</v>
+      </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>24-Nov-2025 08:01:40</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr"/>
+          <t>22-Nov-2025 12:59:10</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>24-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -13638,12 +13648,12 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>VlllX</t>
+          <t>lVl</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>eleven thousand three hundred fifty</t>
+          <t>eight thousand two hundred fifty</t>
         </is>
       </c>
       <c r="L87" t="n">
@@ -13661,13 +13671,13 @@
         <v>1234</v>
       </c>
       <c r="P87" t="n">
-        <v>11000317917995</v>
+        <v>11000317794411</v>
       </c>
       <c r="Q87" t="n">
-        <v>1763951385</v>
+        <v>1763796507</v>
       </c>
       <c r="R87" t="n">
-        <v>108625745822</v>
+        <v>108615558861</v>
       </c>
       <c r="S87" t="inlineStr">
         <is>
@@ -13686,7 +13696,7 @@
       </c>
       <c r="V87" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W87" t="inlineStr">
@@ -13709,18 +13719,24 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA87" t="inlineStr"/>
-      <c r="AB87" t="inlineStr"/>
+      <c r="AA87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB87" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC87" t="n">
         <v>0</v>
       </c>
       <c r="AD87" t="n">
         <v>0</v>
       </c>
-      <c r="AE87" t="inlineStr"/>
+      <c r="AE87" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF87" t="inlineStr">
         <is>
-          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
         </is>
       </c>
       <c r="AG87" t="inlineStr"/>
@@ -13730,39 +13746,41 @@
         </is>
       </c>
       <c r="AI87" t="n">
-        <v>19571</v>
+        <v>18114</v>
       </c>
       <c r="AJ87" t="inlineStr">
         <is>
-          <t>264841</t>
+          <t>262147,263524</t>
         </is>
       </c>
       <c r="AK87" t="inlineStr">
         <is>
-          <t>2045</t>
+          <t>2037,2040</t>
         </is>
       </c>
       <c r="AL87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>14511</v>
+        <v>14160</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>DHARMAVARAPU MADHULICA SRI</t>
+          <t>DHARMAVARAPU CHANDANA RAMYA</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>8374970989</v>
       </c>
       <c r="D88" t="n">
-        <v>11850</v>
-      </c>
-      <c r="E88" t="inlineStr"/>
+        <v>11350</v>
+      </c>
+      <c r="E88" t="n">
+        <v>11350</v>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>24-Nov-2025 08:07:11</t>
+          <t>24-Nov-2025 08:01:40</t>
         </is>
       </c>
       <c r="G88" t="inlineStr"/>
@@ -13778,12 +13796,12 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Multi</t>
+          <t>VlllX</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>eleven thousand eight hundred fifty</t>
+          <t>eleven thousand three hundred fifty</t>
         </is>
       </c>
       <c r="L88" t="n">
@@ -13801,13 +13819,13 @@
         <v>1234</v>
       </c>
       <c r="P88" t="n">
-        <v>11000317919152</v>
+        <v>11000317917995</v>
       </c>
       <c r="Q88" t="n">
-        <v>1763951723</v>
+        <v>1763951385</v>
       </c>
       <c r="R88" t="n">
-        <v>108625767984</v>
+        <v>108625745822</v>
       </c>
       <c r="S88" t="inlineStr">
         <is>
@@ -13826,12 +13844,12 @@
       </c>
       <c r="V88" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W88" t="inlineStr">
         <is>
-          <t>IFSC0000000</t>
+          <t>SIBL0000899</t>
         </is>
       </c>
       <c r="X88" t="inlineStr">
@@ -13849,16 +13867,26 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA88" t="inlineStr"/>
-      <c r="AB88" t="inlineStr"/>
+      <c r="AA88" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB88" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC88" t="n">
         <v>0</v>
       </c>
       <c r="AD88" t="n">
         <v>0</v>
       </c>
-      <c r="AE88" t="inlineStr"/>
-      <c r="AF88" t="inlineStr"/>
+      <c r="AE88" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF88" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
       <c r="AG88" t="inlineStr"/>
       <c r="AH88" t="inlineStr">
         <is>
@@ -13866,42 +13894,48 @@
         </is>
       </c>
       <c r="AI88" t="n">
-        <v>19336</v>
+        <v>19571</v>
       </c>
       <c r="AJ88" t="inlineStr">
         <is>
-          <t>263218,264721</t>
+          <t>264841</t>
         </is>
       </c>
       <c r="AK88" t="inlineStr">
         <is>
-          <t>2037,2045</t>
+          <t>2045</t>
         </is>
       </c>
       <c r="AL88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>17103</v>
+        <v>14511</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PANDRANKI BHAVITHA SRI</t>
+          <t>DHARMAVARAPU MADHULICA SRI</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>6301729629</v>
+        <v>8374970989</v>
       </c>
       <c r="D89" t="n">
-        <v>6750</v>
-      </c>
-      <c r="E89" t="inlineStr"/>
+        <v>11850</v>
+      </c>
+      <c r="E89" t="n">
+        <v>11850</v>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>24-Nov-2025 08:19:39</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr"/>
+          <t>24-Nov-2025 08:07:11</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>25-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -13914,12 +13948,12 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>PREKGUKG</t>
+          <t>Multi</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>six thousand seven hundred fifty</t>
+          <t>eleven thousand eight hundred fifty</t>
         </is>
       </c>
       <c r="L89" t="n">
@@ -13937,13 +13971,13 @@
         <v>1234</v>
       </c>
       <c r="P89" t="n">
-        <v>11000317919499</v>
+        <v>11000317919152</v>
       </c>
       <c r="Q89" t="n">
-        <v>1763952416</v>
+        <v>1763951723</v>
       </c>
       <c r="R89" t="n">
-        <v>108625814663</v>
+        <v>108625767984</v>
       </c>
       <c r="S89" t="inlineStr">
         <is>
@@ -13962,12 +13996,12 @@
       </c>
       <c r="V89" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W89" t="inlineStr">
         <is>
-          <t>SIBL0000899</t>
+          <t>IFSC0000000</t>
         </is>
       </c>
       <c r="X89" t="inlineStr">
@@ -13985,20 +14019,22 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA89" t="inlineStr"/>
-      <c r="AB89" t="inlineStr"/>
+      <c r="AA89" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB89" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC89" t="n">
         <v>0</v>
       </c>
       <c r="AD89" t="n">
         <v>0</v>
       </c>
-      <c r="AE89" t="inlineStr"/>
-      <c r="AF89" t="inlineStr">
-        <is>
-          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
-        </is>
-      </c>
+      <c r="AE89" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF89" t="inlineStr"/>
       <c r="AG89" t="inlineStr"/>
       <c r="AH89" t="inlineStr">
         <is>
@@ -14006,42 +14042,48 @@
         </is>
       </c>
       <c r="AI89" t="n">
-        <v>18038</v>
+        <v>19336</v>
       </c>
       <c r="AJ89" t="inlineStr">
         <is>
-          <t>263436</t>
+          <t>263218,264721</t>
         </is>
       </c>
       <c r="AK89" t="inlineStr">
         <is>
-          <t>2039</t>
+          <t>2037,2045</t>
         </is>
       </c>
       <c r="AL89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>16067</v>
+        <v>17103</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MOHAMMAD AFZAL</t>
+          <t>PANDRANKI BHAVITHA SRI</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>9885519010</v>
+        <v>6301729629</v>
       </c>
       <c r="D90" t="n">
-        <v>22000</v>
-      </c>
-      <c r="E90" t="inlineStr"/>
+        <v>6750</v>
+      </c>
+      <c r="E90" t="n">
+        <v>6750</v>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>24-Nov-2025 10:20:54</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr"/>
+          <t>24-Nov-2025 08:19:39</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>25-Nov-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H90" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -14054,12 +14096,12 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Multi</t>
+          <t>PREKGUKG</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t xml:space="preserve">twenty two thousand </t>
+          <t>six thousand seven hundred fifty</t>
         </is>
       </c>
       <c r="L90" t="n">
@@ -14077,13 +14119,13 @@
         <v>1234</v>
       </c>
       <c r="P90" t="n">
-        <v>11000317934837</v>
+        <v>11000317919499</v>
       </c>
       <c r="Q90" t="n">
-        <v>1763959817</v>
+        <v>1763952416</v>
       </c>
       <c r="R90" t="n">
-        <v>694416410395</v>
+        <v>108625814663</v>
       </c>
       <c r="S90" t="inlineStr">
         <is>
@@ -14102,12 +14144,12 @@
       </c>
       <c r="V90" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W90" t="inlineStr">
         <is>
-          <t>IFSC0000000</t>
+          <t>SIBL0000899</t>
         </is>
       </c>
       <c r="X90" t="inlineStr">
@@ -14125,16 +14167,26 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA90" t="inlineStr"/>
-      <c r="AB90" t="inlineStr"/>
+      <c r="AA90" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB90" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC90" t="n">
         <v>0</v>
       </c>
       <c r="AD90" t="n">
         <v>0</v>
       </c>
-      <c r="AE90" t="inlineStr"/>
-      <c r="AF90" t="inlineStr"/>
+      <c r="AE90" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF90" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
       <c r="AG90" t="inlineStr"/>
       <c r="AH90" t="inlineStr">
         <is>
@@ -14142,19 +14194,923 @@
         </is>
       </c>
       <c r="AI90" t="n">
+        <v>18038</v>
+      </c>
+      <c r="AJ90" t="inlineStr">
+        <is>
+          <t>263436</t>
+        </is>
+      </c>
+      <c r="AK90" t="inlineStr">
+        <is>
+          <t>2039</t>
+        </is>
+      </c>
+      <c r="AL90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>16067</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>MOHAMMAD AFZAL</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>9885519010</v>
+      </c>
+      <c r="D91" t="n">
+        <v>22000</v>
+      </c>
+      <c r="E91" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>24-Nov-2025 10:20:54</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>25-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">twenty two thousand </t>
+        </is>
+      </c>
+      <c r="L91" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N91" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O91" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P91" t="n">
+        <v>11000317934837</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>1763959817</v>
+      </c>
+      <c r="R91" t="n">
+        <v>694416410395</v>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>IFSC0000000</t>
+        </is>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA91" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB91" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF91" t="inlineStr"/>
+      <c r="AG91" t="inlineStr"/>
+      <c r="AH91" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI91" t="n">
         <v>19319</v>
       </c>
-      <c r="AJ90" t="inlineStr">
+      <c r="AJ91" t="inlineStr">
         <is>
           <t>263145,264648,266298</t>
         </is>
       </c>
-      <c r="AK90" t="inlineStr">
+      <c r="AK91" t="inlineStr">
         <is>
           <t>2037,2044,2052</t>
         </is>
       </c>
-      <c r="AL90" t="inlineStr">
+      <c r="AL91" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>16555</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>GANTEDA CHERISHMA</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>9676361548</v>
+      </c>
+      <c r="D92" t="n">
+        <v>8850</v>
+      </c>
+      <c r="E92" t="n">
+        <v>8850</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>25-Nov-2025 09:02:25</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>26-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>eight thousand eight hundred fifty</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O92" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P92" t="n">
+        <v>11000318061560</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>1764041529</v>
+      </c>
+      <c r="R92" t="n">
+        <v>285283553470</v>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z92" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA92" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB92" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE92" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF92" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG92" t="inlineStr"/>
+      <c r="AH92" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI92" t="n">
+        <v>18789</v>
+      </c>
+      <c r="AJ92" t="inlineStr">
+        <is>
+          <t>262103,264102</t>
+        </is>
+      </c>
+      <c r="AK92" t="inlineStr">
+        <is>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="AL92" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>15863</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>BOMMIDI BALA SURYA BHUVAN</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>6300875193</v>
+      </c>
+      <c r="D93" t="n">
+        <v>8550</v>
+      </c>
+      <c r="E93" t="n">
+        <v>8550</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>25-Nov-2025 12:04:15</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>26-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>eight thousand five hundred fifty</t>
+        </is>
+      </c>
+      <c r="L93" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N93" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O93" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P93" t="n">
+        <v>11000318091639</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>1764052436</v>
+      </c>
+      <c r="R93" t="n">
+        <v>514342923427</v>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA93" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB93" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE93" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF93" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG93" t="inlineStr"/>
+      <c r="AH93" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI93" t="n">
+        <v>18543</v>
+      </c>
+      <c r="AJ93" t="inlineStr">
+        <is>
+          <t>262382,264003</t>
+        </is>
+      </c>
+      <c r="AK93" t="inlineStr">
+        <is>
+          <t>2037,2041</t>
+        </is>
+      </c>
+      <c r="AL93" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>17295</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>PALAKONDA PUDARJUN</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>9493856632</v>
+      </c>
+      <c r="D94" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E94" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>25-Nov-2025 19:32:34</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>26-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L94" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O94" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P94" t="n">
+        <v>11000318159831</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>1764079329</v>
+      </c>
+      <c r="R94" t="n">
+        <v>569509465610</v>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA94" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB94" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE94" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF94" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG94" t="inlineStr"/>
+      <c r="AH94" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI94" t="n">
+        <v>20005</v>
+      </c>
+      <c r="AJ94" t="inlineStr">
+        <is>
+          <t>265045</t>
+        </is>
+      </c>
+      <c r="AK94" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL94" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>16196</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>BOTTA V K SAMTHOSHI VARSHITHA</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>9059927162</v>
+      </c>
+      <c r="D95" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>26-Nov-2025 13:06:35</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L95" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N95" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O95" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P95" t="n">
+        <v>11000318238042</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>1764142579</v>
+      </c>
+      <c r="R95" t="n">
+        <v>779334795869</v>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr"/>
+      <c r="AB95" t="inlineStr"/>
+      <c r="AC95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE95" t="inlineStr"/>
+      <c r="AF95" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG95" t="inlineStr"/>
+      <c r="AH95" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI95" t="n">
+        <v>19597</v>
+      </c>
+      <c r="AJ95" t="inlineStr">
+        <is>
+          <t>261864</t>
+        </is>
+      </c>
+      <c r="AK95" t="inlineStr">
+        <is>
+          <t>2036</t>
+        </is>
+      </c>
+      <c r="AL95" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>14874</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>BOTTA RAM VIGNESH SANTHOSH SAI RISHIK</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>9059927162</v>
+      </c>
+      <c r="D96" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>26-Nov-2025 13:08:30</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N96" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O96" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P96" t="n">
+        <v>11000318238143</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>1764142689</v>
+      </c>
+      <c r="R96" t="n">
+        <v>640249767855</v>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr"/>
+      <c r="AB96" t="inlineStr"/>
+      <c r="AC96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE96" t="inlineStr"/>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr"/>
+      <c r="AH96" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI96" t="n">
+        <v>19186</v>
+      </c>
+      <c r="AJ96" t="inlineStr">
+        <is>
+          <t>261642</t>
+        </is>
+      </c>
+      <c r="AK96" t="inlineStr">
+        <is>
+          <t>2035</t>
+        </is>
+      </c>
+      <c r="AL96" t="inlineStr">
         <is>
           <t>UPI INTENT</t>
         </is>

</xml_diff>

<commit_message>
Remove obsolete data files and update reports
Deleted several outdated source notebooks, workflow files, and merged_fee_collection.csv. Moved and updated fee collection and attendance data files, added new Postgres backup files, and updated various output and report files to reflect the latest data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -14843,7 +14843,9 @@
       <c r="D95" t="n">
         <v>11350</v>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="n">
+        <v>11350</v>
+      </c>
       <c r="F95" t="inlineStr">
         <is>
           <t>26-Nov-2025 13:06:35</t>
@@ -14910,7 +14912,7 @@
       </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W95" t="inlineStr">
@@ -14933,15 +14935,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA95" t="inlineStr"/>
-      <c r="AB95" t="inlineStr"/>
+      <c r="AA95" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB95" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC95" t="n">
         <v>0</v>
       </c>
       <c r="AD95" t="n">
         <v>0</v>
       </c>
-      <c r="AE95" t="inlineStr"/>
+      <c r="AE95" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF95" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -14987,7 +14995,9 @@
       <c r="D96" t="n">
         <v>10750</v>
       </c>
-      <c r="E96" t="inlineStr"/>
+      <c r="E96" t="n">
+        <v>10750</v>
+      </c>
       <c r="F96" t="inlineStr">
         <is>
           <t>26-Nov-2025 13:08:30</t>
@@ -15054,7 +15064,7 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W96" t="inlineStr">
@@ -15077,15 +15087,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA96" t="inlineStr"/>
-      <c r="AB96" t="inlineStr"/>
+      <c r="AA96" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB96" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC96" t="n">
         <v>0</v>
       </c>
       <c r="AD96" t="n">
         <v>0</v>
       </c>
-      <c r="AE96" t="inlineStr"/>
+      <c r="AE96" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF96" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>

</xml_diff>

<commit_message>
Update daywise fees collection data
Corrected and updated entries in output_data/daywise_fees_collection.csv, including changes to receipt numbers, amounts, and student records. This ensures the data reflects the latest and most accurate fee collection information.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL97"/>
+  <dimension ref="A1:AL99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15288,6 +15288,286 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>15962</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>BANALA VAIBHAV</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>9248863180</v>
+      </c>
+      <c r="D98" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>02-Dec-2025 10:00:57</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N98" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O98" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P98" t="n">
+        <v>11000318889672</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>1764649784</v>
+      </c>
+      <c r="R98" t="n">
+        <v>108676570140</v>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr"/>
+      <c r="AB98" t="inlineStr"/>
+      <c r="AC98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE98" t="inlineStr"/>
+      <c r="AF98" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG98" t="inlineStr"/>
+      <c r="AH98" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI98" t="n">
+        <v>19562</v>
+      </c>
+      <c r="AJ98" t="inlineStr">
+        <is>
+          <t>266565</t>
+        </is>
+      </c>
+      <c r="AK98" t="inlineStr">
+        <is>
+          <t>2053</t>
+        </is>
+      </c>
+      <c r="AL98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>17307</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>HEYAN RUUDRA RAPOL</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>9991367333</v>
+      </c>
+      <c r="D99" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>02-Dec-2025 11:23:13</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L99" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N99" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O99" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P99" t="n">
+        <v>11000318907761</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>1764654572</v>
+      </c>
+      <c r="R99" t="n">
+        <v>108677081867</v>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr"/>
+      <c r="AB99" t="inlineStr"/>
+      <c r="AC99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE99" t="inlineStr"/>
+      <c r="AF99" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG99" t="inlineStr"/>
+      <c r="AH99" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI99" t="n">
+        <v>20016</v>
+      </c>
+      <c r="AJ99" t="inlineStr">
+        <is>
+          <t>265830</t>
+        </is>
+      </c>
+      <c r="AK99" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="AL99" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Data Updated Upto 05th December 2025
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -15759,13 +15759,19 @@
       <c r="D101" t="n">
         <v>8350</v>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="n">
+        <v>8350</v>
+      </c>
       <c r="F101" t="inlineStr">
         <is>
           <t>04-Dec-2025 17:57:16</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>05-Dec-2025 00:00:00</t>
+        </is>
+      </c>
       <c r="H101" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -15826,7 +15832,7 @@
       </c>
       <c r="V101" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W101" t="inlineStr">
@@ -15849,15 +15855,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA101" t="inlineStr"/>
-      <c r="AB101" t="inlineStr"/>
+      <c r="AA101" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB101" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC101" t="n">
         <v>0</v>
       </c>
       <c r="AD101" t="n">
         <v>0</v>
       </c>
-      <c r="AE101" t="inlineStr"/>
+      <c r="AE101" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF101" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>

</xml_diff>

<commit_message>
Data Updated Upto 10th Dec 2025
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL101"/>
+  <dimension ref="A1:AL105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15900,6 +15900,618 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>15762</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>PILAKA VINISHA REDDY</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>9505890135</v>
+      </c>
+      <c r="D102" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E102" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>06-Dec-2025 09:17:33</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>08-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L102" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N102" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O102" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P102" t="n">
+        <v>11000319490500</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>1764992795</v>
+      </c>
+      <c r="R102" t="n">
+        <v>108703980088</v>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA102" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB102" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE102" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF102" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG102" t="inlineStr"/>
+      <c r="AH102" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI102" t="n">
+        <v>18805</v>
+      </c>
+      <c r="AJ102" t="inlineStr">
+        <is>
+          <t>265779</t>
+        </is>
+      </c>
+      <c r="AK102" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="AL102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>15868</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>MYLABATHULA MEDHANSH</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>9949134987</v>
+      </c>
+      <c r="D103" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E103" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>07-Dec-2025 21:32:51</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>08-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L103" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N103" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O103" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P103" t="n">
+        <v>11000319686064</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>1765123332</v>
+      </c>
+      <c r="R103" t="n">
+        <v>213323909356</v>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA103" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB103" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE103" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF103" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG103" t="inlineStr"/>
+      <c r="AH103" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI103" t="n">
+        <v>18624</v>
+      </c>
+      <c r="AJ103" t="inlineStr">
+        <is>
+          <t>265707</t>
+        </is>
+      </c>
+      <c r="AK103" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL103" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>15533</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>SHAIK FARHEEN</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>9652279329</v>
+      </c>
+      <c r="D104" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E104" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>08-Dec-2025 15:32:58</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>09-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L104" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N104" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O104" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P104" t="n">
+        <v>11000319809148</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>1765188111</v>
+      </c>
+      <c r="R104" t="n">
+        <v>108719254095</v>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA104" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB104" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE104" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF104" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG104" t="inlineStr"/>
+      <c r="AH104" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI104" t="n">
+        <v>18907</v>
+      </c>
+      <c r="AJ104" t="inlineStr">
+        <is>
+          <t>265963</t>
+        </is>
+      </c>
+      <c r="AK104" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="AL104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>17179</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BORA LYDIA</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>6309196999</v>
+      </c>
+      <c r="D105" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E105" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>08-Dec-2025 17:43:10</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>09-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L105" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N105" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O105" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P105" t="n">
+        <v>11000319830313</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>1765195873</v>
+      </c>
+      <c r="R105" t="n">
+        <v>108720139585</v>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W105" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA105" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB105" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE105" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF105" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG105" t="inlineStr"/>
+      <c r="AH105" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI105" t="n">
+        <v>19894</v>
+      </c>
+      <c r="AJ105" t="inlineStr">
+        <is>
+          <t>264985</t>
+        </is>
+      </c>
+      <c r="AK105" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL105" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove main.py and update output data files
Deleted main.py and updated multiple output data files, including fee collection reports, student lists, and Power BI dashboard. Also replaced an old PostgreSQL backup with a new one. These changes likely reflect a major refactor or migration of the main processing logic and data outputs.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL105"/>
+  <dimension ref="A1:AL129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16512,6 +16512,3678 @@
       </c>
       <c r="AL105" t="inlineStr"/>
     </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>17146</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>RONGALI JASMIKA</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>7793910192</v>
+      </c>
+      <c r="D106" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E106" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>12-Dec-2025 10:57:59</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>15-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L106" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N106" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O106" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P106" t="n">
+        <v>11000340117361</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>1765517263</v>
+      </c>
+      <c r="R106" t="n">
+        <v>534655013098</v>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA106" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB106" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE106" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF106" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG106" t="inlineStr"/>
+      <c r="AH106" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI106" t="n">
+        <v>19849</v>
+      </c>
+      <c r="AJ106" t="inlineStr">
+        <is>
+          <t>265097</t>
+        </is>
+      </c>
+      <c r="AK106" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL106" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>17147</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>RONGALI YERNI VENKATA RAKESH</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>7793910192</v>
+      </c>
+      <c r="D107" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E107" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>12-Dec-2025 10:58:54</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>15-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L107" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N107" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O107" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P107" t="n">
+        <v>11000340117427</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>1765517323</v>
+      </c>
+      <c r="R107" t="n">
+        <v>571217384715</v>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB107" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE107" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF107" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG107" t="inlineStr"/>
+      <c r="AH107" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI107" t="n">
+        <v>19850</v>
+      </c>
+      <c r="AJ107" t="inlineStr">
+        <is>
+          <t>265556</t>
+        </is>
+      </c>
+      <c r="AK107" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL107" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>17370</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>AKKURADA VARUN</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>8500847900</v>
+      </c>
+      <c r="D108" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E108" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>12-Dec-2025 15:19:14</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>15-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L108" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N108" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O108" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P108" t="n">
+        <v>11000340161581</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>1765532834</v>
+      </c>
+      <c r="R108" t="n">
+        <v>108745991711</v>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA108" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB108" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE108" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF108" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG108" t="inlineStr"/>
+      <c r="AH108" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI108" t="n">
+        <v>20089</v>
+      </c>
+      <c r="AJ108" t="inlineStr">
+        <is>
+          <t>268484</t>
+        </is>
+      </c>
+      <c r="AK108" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>17336</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>GOGALAMANDA ASHWIN</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>9133615133</v>
+      </c>
+      <c r="D109" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E109" t="n">
+        <v>10750</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>13-Dec-2025 10:25:13</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L109" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N109" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O109" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P109" t="n">
+        <v>11000340240544</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>1765601703</v>
+      </c>
+      <c r="R109" t="n">
+        <v>790303117843</v>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W109" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA109" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB109" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE109" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF109" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG109" t="inlineStr"/>
+      <c r="AH109" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI109" t="n">
+        <v>20064</v>
+      </c>
+      <c r="AJ109" t="inlineStr">
+        <is>
+          <t>266318</t>
+        </is>
+      </c>
+      <c r="AK109" t="inlineStr">
+        <is>
+          <t>2052</t>
+        </is>
+      </c>
+      <c r="AL109" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>17367</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>EVAAN CHODAM</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>7995919129</v>
+      </c>
+      <c r="D110" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E110" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>13-Dec-2025 15:24:28</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>15-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L110" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N110" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O110" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P110" t="n">
+        <v>11000340278660</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>1765619596</v>
+      </c>
+      <c r="R110" t="n">
+        <v>397896712035</v>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y110" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA110" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB110" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE110" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF110" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG110" t="inlineStr"/>
+      <c r="AH110" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI110" t="n">
+        <v>20086</v>
+      </c>
+      <c r="AJ110" t="inlineStr">
+        <is>
+          <t>268470</t>
+        </is>
+      </c>
+      <c r="AK110" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL110" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>16796</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>MAHENDRA REDDY GUDLA</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>9948345552</v>
+      </c>
+      <c r="D111" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E111" t="n">
+        <v>8650</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>15-Dec-2025 11:57:08</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L111" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N111" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O111" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P111" t="n">
+        <v>11000340453923</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>1765779979</v>
+      </c>
+      <c r="R111" t="n">
+        <v>231872222125</v>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA111" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB111" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE111" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF111" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG111" t="inlineStr"/>
+      <c r="AH111" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI111" t="n">
+        <v>19010</v>
+      </c>
+      <c r="AJ111" t="inlineStr">
+        <is>
+          <t>266145</t>
+        </is>
+      </c>
+      <c r="AK111" t="inlineStr">
+        <is>
+          <t>2051</t>
+        </is>
+      </c>
+      <c r="AL111" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>16797</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>YASHWANTH REDDY GUDLA</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>9948345552</v>
+      </c>
+      <c r="D112" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E112" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>15-Dec-2025 11:58:00</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>16-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L112" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N112" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O112" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P112" t="n">
+        <v>11000340456018</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>1765780062</v>
+      </c>
+      <c r="R112" t="n">
+        <v>717946201991</v>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA112" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB112" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE112" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF112" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG112" t="inlineStr"/>
+      <c r="AH112" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI112" t="n">
+        <v>18786</v>
+      </c>
+      <c r="AJ112" t="inlineStr">
+        <is>
+          <t>265832</t>
+        </is>
+      </c>
+      <c r="AK112" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="AL112" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>16936</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>HARIPRIYA RAVADA</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>6305148581</v>
+      </c>
+      <c r="D113" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E113" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>16-Dec-2025 12:06:31</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>17-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L113" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N113" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O113" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P113" t="n">
+        <v>11000340619866</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>1765866976</v>
+      </c>
+      <c r="R113" t="n">
+        <v>690206926885</v>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA113" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB113" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE113" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF113" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG113" t="inlineStr"/>
+      <c r="AH113" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI113" t="n">
+        <v>18341</v>
+      </c>
+      <c r="AJ113" t="inlineStr">
+        <is>
+          <t>265338</t>
+        </is>
+      </c>
+      <c r="AK113" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="AL113" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>16906</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>RANVITHA SEERA</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>7095076706</v>
+      </c>
+      <c r="D114" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E114" t="n">
+        <v>10750</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>17-Dec-2025 12:40:11</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N114" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O114" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P114" t="n">
+        <v>11000340759102</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>1765955387</v>
+      </c>
+      <c r="R114" t="n">
+        <v>794450161070</v>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA114" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB114" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE114" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF114" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG114" t="inlineStr"/>
+      <c r="AH114" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI114" t="n">
+        <v>19168</v>
+      </c>
+      <c r="AJ114" t="inlineStr">
+        <is>
+          <t>266241</t>
+        </is>
+      </c>
+      <c r="AK114" t="inlineStr">
+        <is>
+          <t>2052</t>
+        </is>
+      </c>
+      <c r="AL114" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>16937</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>VINAYAK KUMAR</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>7396170082</v>
+      </c>
+      <c r="D115" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E115" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>17-Dec-2025 19:39:33</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>18-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L115" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N115" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O115" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P115" t="n">
+        <v>11000340813371</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>1765980521</v>
+      </c>
+      <c r="R115" t="n">
+        <v>108780945784</v>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA115" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB115" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE115" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF115" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG115" t="inlineStr"/>
+      <c r="AH115" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI115" t="n">
+        <v>18292</v>
+      </c>
+      <c r="AJ115" t="inlineStr">
+        <is>
+          <t>265434</t>
+        </is>
+      </c>
+      <c r="AK115" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="AL115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>15621</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>KEERTHANA MUDDA</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>9573036376</v>
+      </c>
+      <c r="D116" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E116" t="n">
+        <v>11350</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>18-Dec-2025 12:09:57</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L116" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N116" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O116" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P116" t="n">
+        <v>11000340878141</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>1766039017</v>
+      </c>
+      <c r="R116" t="n">
+        <v>297705735742</v>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V116" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W116" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X116" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y116" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z116" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA116" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB116" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE116" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF116" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG116" t="inlineStr"/>
+      <c r="AH116" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI116" t="n">
+        <v>19519</v>
+      </c>
+      <c r="AJ116" t="inlineStr">
+        <is>
+          <t>266531</t>
+        </is>
+      </c>
+      <c r="AK116" t="inlineStr">
+        <is>
+          <t>2053</t>
+        </is>
+      </c>
+      <c r="AL116" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>16914</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>SAI SRAVAN PATNAYAK</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>7337422112</v>
+      </c>
+      <c r="D117" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E117" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>18-Dec-2025 17:07:06</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>19-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L117" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N117" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O117" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P117" t="n">
+        <v>11000340919232</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>1766057697</v>
+      </c>
+      <c r="R117" t="n">
+        <v>108787285351</v>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V117" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W117" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y117" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z117" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA117" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB117" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE117" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF117" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG117" t="inlineStr"/>
+      <c r="AH117" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI117" t="n">
+        <v>18066</v>
+      </c>
+      <c r="AJ117" t="inlineStr">
+        <is>
+          <t>265129</t>
+        </is>
+      </c>
+      <c r="AK117" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>16552</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>GANIREDDY ANUHYA</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>9848537189</v>
+      </c>
+      <c r="D118" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E118" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>18-Dec-2025 20:31:47</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>19-Dec-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L118" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N118" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O118" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P118" t="n">
+        <v>11000340940536</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>1766070034</v>
+      </c>
+      <c r="R118" t="n">
+        <v>1.012025352350549e+17</v>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>BANK OF BARODA FSS</t>
+        </is>
+      </c>
+      <c r="V118" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W118" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y118" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="Z118" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA118" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB118" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE118" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF118" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG118" t="inlineStr"/>
+      <c r="AH118" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI118" t="n">
+        <v>18375</v>
+      </c>
+      <c r="AJ118" t="inlineStr">
+        <is>
+          <t>265457</t>
+        </is>
+      </c>
+      <c r="AK118" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>15824</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>GOLAGANI RITHIK NANDHAN</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>9393123464</v>
+      </c>
+      <c r="D119" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E119" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>31-Dec-2025 07:37:12</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>01-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L119" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N119" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O119" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P119" t="n">
+        <v>11000342204411</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>1767145208</v>
+      </c>
+      <c r="R119" t="n">
+        <v>67115244586</v>
+      </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V119" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W119" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X119" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y119" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z119" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA119" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB119" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE119" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF119" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG119" t="inlineStr"/>
+      <c r="AH119" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI119" t="n">
+        <v>18667</v>
+      </c>
+      <c r="AJ119" t="inlineStr">
+        <is>
+          <t>265672</t>
+        </is>
+      </c>
+      <c r="AK119" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL119" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>17188</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>REYANA SRIJITH</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>9985925345</v>
+      </c>
+      <c r="D120" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E120" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>31-Dec-2025 19:23:00</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>01-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L120" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N120" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O120" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P120" t="n">
+        <v>11000342307101</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>1767189156</v>
+      </c>
+      <c r="R120" t="n">
+        <v>108881246730</v>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y120" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA120" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB120" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE120" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF120" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG120" t="inlineStr"/>
+      <c r="AH120" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI120" t="n">
+        <v>19902</v>
+      </c>
+      <c r="AJ120" t="inlineStr">
+        <is>
+          <t>265340</t>
+        </is>
+      </c>
+      <c r="AK120" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="AL120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>16104</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>KARRI ABHINAY CHARVIK</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>9177965994</v>
+      </c>
+      <c r="D121" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E121" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>31-Dec-2025 20:40:26</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>01-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L121" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N121" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O121" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P121" t="n">
+        <v>11000342315290</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>1767193550</v>
+      </c>
+      <c r="R121" t="n">
+        <v>108881815622</v>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA121" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB121" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE121" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG121" t="inlineStr"/>
+      <c r="AH121" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI121" t="n">
+        <v>18807</v>
+      </c>
+      <c r="AJ121" t="inlineStr">
+        <is>
+          <t>267483</t>
+        </is>
+      </c>
+      <c r="AK121" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>16974</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>KADAJARI ESHAN ESWAR</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>9885130099</v>
+      </c>
+      <c r="D122" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E122" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>01-Jan-2026 09:00:50</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>02-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L122" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N122" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O122" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P122" t="n">
+        <v>11000342341005</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>1767238144</v>
+      </c>
+      <c r="R122" t="n">
+        <v>108884026898</v>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V122" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA122" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB122" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE122" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF122" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG122" t="inlineStr"/>
+      <c r="AH122" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI122" t="n">
+        <v>18273</v>
+      </c>
+      <c r="AJ122" t="inlineStr">
+        <is>
+          <t>265390</t>
+        </is>
+      </c>
+      <c r="AK122" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="AL122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>17219</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>VARTIKA KUMARI</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>8369239788</v>
+      </c>
+      <c r="D123" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E123" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>01-Jan-2026 10:46:18</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>02-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L123" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N123" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O123" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P123" t="n">
+        <v>11000342354253</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>1767244559</v>
+      </c>
+      <c r="R123" t="n">
+        <v>104639698103</v>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V123" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y123" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA123" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB123" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE123" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF123" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG123" t="inlineStr"/>
+      <c r="AH123" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI123" t="n">
+        <v>19931</v>
+      </c>
+      <c r="AJ123" t="inlineStr">
+        <is>
+          <t>265205</t>
+        </is>
+      </c>
+      <c r="AK123" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="AL123" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>17211</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>CHENNA JAIKAR ABHIMANYU</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>8074712848</v>
+      </c>
+      <c r="D124" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E124" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>02-Jan-2026 17:33:21</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>03-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L124" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N124" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O124" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P124" t="n">
+        <v>11000342590071</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>1767355353</v>
+      </c>
+      <c r="R124" t="n">
+        <v>108896145112</v>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V124" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA124" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB124" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE124" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF124" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG124" t="inlineStr"/>
+      <c r="AH124" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI124" t="n">
+        <v>19925</v>
+      </c>
+      <c r="AJ124" t="inlineStr">
+        <is>
+          <t>265220</t>
+        </is>
+      </c>
+      <c r="AK124" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="AL124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>17211</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>CHENNA JAIKAR ABHIMANYU</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>8074712848</v>
+      </c>
+      <c r="D125" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E125" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>02-Jan-2026 17:35:15</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>03-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L125" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N125" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O125" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P125" t="n">
+        <v>11000342590128</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>1767355490</v>
+      </c>
+      <c r="R125" t="n">
+        <v>108896159648</v>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA125" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB125" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE125" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF125" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG125" t="inlineStr"/>
+      <c r="AH125" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI125" t="n">
+        <v>19925</v>
+      </c>
+      <c r="AJ125" t="inlineStr">
+        <is>
+          <t>266870</t>
+        </is>
+      </c>
+      <c r="AK125" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="AL125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>17358</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>SAANVI SAHOO</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>8309736856</v>
+      </c>
+      <c r="D126" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E126" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>03-Jan-2026 11:15:36</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>05-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L126" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N126" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O126" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P126" t="n">
+        <v>11000342680749</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>1767419107</v>
+      </c>
+      <c r="R126" t="n">
+        <v>600378887759</v>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W126" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA126" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB126" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE126" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF126" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG126" t="inlineStr"/>
+      <c r="AH126" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI126" t="n">
+        <v>20077</v>
+      </c>
+      <c r="AJ126" t="inlineStr">
+        <is>
+          <t>268294</t>
+        </is>
+      </c>
+      <c r="AK126" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="AL126" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>16507</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>POTNURU YELEENA</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>8374132397</v>
+      </c>
+      <c r="D127" t="n">
+        <v>15500</v>
+      </c>
+      <c r="E127" t="n">
+        <v>15500</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>07-Jan-2026 08:41:12</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>08-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>fifteen thousand five hundred</t>
+        </is>
+      </c>
+      <c r="L127" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N127" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O127" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P127" t="n">
+        <v>11000343525514</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>1767755445</v>
+      </c>
+      <c r="R127" t="n">
+        <v>279709918647</v>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA127" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB127" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC127" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD127" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE127" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF127" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG127" t="inlineStr"/>
+      <c r="AH127" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI127" t="n">
+        <v>18352</v>
+      </c>
+      <c r="AJ127" t="inlineStr">
+        <is>
+          <t>265332,266982</t>
+        </is>
+      </c>
+      <c r="AK127" t="inlineStr">
+        <is>
+          <t>2048,2056</t>
+        </is>
+      </c>
+      <c r="AL127" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>16894</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>SUGGI VENKATA SAI VISHNU VARDHAN</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>8500793683</v>
+      </c>
+      <c r="D128" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E128" t="n">
+        <v>8650</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>07-Jan-2026 17:04:48</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L128" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N128" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O128" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P128" t="n">
+        <v>11000343669593</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>1767785538</v>
+      </c>
+      <c r="R128" t="n">
+        <v>691063181825</v>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z128" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA128" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB128" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC128" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD128" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE128" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF128" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG128" t="inlineStr"/>
+      <c r="AH128" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI128" t="n">
+        <v>19146</v>
+      </c>
+      <c r="AJ128" t="inlineStr">
+        <is>
+          <t>266163</t>
+        </is>
+      </c>
+      <c r="AK128" t="inlineStr">
+        <is>
+          <t>2051</t>
+        </is>
+      </c>
+      <c r="AL128" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>17277</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>EDUBILLI MAHASWIN</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>9618641662</v>
+      </c>
+      <c r="D129" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>10-Jan-2026 09:21:38</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L129" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N129" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O129" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P129" t="n">
+        <v>11000344283491</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>1768017067</v>
+      </c>
+      <c r="R129" t="n">
+        <v>108952003059</v>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA129" t="inlineStr"/>
+      <c r="AB129" t="inlineStr"/>
+      <c r="AC129" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD129" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE129" t="inlineStr"/>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG129" t="inlineStr"/>
+      <c r="AH129" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI129" t="n">
+        <v>19988</v>
+      </c>
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>265125</t>
+        </is>
+      </c>
+      <c r="AK129" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL129" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update fee collection data with new January 2026 entries
Added new fee collection records for late January 2026 across multiple classes and payment modes in daywise_fees_collection.csv, daywise_fees_collection_2025-26.csv, and daywise_fees_collection_online.csv. This update ensures the datasets reflect the latest transactions and receipts for accurate reporting.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL175"/>
+  <dimension ref="A1:AL184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27051,13 +27051,19 @@
       <c r="D175" t="n">
         <v>6750</v>
       </c>
-      <c r="E175" t="inlineStr"/>
+      <c r="E175" t="n">
+        <v>6750</v>
+      </c>
       <c r="F175" t="inlineStr">
         <is>
           <t>28-Jan-2026 13:17:23</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr"/>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>29-Jan-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H175" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -27118,7 +27124,7 @@
       </c>
       <c r="V175" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W175" t="inlineStr">
@@ -27141,15 +27147,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA175" t="inlineStr"/>
-      <c r="AB175" t="inlineStr"/>
+      <c r="AA175" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB175" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC175" t="n">
         <v>0</v>
       </c>
       <c r="AD175" t="n">
         <v>0</v>
       </c>
-      <c r="AE175" t="inlineStr"/>
+      <c r="AE175" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF175" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
@@ -27164,13 +27176,1325 @@
       <c r="AI175" t="n">
         <v>19911</v>
       </c>
-      <c r="AJ175" t="n">
-        <v>266720</v>
-      </c>
-      <c r="AK175" t="n">
-        <v>2055</v>
+      <c r="AJ175" t="inlineStr">
+        <is>
+          <t>266720</t>
+        </is>
+      </c>
+      <c r="AK175" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
       </c>
       <c r="AL175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>15025</v>
+      </c>
+      <c r="B176" t="inlineStr"/>
+      <c r="C176" t="n">
+        <v>6300436983</v>
+      </c>
+      <c r="D176" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E176" t="n">
+        <v>10750</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>28-Jan-2026 22:57:16</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L176" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N176" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O176" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P176" t="n">
+        <v>11000347614077</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>1769621069</v>
+      </c>
+      <c r="R176" t="n">
+        <v>109080979496</v>
+      </c>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V176" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X176" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y176" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z176" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA176" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB176" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC176" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD176" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE176" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF176" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG176" t="inlineStr"/>
+      <c r="AH176" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI176" t="n">
+        <v>19264</v>
+      </c>
+      <c r="AJ176" t="inlineStr">
+        <is>
+          <t>266312</t>
+        </is>
+      </c>
+      <c r="AK176" t="inlineStr">
+        <is>
+          <t>2052</t>
+        </is>
+      </c>
+      <c r="AL176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>14179</v>
+      </c>
+      <c r="B177" t="inlineStr"/>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="n">
+        <v>22700</v>
+      </c>
+      <c r="E177" t="n">
+        <v>22700</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>28-Jan-2026 23:22:31</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>twenty two thousand seven hundred</t>
+        </is>
+      </c>
+      <c r="L177" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N177" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O177" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P177" t="n">
+        <v>11000347616233</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>1769622527</v>
+      </c>
+      <c r="R177" t="n">
+        <v>232254793834</v>
+      </c>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V177" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X177" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y177" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z177" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA177" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB177" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC177" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD177" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE177" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF177" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG177" t="inlineStr"/>
+      <c r="AH177" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI177" t="n">
+        <v>19590</v>
+      </c>
+      <c r="AJ177" t="inlineStr">
+        <is>
+          <t>264853,266503</t>
+        </is>
+      </c>
+      <c r="AK177" t="inlineStr">
+        <is>
+          <t>2045,2053</t>
+        </is>
+      </c>
+      <c r="AL177" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>15938</v>
+      </c>
+      <c r="B178" t="inlineStr"/>
+      <c r="C178" t="n">
+        <v>9959307771</v>
+      </c>
+      <c r="D178" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E178" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>29-Jan-2026 02:05:03</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>30-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L178" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N178" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O178" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P178" t="n">
+        <v>11000347619670</v>
+      </c>
+      <c r="Q178" t="n">
+        <v>1769632447</v>
+      </c>
+      <c r="R178" t="n">
+        <v>109081256624</v>
+      </c>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V178" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X178" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y178" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z178" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA178" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB178" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC178" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD178" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE178" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF178" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG178" t="inlineStr"/>
+      <c r="AH178" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI178" t="n">
+        <v>18863</v>
+      </c>
+      <c r="AJ178" t="inlineStr">
+        <is>
+          <t>267586</t>
+        </is>
+      </c>
+      <c r="AK178" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>15237</v>
+      </c>
+      <c r="B179" t="inlineStr"/>
+      <c r="C179" t="inlineStr"/>
+      <c r="D179" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E179" t="n">
+        <v>8650</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>29-Jan-2026 08:02:15</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L179" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N179" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O179" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P179" t="n">
+        <v>11000347624524</v>
+      </c>
+      <c r="Q179" t="n">
+        <v>1769653866</v>
+      </c>
+      <c r="R179" t="n">
+        <v>109082072826</v>
+      </c>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V179" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X179" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y179" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z179" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA179" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB179" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC179" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD179" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE179" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF179" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG179" t="inlineStr"/>
+      <c r="AH179" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI179" t="n">
+        <v>18984</v>
+      </c>
+      <c r="AJ179" t="inlineStr">
+        <is>
+          <t>266061</t>
+        </is>
+      </c>
+      <c r="AK179" t="inlineStr">
+        <is>
+          <t>2051</t>
+        </is>
+      </c>
+      <c r="AL179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>16148</v>
+      </c>
+      <c r="B180" t="inlineStr"/>
+      <c r="C180" t="n">
+        <v>9573851290</v>
+      </c>
+      <c r="D180" t="n">
+        <v>24650</v>
+      </c>
+      <c r="E180" t="n">
+        <v>24650</v>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>29-Jan-2026 11:43:37</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>30-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>twenty four thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N180" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O180" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P180" t="n">
+        <v>11000347665261</v>
+      </c>
+      <c r="Q180" t="n">
+        <v>1769667026</v>
+      </c>
+      <c r="R180" t="n">
+        <v>109083484020</v>
+      </c>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V180" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X180" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y180" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z180" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA180" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB180" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC180" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD180" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE180" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF180" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG180" t="inlineStr"/>
+      <c r="AH180" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI180" t="n">
+        <v>18502</v>
+      </c>
+      <c r="AJ180" t="inlineStr">
+        <is>
+          <t>262506,263894,265544,267194</t>
+        </is>
+      </c>
+      <c r="AK180" t="inlineStr">
+        <is>
+          <t>2037,2041,2049,2057</t>
+        </is>
+      </c>
+      <c r="AL180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>16147</v>
+      </c>
+      <c r="B181" t="inlineStr"/>
+      <c r="C181" t="n">
+        <v>9573851290</v>
+      </c>
+      <c r="D181" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E181" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>29-Jan-2026 11:48:21</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>30-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L181" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N181" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O181" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P181" t="n">
+        <v>11000347667143</v>
+      </c>
+      <c r="Q181" t="n">
+        <v>1769667469</v>
+      </c>
+      <c r="R181" t="n">
+        <v>109083513527</v>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V181" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X181" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z181" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA181" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB181" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC181" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD181" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE181" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF181" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG181" t="inlineStr"/>
+      <c r="AH181" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI181" t="n">
+        <v>18767</v>
+      </c>
+      <c r="AJ181" t="inlineStr">
+        <is>
+          <t>267440</t>
+        </is>
+      </c>
+      <c r="AK181" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>17210</v>
+      </c>
+      <c r="B182" t="inlineStr"/>
+      <c r="C182" t="n">
+        <v>8985833952</v>
+      </c>
+      <c r="D182" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E182" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>29-Jan-2026 18:54:47</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>30-Jan-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L182" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N182" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O182" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P182" t="n">
+        <v>11000347735867</v>
+      </c>
+      <c r="Q182" t="n">
+        <v>1769693071</v>
+      </c>
+      <c r="R182" t="n">
+        <v>639543409302</v>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V182" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W182" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X182" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z182" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA182" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB182" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC182" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD182" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE182" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF182" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG182" t="inlineStr"/>
+      <c r="AH182" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI182" t="n">
+        <v>19924</v>
+      </c>
+      <c r="AJ182" t="inlineStr">
+        <is>
+          <t>266780</t>
+        </is>
+      </c>
+      <c r="AK182" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL182" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>17370</v>
+      </c>
+      <c r="B183" t="inlineStr"/>
+      <c r="C183" t="n">
+        <v>8500847900</v>
+      </c>
+      <c r="D183" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>30-Jan-2026 10:20:21</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L183" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N183" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O183" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P183" t="n">
+        <v>11000347805222</v>
+      </c>
+      <c r="Q183" t="n">
+        <v>1769748539</v>
+      </c>
+      <c r="R183" t="n">
+        <v>782823183812</v>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z183" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA183" t="inlineStr"/>
+      <c r="AB183" t="inlineStr"/>
+      <c r="AC183" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD183" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE183" t="inlineStr"/>
+      <c r="AF183" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG183" t="inlineStr"/>
+      <c r="AH183" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI183" t="n">
+        <v>20089</v>
+      </c>
+      <c r="AJ183" t="inlineStr">
+        <is>
+          <t>268485</t>
+        </is>
+      </c>
+      <c r="AK183" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL183" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>17061</v>
+      </c>
+      <c r="B184" t="inlineStr"/>
+      <c r="C184" t="n">
+        <v>9701751097</v>
+      </c>
+      <c r="D184" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>30-Jan-2026 22:49:30</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L184" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N184" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O184" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P184" t="n">
+        <v>11000347945459</v>
+      </c>
+      <c r="Q184" t="n">
+        <v>1769793554</v>
+      </c>
+      <c r="R184" t="n">
+        <v>603044734989</v>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V184" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X184" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y184" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z184" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA184" t="inlineStr"/>
+      <c r="AB184" t="inlineStr"/>
+      <c r="AC184" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD184" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE184" t="inlineStr"/>
+      <c r="AF184" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG184" t="inlineStr"/>
+      <c r="AH184" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI184" t="n">
+        <v>19153</v>
+      </c>
+      <c r="AJ184" t="inlineStr">
+        <is>
+          <t>266251</t>
+        </is>
+      </c>
+      <c r="AK184" t="inlineStr">
+        <is>
+          <t>2052</t>
+        </is>
+      </c>
+      <c r="AL184" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update fees collection CSVs and add dashboard
Append recent payment records and reconcile fee statuses across output CSVs (daywise_fees_collection*, daywise_fees_collection_online.csv, fee_transcation_atom_report.csv, fees_collection.csv). Update generated/cleaned source files (atom_report_cleaned.xlsx, source_data/atom_report.xlsx, source_data/merged_fee_collection.csv) and KOTAK_DB notebook. Add a new Postgres backup and update Power BI dashboards (modified existing .pbix files and added Kotak_Dashboard_2025_26_Neon.pbix). These changes reflect payments on 2026-01-31 and 2026-02-02 and corresponding balance updates.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL186"/>
+  <dimension ref="A1:AL200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28235,7 +28235,11 @@
           <t>30-Jan-2026 10:20:21</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>31-Jan-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H183" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -28296,7 +28300,7 @@
       </c>
       <c r="V183" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W183" t="inlineStr">
@@ -28523,13 +28527,19 @@
       <c r="D185" t="n">
         <v>7750</v>
       </c>
-      <c r="E185" t="inlineStr"/>
+      <c r="E185" t="n">
+        <v>7750</v>
+      </c>
       <c r="F185" t="inlineStr">
         <is>
           <t>31-Jan-2026 11:39:53</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr"/>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H185" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -28590,7 +28600,7 @@
       </c>
       <c r="V185" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W185" t="inlineStr">
@@ -28613,15 +28623,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA185" t="inlineStr"/>
-      <c r="AB185" t="inlineStr"/>
+      <c r="AA185" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB185" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC185" t="n">
         <v>0</v>
       </c>
       <c r="AD185" t="n">
         <v>0</v>
       </c>
-      <c r="AE185" t="inlineStr"/>
+      <c r="AE185" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF185" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -28659,13 +28675,19 @@
       <c r="D186" t="n">
         <v>6750</v>
       </c>
-      <c r="E186" t="inlineStr"/>
+      <c r="E186" t="n">
+        <v>6750</v>
+      </c>
       <c r="F186" t="inlineStr">
         <is>
           <t>31-Jan-2026 12:22:53</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr"/>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H186" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -28726,7 +28748,7 @@
       </c>
       <c r="V186" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W186" t="inlineStr">
@@ -28749,15 +28771,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA186" t="inlineStr"/>
-      <c r="AB186" t="inlineStr"/>
+      <c r="AA186" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB186" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC186" t="n">
         <v>0</v>
       </c>
       <c r="AD186" t="n">
         <v>0</v>
       </c>
-      <c r="AE186" t="inlineStr"/>
+      <c r="AE186" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF186" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
@@ -28783,6 +28811,2062 @@
         </is>
       </c>
       <c r="AL186" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>16975</v>
+      </c>
+      <c r="B187" t="inlineStr"/>
+      <c r="C187" t="n">
+        <v>9582803185</v>
+      </c>
+      <c r="D187" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E187" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>31-Jan-2026 18:13:43</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L187" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N187" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O187" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P187" t="n">
+        <v>11000348058030</v>
+      </c>
+      <c r="Q187" t="n">
+        <v>1769863383</v>
+      </c>
+      <c r="R187" t="n">
+        <v>109099158804</v>
+      </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V187" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W187" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X187" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z187" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA187" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB187" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC187" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD187" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE187" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF187" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG187" t="inlineStr"/>
+      <c r="AH187" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI187" t="n">
+        <v>18689</v>
+      </c>
+      <c r="AJ187" t="inlineStr">
+        <is>
+          <t>267419</t>
+        </is>
+      </c>
+      <c r="AK187" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>17203</v>
+      </c>
+      <c r="B188" t="inlineStr"/>
+      <c r="C188" t="n">
+        <v>9582803185</v>
+      </c>
+      <c r="D188" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E188" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>31-Jan-2026 18:17:11</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L188" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N188" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O188" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P188" t="n">
+        <v>11000348058210</v>
+      </c>
+      <c r="Q188" t="n">
+        <v>1769863602</v>
+      </c>
+      <c r="R188" t="n">
+        <v>109099182132</v>
+      </c>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V188" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X188" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y188" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z188" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA188" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB188" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC188" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD188" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE188" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF188" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG188" t="inlineStr"/>
+      <c r="AH188" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI188" t="n">
+        <v>19917</v>
+      </c>
+      <c r="AJ188" t="inlineStr">
+        <is>
+          <t>267156</t>
+        </is>
+      </c>
+      <c r="AK188" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>15610</v>
+      </c>
+      <c r="B189" t="inlineStr"/>
+      <c r="C189" t="n">
+        <v>9494128377</v>
+      </c>
+      <c r="D189" t="n">
+        <v>17200</v>
+      </c>
+      <c r="E189" t="n">
+        <v>17200</v>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>31-Jan-2026 21:10:07</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>seventeen thousand two hundred</t>
+        </is>
+      </c>
+      <c r="L189" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N189" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O189" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P189" t="n">
+        <v>11000348075456</v>
+      </c>
+      <c r="Q189" t="n">
+        <v>1769873832</v>
+      </c>
+      <c r="R189" t="n">
+        <v>211520585120</v>
+      </c>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V189" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X189" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y189" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z189" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA189" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB189" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC189" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD189" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE189" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF189" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG189" t="inlineStr"/>
+      <c r="AH189" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI189" t="n">
+        <v>18708</v>
+      </c>
+      <c r="AJ189" t="inlineStr">
+        <is>
+          <t>262434,264169,265819</t>
+        </is>
+      </c>
+      <c r="AK189" t="inlineStr">
+        <is>
+          <t>2037,2042,2050</t>
+        </is>
+      </c>
+      <c r="AL189" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>17299</v>
+      </c>
+      <c r="B190" t="inlineStr"/>
+      <c r="C190" t="n">
+        <v>9959734686</v>
+      </c>
+      <c r="D190" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E190" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>31-Jan-2026 22:18:47</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L190" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N190" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O190" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P190" t="n">
+        <v>11000348084444</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>1769878103</v>
+      </c>
+      <c r="R190" t="n">
+        <v>261849315319</v>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA190" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB190" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC190" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD190" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE190" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF190" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG190" t="inlineStr"/>
+      <c r="AH190" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI190" t="n">
+        <v>20008</v>
+      </c>
+      <c r="AJ190" t="inlineStr">
+        <is>
+          <t>263349</t>
+        </is>
+      </c>
+      <c r="AK190" t="inlineStr">
+        <is>
+          <t>2039</t>
+        </is>
+      </c>
+      <c r="AL190" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>15237</v>
+      </c>
+      <c r="B191" t="inlineStr"/>
+      <c r="C191" t="n">
+        <v>6300436983</v>
+      </c>
+      <c r="D191" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E191" t="n">
+        <v>8650</v>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 10:10:12</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L191" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N191" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O191" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P191" t="n">
+        <v>11000348259685</v>
+      </c>
+      <c r="Q191" t="n">
+        <v>1770007167</v>
+      </c>
+      <c r="R191" t="n">
+        <v>109110162417</v>
+      </c>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V191" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W191" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X191" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y191" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z191" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA191" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB191" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC191" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD191" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE191" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF191" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG191" t="inlineStr"/>
+      <c r="AH191" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI191" t="n">
+        <v>18984</v>
+      </c>
+      <c r="AJ191" t="inlineStr">
+        <is>
+          <t>268309</t>
+        </is>
+      </c>
+      <c r="AK191" t="inlineStr">
+        <is>
+          <t>2059</t>
+        </is>
+      </c>
+      <c r="AL191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>15025</v>
+      </c>
+      <c r="B192" t="inlineStr"/>
+      <c r="C192" t="n">
+        <v>6300436983</v>
+      </c>
+      <c r="D192" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E192" t="n">
+        <v>10750</v>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 10:11:47</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L192" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N192" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O192" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P192" t="n">
+        <v>11000348259812</v>
+      </c>
+      <c r="Q192" t="n">
+        <v>1770007283</v>
+      </c>
+      <c r="R192" t="n">
+        <v>109110173919</v>
+      </c>
+      <c r="S192" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V192" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W192" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X192" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y192" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z192" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA192" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB192" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC192" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD192" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE192" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF192" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG192" t="inlineStr"/>
+      <c r="AH192" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI192" t="n">
+        <v>19264</v>
+      </c>
+      <c r="AJ192" t="inlineStr">
+        <is>
+          <t>268649</t>
+        </is>
+      </c>
+      <c r="AK192" t="inlineStr">
+        <is>
+          <t>2062</t>
+        </is>
+      </c>
+      <c r="AL192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>17103</v>
+      </c>
+      <c r="B193" t="inlineStr"/>
+      <c r="C193" t="n">
+        <v>6301729629</v>
+      </c>
+      <c r="D193" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E193" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 11:03:20</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>03-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L193" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N193" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O193" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P193" t="n">
+        <v>11000348272865</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>1770010319</v>
+      </c>
+      <c r="R193" t="n">
+        <v>109110496570</v>
+      </c>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X193" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z193" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA193" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB193" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC193" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD193" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE193" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF193" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG193" t="inlineStr"/>
+      <c r="AH193" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI193" t="n">
+        <v>18038</v>
+      </c>
+      <c r="AJ193" t="inlineStr">
+        <is>
+          <t>265086</t>
+        </is>
+      </c>
+      <c r="AK193" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="AL193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>17278</v>
+      </c>
+      <c r="B194" t="inlineStr"/>
+      <c r="C194" t="n">
+        <v>9030736744</v>
+      </c>
+      <c r="D194" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E194" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 12:37:32</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>03-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L194" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N194" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O194" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P194" t="n">
+        <v>11000348296762</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>1770015969</v>
+      </c>
+      <c r="R194" t="n">
+        <v>603396699255</v>
+      </c>
+      <c r="S194" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V194" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W194" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X194" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y194" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z194" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA194" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB194" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC194" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD194" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE194" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF194" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG194" t="inlineStr"/>
+      <c r="AH194" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI194" t="n">
+        <v>19989</v>
+      </c>
+      <c r="AJ194" t="inlineStr">
+        <is>
+          <t>266791</t>
+        </is>
+      </c>
+      <c r="AK194" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL194" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>16983</v>
+      </c>
+      <c r="B195" t="inlineStr"/>
+      <c r="C195" t="n">
+        <v>8919560551</v>
+      </c>
+      <c r="D195" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E195" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 12:51:55</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>03-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L195" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N195" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O195" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P195" t="n">
+        <v>11000348300433</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>1770016889</v>
+      </c>
+      <c r="R195" t="n">
+        <v>109111170783</v>
+      </c>
+      <c r="S195" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W195" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X195" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z195" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA195" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB195" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC195" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD195" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE195" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF195" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG195" t="inlineStr"/>
+      <c r="AH195" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI195" t="n">
+        <v>18526</v>
+      </c>
+      <c r="AJ195" t="inlineStr">
+        <is>
+          <t>265609</t>
+        </is>
+      </c>
+      <c r="AK195" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>16983</v>
+      </c>
+      <c r="B196" t="inlineStr"/>
+      <c r="C196" t="n">
+        <v>8919560551</v>
+      </c>
+      <c r="D196" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E196" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 15:01:40</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>03-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L196" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N196" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O196" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P196" t="n">
+        <v>11000348327211</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>1770024680</v>
+      </c>
+      <c r="R196" t="n">
+        <v>109112112619</v>
+      </c>
+      <c r="S196" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V196" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W196" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X196" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z196" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA196" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB196" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC196" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD196" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE196" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF196" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG196" t="inlineStr"/>
+      <c r="AH196" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI196" t="n">
+        <v>18526</v>
+      </c>
+      <c r="AJ196" t="inlineStr">
+        <is>
+          <t>267259</t>
+        </is>
+      </c>
+      <c r="AK196" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>16981</v>
+      </c>
+      <c r="B197" t="inlineStr"/>
+      <c r="C197" t="n">
+        <v>8919560551</v>
+      </c>
+      <c r="D197" t="n">
+        <v>15500</v>
+      </c>
+      <c r="E197" t="n">
+        <v>15500</v>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 15:03:03</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>03-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>fifteen thousand five hundred</t>
+        </is>
+      </c>
+      <c r="L197" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N197" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O197" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P197" t="n">
+        <v>11000348327327</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>1770024758</v>
+      </c>
+      <c r="R197" t="n">
+        <v>109112123447</v>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W197" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X197" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z197" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA197" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB197" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC197" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD197" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE197" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF197" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG197" t="inlineStr"/>
+      <c r="AH197" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI197" t="n">
+        <v>18142</v>
+      </c>
+      <c r="AJ197" t="inlineStr">
+        <is>
+          <t>265260,266910</t>
+        </is>
+      </c>
+      <c r="AK197" t="inlineStr">
+        <is>
+          <t>2048,2056</t>
+        </is>
+      </c>
+      <c r="AL197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>16046</v>
+      </c>
+      <c r="B198" t="inlineStr"/>
+      <c r="C198" t="n">
+        <v>9177919989</v>
+      </c>
+      <c r="D198" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E198" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>02-Feb-2026 18:47:03</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>03-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L198" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N198" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O198" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P198" t="n">
+        <v>11000348365273</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>1770038166</v>
+      </c>
+      <c r="R198" t="n">
+        <v>109113635360</v>
+      </c>
+      <c r="S198" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X198" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z198" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA198" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB198" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC198" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD198" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE198" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF198" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG198" t="inlineStr"/>
+      <c r="AH198" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI198" t="n">
+        <v>18940</v>
+      </c>
+      <c r="AJ198" t="inlineStr">
+        <is>
+          <t>267616</t>
+        </is>
+      </c>
+      <c r="AK198" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>17149</v>
+      </c>
+      <c r="B199" t="inlineStr"/>
+      <c r="C199" t="n">
+        <v>9989075944</v>
+      </c>
+      <c r="D199" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>03-Feb-2026 12:28:23</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L199" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N199" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O199" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P199" t="n">
+        <v>11000348471340</v>
+      </c>
+      <c r="Q199" t="n">
+        <v>1770101732</v>
+      </c>
+      <c r="R199" t="n">
+        <v>109118392390</v>
+      </c>
+      <c r="S199" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X199" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z199" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA199" t="inlineStr"/>
+      <c r="AB199" t="inlineStr"/>
+      <c r="AC199" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD199" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE199" t="inlineStr"/>
+      <c r="AF199" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG199" t="inlineStr"/>
+      <c r="AH199" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI199" t="n">
+        <v>19852</v>
+      </c>
+      <c r="AJ199" t="inlineStr">
+        <is>
+          <t>266040</t>
+        </is>
+      </c>
+      <c r="AK199" t="inlineStr">
+        <is>
+          <t>2051</t>
+        </is>
+      </c>
+      <c r="AL199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>16992</v>
+      </c>
+      <c r="B200" t="inlineStr"/>
+      <c r="C200" t="n">
+        <v>7207505036</v>
+      </c>
+      <c r="D200" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>03-Feb-2026 20:53:32</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L200" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N200" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O200" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P200" t="n">
+        <v>11000348551835</v>
+      </c>
+      <c r="Q200" t="n">
+        <v>1770132067</v>
+      </c>
+      <c r="R200" t="n">
+        <v>337099556372</v>
+      </c>
+      <c r="S200" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V200" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W200" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X200" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z200" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA200" t="inlineStr"/>
+      <c r="AB200" t="inlineStr"/>
+      <c r="AC200" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD200" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE200" t="inlineStr"/>
+      <c r="AF200" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG200" t="inlineStr"/>
+      <c r="AH200" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI200" t="n">
+        <v>18360</v>
+      </c>
+      <c r="AJ200" t="inlineStr">
+        <is>
+          <t>267018</t>
+        </is>
+      </c>
+      <c r="AK200" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="AL200" t="inlineStr">
         <is>
           <t>UPI INTENT</t>
         </is>

</xml_diff>

<commit_message>
Import new fee transactions & reconcile totals
Append recent payment rows (Feb 3–4) to daywise fee reports (daywise_fees_collection.csv, daywise_fees_collection_2025-26.csv, daywise_fees_collection_online.csv) and add captured/lateUpdate entries to fee_transcation_atom_report.csv. Update fees_collection.csv to reflect reconciled payments for multiple students (Total_Fee_Paid and Total_Due adjusted to show full/updated payments). Add new Postgres backup output_data/postgres_backups/backup_ksdb_2026-02-05_07-09-53.sql and remove the previous 2026-02-04 backup. Also update binary reports/source data (atom_report_cleaned.xlsx, source_data/atom_report.xlsx, source_data/merged_fee_collection.csv) and the PowerBI file (Kotak_Dashboard_2025.pbix) to incorporate the latest data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL200"/>
+  <dimension ref="A1:AL204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30607,7 +30607,9 @@
       <c r="D199" t="n">
         <v>8650</v>
       </c>
-      <c r="E199" t="inlineStr"/>
+      <c r="E199" t="n">
+        <v>8650</v>
+      </c>
       <c r="F199" t="inlineStr">
         <is>
           <t>03-Feb-2026 12:28:23</t>
@@ -30674,7 +30676,7 @@
       </c>
       <c r="V199" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W199" t="inlineStr">
@@ -30697,15 +30699,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA199" t="inlineStr"/>
-      <c r="AB199" t="inlineStr"/>
+      <c r="AA199" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB199" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC199" t="n">
         <v>0</v>
       </c>
       <c r="AD199" t="n">
         <v>0</v>
       </c>
-      <c r="AE199" t="inlineStr"/>
+      <c r="AE199" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF199" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
@@ -30743,13 +30751,19 @@
       <c r="D200" t="n">
         <v>7750</v>
       </c>
-      <c r="E200" t="inlineStr"/>
+      <c r="E200" t="n">
+        <v>7750</v>
+      </c>
       <c r="F200" t="inlineStr">
         <is>
           <t>03-Feb-2026 20:53:32</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>04-Feb-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H200" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -30810,7 +30824,7 @@
       </c>
       <c r="V200" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W200" t="inlineStr">
@@ -30833,15 +30847,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA200" t="inlineStr"/>
-      <c r="AB200" t="inlineStr"/>
+      <c r="AA200" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB200" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC200" t="n">
         <v>0</v>
       </c>
       <c r="AD200" t="n">
         <v>0</v>
       </c>
-      <c r="AE200" t="inlineStr"/>
+      <c r="AE200" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF200" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -30871,6 +30891,558 @@
           <t>UPI INTENT</t>
         </is>
       </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>17307</v>
+      </c>
+      <c r="B201" t="inlineStr"/>
+      <c r="C201" t="n">
+        <v>9991367333</v>
+      </c>
+      <c r="D201" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>04-Feb-2026 07:05:09</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L201" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N201" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O201" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P201" t="n">
+        <v>11000348575099</v>
+      </c>
+      <c r="Q201" t="n">
+        <v>1770168829</v>
+      </c>
+      <c r="R201" t="n">
+        <v>109123051045</v>
+      </c>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W201" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X201" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z201" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA201" t="inlineStr"/>
+      <c r="AB201" t="inlineStr"/>
+      <c r="AC201" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD201" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE201" t="inlineStr"/>
+      <c r="AF201" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG201" t="inlineStr"/>
+      <c r="AH201" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI201" t="n">
+        <v>20016</v>
+      </c>
+      <c r="AJ201" t="inlineStr">
+        <is>
+          <t>267480</t>
+        </is>
+      </c>
+      <c r="AK201" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>17069</v>
+      </c>
+      <c r="B202" t="inlineStr"/>
+      <c r="C202" t="n">
+        <v>8885883431</v>
+      </c>
+      <c r="D202" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>04-Feb-2026 09:56:04</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L202" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N202" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O202" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P202" t="n">
+        <v>11000348596178</v>
+      </c>
+      <c r="Q202" t="n">
+        <v>1770179127</v>
+      </c>
+      <c r="R202" t="n">
+        <v>496896024593</v>
+      </c>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W202" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X202" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z202" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA202" t="inlineStr"/>
+      <c r="AB202" t="inlineStr"/>
+      <c r="AC202" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD202" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE202" t="inlineStr"/>
+      <c r="AF202" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG202" t="inlineStr"/>
+      <c r="AH202" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI202" t="n">
+        <v>18960</v>
+      </c>
+      <c r="AJ202" t="inlineStr">
+        <is>
+          <t>267577</t>
+        </is>
+      </c>
+      <c r="AK202" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL202" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>15728</v>
+      </c>
+      <c r="B203" t="inlineStr"/>
+      <c r="C203" t="n">
+        <v>7893025312</v>
+      </c>
+      <c r="D203" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>04-Feb-2026 10:05:07</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L203" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N203" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O203" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P203" t="n">
+        <v>11000348597736</v>
+      </c>
+      <c r="Q203" t="n">
+        <v>1770179690</v>
+      </c>
+      <c r="R203" t="n">
+        <v>230527479236</v>
+      </c>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V203" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W203" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X203" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y203" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z203" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA203" t="inlineStr"/>
+      <c r="AB203" t="inlineStr"/>
+      <c r="AC203" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD203" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE203" t="inlineStr"/>
+      <c r="AF203" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG203" t="inlineStr"/>
+      <c r="AH203" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI203" t="n">
+        <v>19462</v>
+      </c>
+      <c r="AJ203" t="inlineStr">
+        <is>
+          <t>268164</t>
+        </is>
+      </c>
+      <c r="AK203" t="inlineStr">
+        <is>
+          <t>2061</t>
+        </is>
+      </c>
+      <c r="AL203" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>15541</v>
+      </c>
+      <c r="B204" t="inlineStr"/>
+      <c r="C204" t="n">
+        <v>9849969449</v>
+      </c>
+      <c r="D204" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>04-Feb-2026 23:05:27</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L204" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N204" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O204" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P204" t="n">
+        <v>11000348724700</v>
+      </c>
+      <c r="Q204" t="n">
+        <v>1770226187</v>
+      </c>
+      <c r="R204" t="n">
+        <v>109128651847</v>
+      </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W204" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X204" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y204" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z204" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA204" t="inlineStr"/>
+      <c r="AB204" t="inlineStr"/>
+      <c r="AC204" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD204" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE204" t="inlineStr"/>
+      <c r="AF204" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG204" t="inlineStr"/>
+      <c r="AH204" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI204" t="n">
+        <v>18766</v>
+      </c>
+      <c r="AJ204" t="inlineStr">
+        <is>
+          <t>265813</t>
+        </is>
+      </c>
+      <c r="AK204" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="AL204" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refresh reports and exported data
Regenerated and updated several output and source data files: refreshed atom_report_cleaned.xlsx, multiple daywise_fees_collection CSVs (including reordering/cleaning of entries), fee transaction and fees report CSVs, and merged_fee_collection/source atom_report.xlsx. Replaced postgres backup with a new dated dump, and updated Power BI dashboard (.pbix) and KOTAK_DB notebook. These changes reflect an updated export/backup cycle and cleaned fee collection data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -30903,13 +30903,19 @@
       <c r="D201" t="n">
         <v>8350</v>
       </c>
-      <c r="E201" t="inlineStr"/>
+      <c r="E201" t="n">
+        <v>8350</v>
+      </c>
       <c r="F201" t="inlineStr">
         <is>
           <t>04-Feb-2026 07:05:09</t>
         </is>
       </c>
-      <c r="G201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>05-Feb-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H201" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -30970,7 +30976,7 @@
       </c>
       <c r="V201" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W201" t="inlineStr">
@@ -30993,15 +30999,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA201" t="inlineStr"/>
-      <c r="AB201" t="inlineStr"/>
+      <c r="AA201" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB201" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC201" t="n">
         <v>0</v>
       </c>
       <c r="AD201" t="n">
         <v>0</v>
       </c>
-      <c r="AE201" t="inlineStr"/>
+      <c r="AE201" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF201" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -31039,13 +31051,19 @@
       <c r="D202" t="n">
         <v>8350</v>
       </c>
-      <c r="E202" t="inlineStr"/>
+      <c r="E202" t="n">
+        <v>8350</v>
+      </c>
       <c r="F202" t="inlineStr">
         <is>
           <t>04-Feb-2026 09:56:04</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr"/>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>05-Feb-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H202" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -31106,7 +31124,7 @@
       </c>
       <c r="V202" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W202" t="inlineStr">
@@ -31129,15 +31147,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA202" t="inlineStr"/>
-      <c r="AB202" t="inlineStr"/>
+      <c r="AA202" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB202" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC202" t="n">
         <v>0</v>
       </c>
       <c r="AD202" t="n">
         <v>0</v>
       </c>
-      <c r="AE202" t="inlineStr"/>
+      <c r="AE202" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF202" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -31179,7 +31203,9 @@
       <c r="D203" t="n">
         <v>11350</v>
       </c>
-      <c r="E203" t="inlineStr"/>
+      <c r="E203" t="n">
+        <v>11350</v>
+      </c>
       <c r="F203" t="inlineStr">
         <is>
           <t>04-Feb-2026 10:05:07</t>
@@ -31246,7 +31272,7 @@
       </c>
       <c r="V203" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W203" t="inlineStr">
@@ -31269,15 +31295,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA203" t="inlineStr"/>
-      <c r="AB203" t="inlineStr"/>
+      <c r="AA203" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB203" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC203" t="n">
         <v>0</v>
       </c>
       <c r="AD203" t="n">
         <v>0</v>
       </c>
-      <c r="AE203" t="inlineStr"/>
+      <c r="AE203" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF203" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -31319,13 +31351,19 @@
       <c r="D204" t="n">
         <v>8350</v>
       </c>
-      <c r="E204" t="inlineStr"/>
+      <c r="E204" t="n">
+        <v>8350</v>
+      </c>
       <c r="F204" t="inlineStr">
         <is>
           <t>04-Feb-2026 23:05:27</t>
         </is>
       </c>
-      <c r="G204" t="inlineStr"/>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>05-Feb-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H204" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -31386,7 +31424,7 @@
       </c>
       <c r="V204" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W204" t="inlineStr">
@@ -31409,15 +31447,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA204" t="inlineStr"/>
-      <c r="AB204" t="inlineStr"/>
+      <c r="AA204" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB204" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC204" t="n">
         <v>0</v>
       </c>
       <c r="AD204" t="n">
         <v>0</v>
       </c>
-      <c r="AE204" t="inlineStr"/>
+      <c r="AE204" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF204" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>

</xml_diff>

<commit_message>
Refresh generated reports; add new DB backup
Update output reports and source data with latest fee and student records. Modified multiple files under output_data (atom_report_cleaned.xlsx, daywise_fees_collection.csv and its per-year/online variants, fee_concession_report.csv and combined, fee_transcation_atom_report.csv, fees_collection.csv, fees_report.csv, student_list.csv, students_data.csv). Removed old backup_ksdb_2026-02-06 and added new postgres backup backup_ksdb_2026-02-20. Also updated Power BI dashboards (KOTAK_DBMS_DASHBOARD.pbix, Kotak_Dashboard_2025.pbix), notebook (source_code/KOTAK_DB.ipynb), and refreshed source_data (atom_report.xlsx, merged_fee_collection.csv) to reflect current data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL204"/>
+  <dimension ref="A1:AL222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31488,6 +31488,2710 @@
       </c>
       <c r="AL204" t="inlineStr"/>
     </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>16400</v>
+      </c>
+      <c r="B205" t="inlineStr"/>
+      <c r="C205" t="n">
+        <v>9542502425</v>
+      </c>
+      <c r="D205" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E205" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>06-Feb-2026 15:42:50</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>07-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L205" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N205" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O205" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P205" t="n">
+        <v>11000348990079</v>
+      </c>
+      <c r="Q205" t="n">
+        <v>1770372650</v>
+      </c>
+      <c r="R205" t="n">
+        <v>696631043153</v>
+      </c>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V205" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W205" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X205" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y205" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z205" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA205" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB205" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC205" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD205" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE205" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF205" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG205" t="inlineStr"/>
+      <c r="AH205" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI205" t="n">
+        <v>18422</v>
+      </c>
+      <c r="AJ205" t="inlineStr">
+        <is>
+          <t>267145</t>
+        </is>
+      </c>
+      <c r="AK205" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL205" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>15762</v>
+      </c>
+      <c r="B206" t="inlineStr"/>
+      <c r="C206" t="n">
+        <v>9505890135</v>
+      </c>
+      <c r="D206" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E206" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>07-Feb-2026 11:49:02</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>09-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L206" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N206" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O206" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P206" t="n">
+        <v>11000349086368</v>
+      </c>
+      <c r="Q206" t="n">
+        <v>1770445075</v>
+      </c>
+      <c r="R206" t="n">
+        <v>109145651654</v>
+      </c>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V206" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W206" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X206" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y206" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z206" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA206" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB206" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC206" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD206" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE206" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF206" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG206" t="inlineStr"/>
+      <c r="AH206" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI206" t="n">
+        <v>18805</v>
+      </c>
+      <c r="AJ206" t="inlineStr">
+        <is>
+          <t>267429</t>
+        </is>
+      </c>
+      <c r="AK206" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>17229</v>
+      </c>
+      <c r="B207" t="inlineStr"/>
+      <c r="C207" t="n">
+        <v>9985965602</v>
+      </c>
+      <c r="D207" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E207" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>08-Feb-2026 12:35:23</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>09-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L207" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N207" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O207" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P207" t="n">
+        <v>11000349188445</v>
+      </c>
+      <c r="Q207" t="n">
+        <v>1770534277</v>
+      </c>
+      <c r="R207" t="n">
+        <v>773499900668</v>
+      </c>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V207" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W207" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X207" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y207" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z207" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA207" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB207" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC207" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD207" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE207" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF207" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG207" t="inlineStr"/>
+      <c r="AH207" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI207" t="n">
+        <v>19941</v>
+      </c>
+      <c r="AJ207" t="inlineStr">
+        <is>
+          <t>267541</t>
+        </is>
+      </c>
+      <c r="AK207" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL207" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>16342</v>
+      </c>
+      <c r="B208" t="inlineStr"/>
+      <c r="C208" t="n">
+        <v>9866955786</v>
+      </c>
+      <c r="D208" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E208" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>08-Feb-2026 14:40:50</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>09-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L208" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N208" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O208" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P208" t="n">
+        <v>11000349199255</v>
+      </c>
+      <c r="Q208" t="n">
+        <v>1770541823</v>
+      </c>
+      <c r="R208" t="n">
+        <v>89695506546</v>
+      </c>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V208" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W208" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X208" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y208" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z208" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA208" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB208" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC208" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD208" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE208" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF208" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG208" t="inlineStr"/>
+      <c r="AH208" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI208" t="n">
+        <v>18265</v>
+      </c>
+      <c r="AJ208" t="inlineStr">
+        <is>
+          <t>267000</t>
+        </is>
+      </c>
+      <c r="AK208" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="AL208" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>16052</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>GURRALA RUSHABH NARAYAN</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>9704995001</v>
+      </c>
+      <c r="D209" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E209" t="n">
+        <v>10750</v>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>09-Feb-2026 21:49:08</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr"/>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L209" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N209" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O209" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P209" t="n">
+        <v>11000349412641</v>
+      </c>
+      <c r="Q209" t="n">
+        <v>1770653878</v>
+      </c>
+      <c r="R209" t="n">
+        <v>109162303649</v>
+      </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V209" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W209" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X209" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y209" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z209" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA209" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB209" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC209" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD209" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE209" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF209" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG209" t="inlineStr"/>
+      <c r="AH209" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI209" t="n">
+        <v>19325</v>
+      </c>
+      <c r="AJ209" t="inlineStr">
+        <is>
+          <t>268659</t>
+        </is>
+      </c>
+      <c r="AK209" t="inlineStr">
+        <is>
+          <t>2062</t>
+        </is>
+      </c>
+      <c r="AL209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>16167</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>VELAMALA LAKSHITHA</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>8886569151</v>
+      </c>
+      <c r="D210" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E210" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>10-Feb-2026 07:23:05</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>11-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L210" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N210" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O210" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P210" t="n">
+        <v>11000349433264</v>
+      </c>
+      <c r="Q210" t="n">
+        <v>1770688284</v>
+      </c>
+      <c r="R210" t="n">
+        <v>109163767115</v>
+      </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V210" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W210" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X210" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y210" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z210" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA210" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB210" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE210" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF210" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG210" t="inlineStr"/>
+      <c r="AH210" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI210" t="n">
+        <v>18687</v>
+      </c>
+      <c r="AJ210" t="inlineStr">
+        <is>
+          <t>265804</t>
+        </is>
+      </c>
+      <c r="AK210" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="AL210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>16353</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>RETOJI HRIDAYANSH VICTOR</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>9395553084</v>
+      </c>
+      <c r="D211" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E211" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>10-Feb-2026 17:03:05</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>11-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L211" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N211" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O211" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P211" t="n">
+        <v>11000349550616</v>
+      </c>
+      <c r="Q211" t="n">
+        <v>1770723058</v>
+      </c>
+      <c r="R211" t="n">
+        <v>109167537406</v>
+      </c>
+      <c r="S211" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V211" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W211" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X211" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y211" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z211" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA211" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB211" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE211" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF211" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG211" t="inlineStr"/>
+      <c r="AH211" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI211" t="n">
+        <v>18469</v>
+      </c>
+      <c r="AJ211" t="inlineStr">
+        <is>
+          <t>265534</t>
+        </is>
+      </c>
+      <c r="AK211" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>17260</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>SIDDI SHANMUKHA SAI MANI DEEPANSH</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>6305761566</v>
+      </c>
+      <c r="D212" t="n">
+        <v>16700</v>
+      </c>
+      <c r="E212" t="n">
+        <v>16700</v>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>11-Feb-2026 07:45:40</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>12-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>sixteen thousand seven hundred</t>
+        </is>
+      </c>
+      <c r="L212" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N212" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O212" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P212" t="n">
+        <v>11000349611971</v>
+      </c>
+      <c r="Q212" t="n">
+        <v>1770776081</v>
+      </c>
+      <c r="R212" t="n">
+        <v>109170679443</v>
+      </c>
+      <c r="S212" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V212" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W212" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X212" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y212" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z212" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA212" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB212" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE212" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF212" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG212" t="inlineStr"/>
+      <c r="AH212" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI212" t="n">
+        <v>19972</v>
+      </c>
+      <c r="AJ212" t="inlineStr">
+        <is>
+          <t>265869,267519</t>
+        </is>
+      </c>
+      <c r="AK212" t="inlineStr">
+        <is>
+          <t>2050,2058</t>
+        </is>
+      </c>
+      <c r="AL212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>17259</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>SIDDI SHANMUKHA SESA SAI DHANUSH</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>6305761566</v>
+      </c>
+      <c r="D213" t="n">
+        <v>21500</v>
+      </c>
+      <c r="E213" t="n">
+        <v>21500</v>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>11-Feb-2026 08:00:22</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr"/>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>twenty one thousand five hundred</t>
+        </is>
+      </c>
+      <c r="L213" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N213" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O213" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P213" t="n">
+        <v>11000349612523</v>
+      </c>
+      <c r="Q213" t="n">
+        <v>1770776819</v>
+      </c>
+      <c r="R213" t="n">
+        <v>109170756189</v>
+      </c>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V213" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W213" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X213" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y213" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z213" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA213" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB213" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE213" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF213" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG213" t="inlineStr"/>
+      <c r="AH213" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI213" t="n">
+        <v>19971</v>
+      </c>
+      <c r="AJ213" t="inlineStr">
+        <is>
+          <t>266353,268690</t>
+        </is>
+      </c>
+      <c r="AK213" t="inlineStr">
+        <is>
+          <t>2052,2062</t>
+        </is>
+      </c>
+      <c r="AL213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>16615</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>RAKESH NAMMI</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>9502806409</v>
+      </c>
+      <c r="D214" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E214" t="n">
+        <v>8650</v>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>13-Feb-2026 08:29:21</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L214" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N214" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O214" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P214" t="n">
+        <v>11000349933934</v>
+      </c>
+      <c r="Q214" t="n">
+        <v>1770951465</v>
+      </c>
+      <c r="R214" t="n">
+        <v>456479327537</v>
+      </c>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V214" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W214" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X214" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y214" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z214" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA214" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB214" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE214" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF214" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG214" t="inlineStr"/>
+      <c r="AH214" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI214" t="n">
+        <v>19097</v>
+      </c>
+      <c r="AJ214" t="inlineStr">
+        <is>
+          <t>268335</t>
+        </is>
+      </c>
+      <c r="AK214" t="inlineStr">
+        <is>
+          <t>2059</t>
+        </is>
+      </c>
+      <c r="AL214" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>14652</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>HEMANTH NAMMI</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>9502806409</v>
+      </c>
+      <c r="D215" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E215" t="n">
+        <v>11350</v>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>13-Feb-2026 08:30:55</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L215" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N215" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O215" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P215" t="n">
+        <v>11000349933992</v>
+      </c>
+      <c r="Q215" t="n">
+        <v>1770951642</v>
+      </c>
+      <c r="R215" t="n">
+        <v>186282312824</v>
+      </c>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V215" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W215" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X215" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y215" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z215" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA215" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB215" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC215" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD215" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE215" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF215" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG215" t="inlineStr"/>
+      <c r="AH215" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI215" t="n">
+        <v>19448</v>
+      </c>
+      <c r="AJ215" t="inlineStr">
+        <is>
+          <t>268100</t>
+        </is>
+      </c>
+      <c r="AK215" t="inlineStr">
+        <is>
+          <t>2061</t>
+        </is>
+      </c>
+      <c r="AL215" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>17367</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>EVAAN CHODAM</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>7995919129</v>
+      </c>
+      <c r="D216" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E216" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>13-Feb-2026 09:38:08</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>16-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L216" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N216" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O216" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P216" t="n">
+        <v>11000349945161</v>
+      </c>
+      <c r="Q216" t="n">
+        <v>1770955661</v>
+      </c>
+      <c r="R216" t="n">
+        <v>834632436491</v>
+      </c>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V216" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W216" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X216" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y216" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z216" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA216" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB216" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC216" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD216" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE216" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF216" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG216" t="inlineStr"/>
+      <c r="AH216" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI216" t="n">
+        <v>20086</v>
+      </c>
+      <c r="AJ216" t="inlineStr">
+        <is>
+          <t>268471</t>
+        </is>
+      </c>
+      <c r="AK216" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL216" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>15952</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>AFREEN BEGUM</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>8099960677</v>
+      </c>
+      <c r="D217" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E217" t="n">
+        <v>11350</v>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>13-Feb-2026 18:18:42</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L217" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N217" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O217" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P217" t="n">
+        <v>11000350040172</v>
+      </c>
+      <c r="Q217" t="n">
+        <v>1770986795</v>
+      </c>
+      <c r="R217" t="n">
+        <v>321558195549</v>
+      </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V217" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W217" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X217" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y217" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z217" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA217" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB217" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC217" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD217" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE217" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF217" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG217" t="inlineStr"/>
+      <c r="AH217" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI217" t="n">
+        <v>19419</v>
+      </c>
+      <c r="AJ217" t="inlineStr">
+        <is>
+          <t>268015</t>
+        </is>
+      </c>
+      <c r="AK217" t="inlineStr">
+        <is>
+          <t>2061</t>
+        </is>
+      </c>
+      <c r="AL217" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>15009</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>GOLAGANI GEETHANJALI</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>9393123464</v>
+      </c>
+      <c r="D218" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E218" t="n">
+        <v>8650</v>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>14-Feb-2026 08:24:58</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L218" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N218" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O218" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P218" t="n">
+        <v>11000350075558</v>
+      </c>
+      <c r="Q218" t="n">
+        <v>1771037667</v>
+      </c>
+      <c r="R218" t="n">
+        <v>759841106307</v>
+      </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V218" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W218" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X218" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y218" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z218" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA218" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB218" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC218" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD218" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE218" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF218" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG218" t="inlineStr"/>
+      <c r="AH218" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI218" t="n">
+        <v>19026</v>
+      </c>
+      <c r="AJ218" t="inlineStr">
+        <is>
+          <t>266050</t>
+        </is>
+      </c>
+      <c r="AK218" t="inlineStr">
+        <is>
+          <t>2051</t>
+        </is>
+      </c>
+      <c r="AL218" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>15095</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>KORUKONDA KALYANI</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>9885668424</v>
+      </c>
+      <c r="D219" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E219" t="n">
+        <v>11350</v>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>17-Feb-2026 09:06:11</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L219" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N219" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O219" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P219" t="n">
+        <v>11000350432476</v>
+      </c>
+      <c r="Q219" t="n">
+        <v>1771299354</v>
+      </c>
+      <c r="R219" t="n">
+        <v>387026729931</v>
+      </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V219" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W219" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X219" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y219" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z219" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA219" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB219" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC219" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD219" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE219" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF219" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG219" t="inlineStr"/>
+      <c r="AH219" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI219" t="n">
+        <v>19580</v>
+      </c>
+      <c r="AJ219" t="inlineStr">
+        <is>
+          <t>268160</t>
+        </is>
+      </c>
+      <c r="AK219" t="inlineStr">
+        <is>
+          <t>2061</t>
+        </is>
+      </c>
+      <c r="AL219" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>16615</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>RAKESH NAMMI</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>9502806409</v>
+      </c>
+      <c r="D220" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>18-Feb-2026 10:49:40</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L220" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N220" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O220" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P220" t="n">
+        <v>11000350603509</v>
+      </c>
+      <c r="Q220" t="n">
+        <v>1771391968</v>
+      </c>
+      <c r="R220" t="n">
+        <v>821324645171</v>
+      </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V220" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W220" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X220" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y220" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z220" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA220" t="inlineStr"/>
+      <c r="AB220" t="inlineStr"/>
+      <c r="AC220" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD220" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE220" t="inlineStr"/>
+      <c r="AF220" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG220" t="inlineStr"/>
+      <c r="AH220" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI220" t="n">
+        <v>19097</v>
+      </c>
+      <c r="AJ220" t="inlineStr">
+        <is>
+          <t>266170</t>
+        </is>
+      </c>
+      <c r="AK220" t="inlineStr">
+        <is>
+          <t>2051</t>
+        </is>
+      </c>
+      <c r="AL220" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>15618</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>CHINTAPALLI CHANDINI</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>9985304942</v>
+      </c>
+      <c r="D221" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>18-Feb-2026 20:11:30</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L221" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N221" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O221" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P221" t="n">
+        <v>11000350731551</v>
+      </c>
+      <c r="Q221" t="n">
+        <v>1771425670</v>
+      </c>
+      <c r="R221" t="n">
+        <v>163162136750</v>
+      </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V221" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W221" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X221" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y221" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z221" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA221" t="inlineStr"/>
+      <c r="AB221" t="inlineStr"/>
+      <c r="AC221" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD221" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE221" t="inlineStr"/>
+      <c r="AF221" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG221" t="inlineStr"/>
+      <c r="AH221" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI221" t="n">
+        <v>18866</v>
+      </c>
+      <c r="AJ221" t="inlineStr">
+        <is>
+          <t>267547</t>
+        </is>
+      </c>
+      <c r="AK221" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL221" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>14706</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>CHINTAPALLI CHATHAN SWAROOP</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>9985304942</v>
+      </c>
+      <c r="D222" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>18-Feb-2026 20:13:07</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L222" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N222" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O222" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P222" t="n">
+        <v>11000350731636</v>
+      </c>
+      <c r="Q222" t="n">
+        <v>1771425769</v>
+      </c>
+      <c r="R222" t="n">
+        <v>842044167452</v>
+      </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U222" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V222" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W222" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X222" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y222" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z222" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA222" t="inlineStr"/>
+      <c r="AB222" t="inlineStr"/>
+      <c r="AC222" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD222" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE222" t="inlineStr"/>
+      <c r="AF222" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG222" t="inlineStr"/>
+      <c r="AH222" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI222" t="n">
+        <v>19397</v>
+      </c>
+      <c r="AJ222" t="inlineStr">
+        <is>
+          <t>268068</t>
+        </is>
+      </c>
+      <c r="AK222" t="inlineStr">
+        <is>
+          <t>2061</t>
+        </is>
+      </c>
+      <c r="AL222" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh reports, backups and source data
Refresh generated data and assets: updated multiple output CSVs/Excel files (including daywise_fees_collection.csv and atom_report_cleaned.xlsx) to include recent fee transactions through Feb 2026, updated other fees reports, refreshed source_data/atom_report.xlsx and merged_fee_collection.csv, updated Power BI dashboard (Kotak_Dashboard_2025.pbix), and rotated/renamed the postgres backup in output_data/postgres_backups. Routine refresh to incorporate latest transactions and a new backup snapshot.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL222"/>
+  <dimension ref="A1:AL250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33775,7 +33775,9 @@
       <c r="D220" t="n">
         <v>8650</v>
       </c>
-      <c r="E220" t="inlineStr"/>
+      <c r="E220" t="n">
+        <v>8650</v>
+      </c>
       <c r="F220" t="inlineStr">
         <is>
           <t>18-Feb-2026 10:49:40</t>
@@ -33842,7 +33844,7 @@
       </c>
       <c r="V220" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W220" t="inlineStr">
@@ -33865,15 +33867,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA220" t="inlineStr"/>
-      <c r="AB220" t="inlineStr"/>
+      <c r="AA220" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB220" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC220" t="n">
         <v>0</v>
       </c>
       <c r="AD220" t="n">
         <v>0</v>
       </c>
-      <c r="AE220" t="inlineStr"/>
+      <c r="AE220" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF220" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
@@ -33919,13 +33927,19 @@
       <c r="D221" t="n">
         <v>8350</v>
       </c>
-      <c r="E221" t="inlineStr"/>
+      <c r="E221" t="n">
+        <v>8350</v>
+      </c>
       <c r="F221" t="inlineStr">
         <is>
           <t>18-Feb-2026 20:11:30</t>
         </is>
       </c>
-      <c r="G221" t="inlineStr"/>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>20-Feb-2026 00:00:00</t>
+        </is>
+      </c>
       <c r="H221" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -33986,7 +34000,7 @@
       </c>
       <c r="V221" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W221" t="inlineStr">
@@ -34009,15 +34023,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA221" t="inlineStr"/>
-      <c r="AB221" t="inlineStr"/>
+      <c r="AA221" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB221" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC221" t="n">
         <v>0</v>
       </c>
       <c r="AD221" t="n">
         <v>0</v>
       </c>
-      <c r="AE221" t="inlineStr"/>
+      <c r="AE221" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF221" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -34063,7 +34083,9 @@
       <c r="D222" t="n">
         <v>11350</v>
       </c>
-      <c r="E222" t="inlineStr"/>
+      <c r="E222" t="n">
+        <v>11350</v>
+      </c>
       <c r="F222" t="inlineStr">
         <is>
           <t>18-Feb-2026 20:13:07</t>
@@ -34130,7 +34152,7 @@
       </c>
       <c r="V222" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W222" t="inlineStr">
@@ -34153,15 +34175,21 @@
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="AA222" t="inlineStr"/>
-      <c r="AB222" t="inlineStr"/>
+      <c r="AA222" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB222" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC222" t="n">
         <v>0</v>
       </c>
       <c r="AD222" t="n">
         <v>0</v>
       </c>
-      <c r="AE222" t="inlineStr"/>
+      <c r="AE222" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF222" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -34187,6 +34215,4230 @@
         </is>
       </c>
       <c r="AL222" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>14888</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>SHAIK GOUSIA NASRIN</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>7207749584</v>
+      </c>
+      <c r="D223" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E223" t="n">
+        <v>10750</v>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>20-Feb-2026 07:56:35</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr"/>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L223" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N223" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O223" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P223" t="n">
+        <v>11000350963982</v>
+      </c>
+      <c r="Q223" t="n">
+        <v>1771554340</v>
+      </c>
+      <c r="R223" t="n">
+        <v>109227319525</v>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T223" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U223" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V223" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W223" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X223" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y223" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z223" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA223" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB223" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC223" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD223" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE223" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF223" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG223" t="inlineStr"/>
+      <c r="AH223" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI223" t="n">
+        <v>19200</v>
+      </c>
+      <c r="AJ223" t="inlineStr">
+        <is>
+          <t>266268</t>
+        </is>
+      </c>
+      <c r="AK223" t="inlineStr">
+        <is>
+          <t>2052</t>
+        </is>
+      </c>
+      <c r="AL223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>17188</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>REYANA SRIJITH</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>9985925345</v>
+      </c>
+      <c r="D224" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E224" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>22-Feb-2026 12:39:56</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>23-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L224" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N224" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O224" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P224" t="n">
+        <v>11000351187164</v>
+      </c>
+      <c r="Q224" t="n">
+        <v>1771744152</v>
+      </c>
+      <c r="R224" t="n">
+        <v>109240823792</v>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T224" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V224" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W224" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X224" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y224" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z224" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA224" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB224" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC224" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD224" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE224" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF224" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG224" t="inlineStr"/>
+      <c r="AH224" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI224" t="n">
+        <v>19902</v>
+      </c>
+      <c r="AJ224" t="inlineStr">
+        <is>
+          <t>266990</t>
+        </is>
+      </c>
+      <c r="AK224" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="AL224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>16056</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>GANIREDDY AISHWARYA</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>6302459147</v>
+      </c>
+      <c r="D225" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E225" t="n">
+        <v>8650</v>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>22-Feb-2026 22:22:18</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L225" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N225" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O225" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P225" t="n">
+        <v>11000351226381</v>
+      </c>
+      <c r="Q225" t="n">
+        <v>1771778816</v>
+      </c>
+      <c r="R225" t="n">
+        <v>302542306467</v>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V225" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W225" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X225" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y225" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z225" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA225" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB225" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC225" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD225" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE225" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF225" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG225" t="inlineStr"/>
+      <c r="AH225" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI225" t="n">
+        <v>19023</v>
+      </c>
+      <c r="AJ225" t="inlineStr">
+        <is>
+          <t>266049</t>
+        </is>
+      </c>
+      <c r="AK225" t="inlineStr">
+        <is>
+          <t>2051</t>
+        </is>
+      </c>
+      <c r="AL225" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>16552</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>GANIREDDY ANUHYA</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>9848537189</v>
+      </c>
+      <c r="D226" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E226" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>22-Feb-2026 22:46:16</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>23-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L226" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N226" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O226" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P226" t="n">
+        <v>11000351228098</v>
+      </c>
+      <c r="Q226" t="n">
+        <v>1771779418</v>
+      </c>
+      <c r="R226" t="n">
+        <v>640262345476</v>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T226" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V226" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W226" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X226" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y226" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z226" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA226" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB226" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC226" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD226" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE226" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF226" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG226" t="inlineStr"/>
+      <c r="AH226" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI226" t="n">
+        <v>18375</v>
+      </c>
+      <c r="AJ226" t="inlineStr">
+        <is>
+          <t>267107</t>
+        </is>
+      </c>
+      <c r="AK226" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL226" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>16208</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>MYCHERLA SHASANK</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>7386344393</v>
+      </c>
+      <c r="D227" t="n">
+        <v>11350</v>
+      </c>
+      <c r="E227" t="n">
+        <v>11350</v>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>23-Feb-2026 11:09:23</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr"/>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L227" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N227" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O227" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P227" t="n">
+        <v>11000351269193</v>
+      </c>
+      <c r="Q227" t="n">
+        <v>1771825072</v>
+      </c>
+      <c r="R227" t="n">
+        <v>109246378284</v>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V227" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W227" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X227" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y227" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z227" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA227" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB227" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC227" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD227" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE227" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF227" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG227" t="inlineStr"/>
+      <c r="AH227" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI227" t="n">
+        <v>19412</v>
+      </c>
+      <c r="AJ227" t="inlineStr">
+        <is>
+          <t>268102</t>
+        </is>
+      </c>
+      <c r="AK227" t="inlineStr">
+        <is>
+          <t>2061</t>
+        </is>
+      </c>
+      <c r="AL227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>16906</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>RANVITHA SEERA</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>7095076706</v>
+      </c>
+      <c r="D228" t="n">
+        <v>10750</v>
+      </c>
+      <c r="E228" t="n">
+        <v>10750</v>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>23-Feb-2026 17:39:15</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr"/>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>ten thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L228" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N228" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O228" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P228" t="n">
+        <v>11000351328822</v>
+      </c>
+      <c r="Q228" t="n">
+        <v>1771848461</v>
+      </c>
+      <c r="R228" t="n">
+        <v>109248745854</v>
+      </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T228" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V228" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W228" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X228" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y228" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z228" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA228" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB228" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC228" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD228" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE228" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF228" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG228" t="inlineStr"/>
+      <c r="AH228" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI228" t="n">
+        <v>19168</v>
+      </c>
+      <c r="AJ228" t="inlineStr">
+        <is>
+          <t>268578</t>
+        </is>
+      </c>
+      <c r="AK228" t="inlineStr">
+        <is>
+          <t>2062</t>
+        </is>
+      </c>
+      <c r="AL228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>17099</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>VINDYA SOWDALA</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>7075489300</v>
+      </c>
+      <c r="D229" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E229" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>24-Feb-2026 17:26:28</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>25-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L229" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N229" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O229" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P229" t="n">
+        <v>11000351453145</v>
+      </c>
+      <c r="Q229" t="n">
+        <v>1771934170</v>
+      </c>
+      <c r="R229" t="n">
+        <v>929800159168</v>
+      </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T229" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V229" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W229" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X229" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y229" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z229" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA229" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB229" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC229" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD229" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE229" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF229" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG229" t="inlineStr"/>
+      <c r="AH229" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI229" t="n">
+        <v>18095</v>
+      </c>
+      <c r="AJ229" t="inlineStr">
+        <is>
+          <t>266761</t>
+        </is>
+      </c>
+      <c r="AK229" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL229" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>17100</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>BHAVIYSA SOWDALA</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>7075489300</v>
+      </c>
+      <c r="D230" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E230" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>24-Feb-2026 17:27:19</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>25-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L230" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N230" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O230" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P230" t="n">
+        <v>11000351454113</v>
+      </c>
+      <c r="Q230" t="n">
+        <v>1771934227</v>
+      </c>
+      <c r="R230" t="n">
+        <v>555789383766</v>
+      </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T230" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U230" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V230" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W230" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X230" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y230" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z230" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA230" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB230" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC230" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD230" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE230" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF230" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG230" t="inlineStr"/>
+      <c r="AH230" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI230" t="n">
+        <v>18638</v>
+      </c>
+      <c r="AJ230" t="inlineStr">
+        <is>
+          <t>267297</t>
+        </is>
+      </c>
+      <c r="AK230" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL230" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>17179</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>BORA LYDIA</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>6309196999</v>
+      </c>
+      <c r="D231" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E231" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>24-Feb-2026 22:50:26</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>25-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L231" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N231" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O231" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P231" t="n">
+        <v>11000351479569</v>
+      </c>
+      <c r="Q231" t="n">
+        <v>1771953532</v>
+      </c>
+      <c r="R231" t="n">
+        <v>145208162</v>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V231" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W231" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X231" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y231" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z231" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA231" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB231" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC231" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD231" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE231" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF231" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG231" t="inlineStr"/>
+      <c r="AH231" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI231" t="n">
+        <v>19894</v>
+      </c>
+      <c r="AJ231" t="inlineStr">
+        <is>
+          <t>266635</t>
+        </is>
+      </c>
+      <c r="AK231" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL231" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>16120</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>TANDU ROSARY ANTHONY</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>9492868687</v>
+      </c>
+      <c r="D232" t="n">
+        <v>25550</v>
+      </c>
+      <c r="E232" t="n">
+        <v>25550</v>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>25-Feb-2026 21:19:38</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>26-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>twenty five thousand five hundred fifty</t>
+        </is>
+      </c>
+      <c r="L232" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N232" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O232" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P232" t="n">
+        <v>11000351595092</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>1772034489</v>
+      </c>
+      <c r="R232" t="n">
+        <v>109262506265</v>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V232" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W232" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X232" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y232" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z232" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA232" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB232" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC232" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD232" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE232" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF232" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG232" t="inlineStr"/>
+      <c r="AH232" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI232" t="n">
+        <v>18727</v>
+      </c>
+      <c r="AJ232" t="inlineStr">
+        <is>
+          <t>261176,262330,264151,265801</t>
+        </is>
+      </c>
+      <c r="AK232" t="inlineStr">
+        <is>
+          <t>2033,2037,2042,2050</t>
+        </is>
+      </c>
+      <c r="AL232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>16977</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>OMMI NIDHISH NANDAN</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>8008110591</v>
+      </c>
+      <c r="D233" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E233" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>26-Feb-2026 16:35:02</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>27-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L233" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N233" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O233" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P233" t="n">
+        <v>11000351694708</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>1772103829</v>
+      </c>
+      <c r="R233" t="n">
+        <v>109267256087</v>
+      </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U233" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V233" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W233" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X233" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y233" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z233" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA233" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB233" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC233" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD233" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE233" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF233" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG233" t="inlineStr"/>
+      <c r="AH233" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI233" t="n">
+        <v>18105</v>
+      </c>
+      <c r="AJ233" t="inlineStr">
+        <is>
+          <t>266784</t>
+        </is>
+      </c>
+      <c r="AK233" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>17105</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>AADHVIK DADIRAO</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>7075570737</v>
+      </c>
+      <c r="D234" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E234" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>26-Feb-2026 20:59:33</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>27-Feb-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L234" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N234" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O234" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P234" t="n">
+        <v>11000351725842</v>
+      </c>
+      <c r="Q234" t="n">
+        <v>1772119422</v>
+      </c>
+      <c r="R234" t="n">
+        <v>109268695191</v>
+      </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U234" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V234" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W234" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X234" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y234" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z234" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA234" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB234" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC234" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD234" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE234" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF234" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG234" t="inlineStr"/>
+      <c r="AH234" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI234" t="n">
+        <v>18096</v>
+      </c>
+      <c r="AJ234" t="inlineStr">
+        <is>
+          <t>266773</t>
+        </is>
+      </c>
+      <c r="AK234" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>17219</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>VARTIKA KUMARI</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>8369239788</v>
+      </c>
+      <c r="D235" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E235" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>27-Feb-2026 19:37:49</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L235" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N235" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O235" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P235" t="n">
+        <v>11000351864684</v>
+      </c>
+      <c r="Q235" t="n">
+        <v>1772201239</v>
+      </c>
+      <c r="R235" t="n">
+        <v>605864009197</v>
+      </c>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T235" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U235" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V235" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W235" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X235" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y235" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z235" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA235" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB235" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC235" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD235" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE235" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF235" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG235" t="inlineStr"/>
+      <c r="AH235" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI235" t="n">
+        <v>19931</v>
+      </c>
+      <c r="AJ235" t="inlineStr">
+        <is>
+          <t>266855</t>
+        </is>
+      </c>
+      <c r="AK235" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="AL235" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>16797</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>YASHWANTH REDDY GUDLA</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>9948345552</v>
+      </c>
+      <c r="D236" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E236" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>28-Feb-2026 08:20:07</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L236" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N236" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O236" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P236" t="n">
+        <v>11000351909240</v>
+      </c>
+      <c r="Q236" t="n">
+        <v>1772246973</v>
+      </c>
+      <c r="R236" t="n">
+        <v>40471991429</v>
+      </c>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T236" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U236" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V236" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W236" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X236" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y236" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z236" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA236" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB236" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC236" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD236" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE236" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF236" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG236" t="inlineStr"/>
+      <c r="AH236" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI236" t="n">
+        <v>18786</v>
+      </c>
+      <c r="AJ236" t="inlineStr">
+        <is>
+          <t>267482</t>
+        </is>
+      </c>
+      <c r="AK236" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL236" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>16796</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>MAHENDRA REDDY GUDLA</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>9948345552</v>
+      </c>
+      <c r="D237" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E237" t="n">
+        <v>8650</v>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>28-Feb-2026 08:21:04</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr"/>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L237" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N237" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O237" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P237" t="n">
+        <v>11000351910047</v>
+      </c>
+      <c r="Q237" t="n">
+        <v>1772247054</v>
+      </c>
+      <c r="R237" t="n">
+        <v>146763616167</v>
+      </c>
+      <c r="S237" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T237" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U237" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V237" t="inlineStr">
+        <is>
+          <t>RNS</t>
+        </is>
+      </c>
+      <c r="W237" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X237" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y237" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z237" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA237" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB237" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC237" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD237" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE237" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF237" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG237" t="inlineStr"/>
+      <c r="AH237" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI237" t="n">
+        <v>19010</v>
+      </c>
+      <c r="AJ237" t="inlineStr">
+        <is>
+          <t>268450</t>
+        </is>
+      </c>
+      <c r="AK237" t="inlineStr">
+        <is>
+          <t>2059</t>
+        </is>
+      </c>
+      <c r="AL237" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>16020</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>DUVVU MAHALAKSHMI</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>9502247535</v>
+      </c>
+      <c r="D238" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E238" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>28-Feb-2026 10:28:45</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L238" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N238" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O238" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P238" t="n">
+        <v>11000351924775</v>
+      </c>
+      <c r="Q238" t="n">
+        <v>1772254681</v>
+      </c>
+      <c r="R238" t="n">
+        <v>920094640606</v>
+      </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V238" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W238" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X238" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y238" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z238" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA238" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB238" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC238" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD238" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE238" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF238" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG238" t="inlineStr"/>
+      <c r="AH238" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI238" t="n">
+        <v>18522</v>
+      </c>
+      <c r="AJ238" t="inlineStr">
+        <is>
+          <t>265602</t>
+        </is>
+      </c>
+      <c r="AK238" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="AL238" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>16036</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>DUVVU BHARGAVA SRI SAI</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>9502247535</v>
+      </c>
+      <c r="D239" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E239" t="n">
+        <v>8350</v>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>28-Feb-2026 10:27:22</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L239" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N239" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O239" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P239" t="n">
+        <v>11000351925096</v>
+      </c>
+      <c r="Q239" t="n">
+        <v>1772254577</v>
+      </c>
+      <c r="R239" t="n">
+        <v>866758700772</v>
+      </c>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V239" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W239" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X239" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y239" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z239" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA239" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB239" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC239" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD239" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE239" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF239" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG239" t="inlineStr"/>
+      <c r="AH239" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI239" t="n">
+        <v>18964</v>
+      </c>
+      <c r="AJ239" t="inlineStr">
+        <is>
+          <t>267620</t>
+        </is>
+      </c>
+      <c r="AK239" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL239" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>16020</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>DUVVU MAHALAKSHMI</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>9502247535</v>
+      </c>
+      <c r="D240" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E240" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>28-Feb-2026 10:38:10</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L240" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N240" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O240" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P240" t="n">
+        <v>11000351927021</v>
+      </c>
+      <c r="Q240" t="n">
+        <v>1772254751</v>
+      </c>
+      <c r="R240" t="n">
+        <v>469507160708</v>
+      </c>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U240" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V240" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W240" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X240" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y240" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z240" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA240" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB240" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC240" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD240" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE240" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF240" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG240" t="inlineStr"/>
+      <c r="AH240" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI240" t="n">
+        <v>18522</v>
+      </c>
+      <c r="AJ240" t="inlineStr">
+        <is>
+          <t>267252</t>
+        </is>
+      </c>
+      <c r="AK240" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL240" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>16914</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>SAI SRAVAN PATNAYAK</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>7337422112</v>
+      </c>
+      <c r="D241" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E241" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>28-Feb-2026 11:55:41</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L241" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N241" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O241" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P241" t="n">
+        <v>11000351942212</v>
+      </c>
+      <c r="Q241" t="n">
+        <v>1772259825</v>
+      </c>
+      <c r="R241" t="n">
+        <v>109278991926</v>
+      </c>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T241" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U241" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V241" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W241" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X241" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y241" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z241" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA241" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB241" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC241" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD241" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE241" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF241" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG241" t="inlineStr"/>
+      <c r="AH241" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI241" t="n">
+        <v>18066</v>
+      </c>
+      <c r="AJ241" t="inlineStr">
+        <is>
+          <t>266779</t>
+        </is>
+      </c>
+      <c r="AK241" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>15863</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>BOMMIDI BALA SURYA BHUVAN</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>6300875193</v>
+      </c>
+      <c r="D242" t="n">
+        <v>16100</v>
+      </c>
+      <c r="E242" t="n">
+        <v>16100</v>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>28-Feb-2026 12:55:32</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>sixteen thousand one hundred</t>
+        </is>
+      </c>
+      <c r="L242" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N242" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O242" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P242" t="n">
+        <v>11000351953158</v>
+      </c>
+      <c r="Q242" t="n">
+        <v>1772263454</v>
+      </c>
+      <c r="R242" t="n">
+        <v>109279356760</v>
+      </c>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T242" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U242" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V242" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W242" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X242" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y242" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z242" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA242" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB242" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC242" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD242" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE242" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF242" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG242" t="inlineStr"/>
+      <c r="AH242" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI242" t="n">
+        <v>18543</v>
+      </c>
+      <c r="AJ242" t="inlineStr">
+        <is>
+          <t>265653,267303</t>
+        </is>
+      </c>
+      <c r="AK242" t="inlineStr">
+        <is>
+          <t>2049,2057</t>
+        </is>
+      </c>
+      <c r="AL242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>17358</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>SAANVI SAHOO</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>8309736856</v>
+      </c>
+      <c r="D243" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E243" t="n">
+        <v>7750</v>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>01-Mar-2026 16:13:35</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 00:00:00</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L243" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N243" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O243" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P243" t="n">
+        <v>11000352070361</v>
+      </c>
+      <c r="Q243" t="n">
+        <v>1772361488</v>
+      </c>
+      <c r="R243" t="n">
+        <v>1.012026060690908e+17</v>
+      </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T243" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>BANK OF BARODA FSS</t>
+        </is>
+      </c>
+      <c r="V243" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W243" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X243" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y243" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="Z243" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA243" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB243" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC243" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD243" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE243" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF243" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG243" t="inlineStr"/>
+      <c r="AH243" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI243" t="n">
+        <v>20077</v>
+      </c>
+      <c r="AJ243" t="inlineStr">
+        <is>
+          <t>268295</t>
+        </is>
+      </c>
+      <c r="AK243" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="AL243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>16031</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>MALLA VAIBHAV SAI</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>9247311340</v>
+      </c>
+      <c r="D244" t="n">
+        <v>8350</v>
+      </c>
+      <c r="E244" t="inlineStr"/>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 08:34:02</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr"/>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="L244" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N244" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O244" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P244" t="n">
+        <v>11000352121038</v>
+      </c>
+      <c r="Q244" t="n">
+        <v>1772420420</v>
+      </c>
+      <c r="R244" t="n">
+        <v>606171974859</v>
+      </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T244" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U244" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V244" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W244" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X244" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y244" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z244" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA244" t="inlineStr"/>
+      <c r="AB244" t="inlineStr"/>
+      <c r="AC244" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD244" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE244" t="inlineStr"/>
+      <c r="AF244" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG244" t="inlineStr"/>
+      <c r="AH244" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI244" t="n">
+        <v>18978</v>
+      </c>
+      <c r="AJ244" t="inlineStr">
+        <is>
+          <t>267636</t>
+        </is>
+      </c>
+      <c r="AK244" t="inlineStr">
+        <is>
+          <t>2058</t>
+        </is>
+      </c>
+      <c r="AL244" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>17177</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>THUTTA HARI CHARANI</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>7337239208</v>
+      </c>
+      <c r="D245" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 09:34:10</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L245" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N245" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O245" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P245" t="n">
+        <v>11000352133780</v>
+      </c>
+      <c r="Q245" t="n">
+        <v>1772424238</v>
+      </c>
+      <c r="R245" t="n">
+        <v>805616523520</v>
+      </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T245" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U245" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V245" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W245" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X245" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y245" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z245" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA245" t="inlineStr"/>
+      <c r="AB245" t="inlineStr"/>
+      <c r="AC245" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD245" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE245" t="inlineStr"/>
+      <c r="AF245" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG245" t="inlineStr"/>
+      <c r="AH245" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI245" t="n">
+        <v>19892</v>
+      </c>
+      <c r="AJ245" t="inlineStr">
+        <is>
+          <t>266661</t>
+        </is>
+      </c>
+      <c r="AK245" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL245" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>16927</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>THUTTA DHANASHVI</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>7337239208</v>
+      </c>
+      <c r="D246" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E246" t="inlineStr"/>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 09:33:18</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr"/>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L246" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N246" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O246" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P246" t="n">
+        <v>11000352134464</v>
+      </c>
+      <c r="Q246" t="n">
+        <v>1772424160</v>
+      </c>
+      <c r="R246" t="n">
+        <v>778077483731</v>
+      </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T246" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U246" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V246" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W246" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X246" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y246" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z246" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA246" t="inlineStr"/>
+      <c r="AB246" t="inlineStr"/>
+      <c r="AC246" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD246" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE246" t="inlineStr"/>
+      <c r="AF246" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG246" t="inlineStr"/>
+      <c r="AH246" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI246" t="n">
+        <v>18339</v>
+      </c>
+      <c r="AJ246" t="inlineStr">
+        <is>
+          <t>266997</t>
+        </is>
+      </c>
+      <c r="AK246" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="AL246" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>16974</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>KADAJARI ESHAN ESWAR</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>9885130099</v>
+      </c>
+      <c r="D247" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 11:31:24</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr"/>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L247" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N247" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O247" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P247" t="n">
+        <v>11000352162203</v>
+      </c>
+      <c r="Q247" t="n">
+        <v>1772431154</v>
+      </c>
+      <c r="R247" t="n">
+        <v>606128095174</v>
+      </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V247" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W247" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X247" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y247" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z247" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA247" t="inlineStr"/>
+      <c r="AB247" t="inlineStr"/>
+      <c r="AC247" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD247" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE247" t="inlineStr"/>
+      <c r="AF247" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG247" t="inlineStr"/>
+      <c r="AH247" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI247" t="n">
+        <v>18273</v>
+      </c>
+      <c r="AJ247" t="inlineStr">
+        <is>
+          <t>267040</t>
+        </is>
+      </c>
+      <c r="AK247" t="inlineStr">
+        <is>
+          <t>2056</t>
+        </is>
+      </c>
+      <c r="AL247" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>17147</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>RONGALI YERNI VENKATA RAKESH</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>7793910192</v>
+      </c>
+      <c r="D248" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E248" t="inlineStr"/>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 12:16:58</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr"/>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="L248" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N248" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O248" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P248" t="n">
+        <v>11000352171807</v>
+      </c>
+      <c r="Q248" t="n">
+        <v>1772433952</v>
+      </c>
+      <c r="R248" t="n">
+        <v>398196116938</v>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T248" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V248" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W248" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X248" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y248" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z248" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA248" t="inlineStr"/>
+      <c r="AB248" t="inlineStr"/>
+      <c r="AC248" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD248" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE248" t="inlineStr"/>
+      <c r="AF248" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG248" t="inlineStr"/>
+      <c r="AH248" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI248" t="n">
+        <v>19850</v>
+      </c>
+      <c r="AJ248" t="inlineStr">
+        <is>
+          <t>267206</t>
+        </is>
+      </c>
+      <c r="AK248" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL248" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>17146</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>RONGALI JASMIKA</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>7793910192</v>
+      </c>
+      <c r="D249" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 12:12:45</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr"/>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L249" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N249" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O249" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P249" t="n">
+        <v>11000352172149</v>
+      </c>
+      <c r="Q249" t="n">
+        <v>1772433686</v>
+      </c>
+      <c r="R249" t="n">
+        <v>201120935621</v>
+      </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U249" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V249" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W249" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X249" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y249" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z249" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA249" t="inlineStr"/>
+      <c r="AB249" t="inlineStr"/>
+      <c r="AC249" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD249" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE249" t="inlineStr"/>
+      <c r="AF249" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG249" t="inlineStr"/>
+      <c r="AH249" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI249" t="n">
+        <v>19849</v>
+      </c>
+      <c r="AJ249" t="inlineStr">
+        <is>
+          <t>266747</t>
+        </is>
+      </c>
+      <c r="AK249" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL249" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>16375</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>AYESHA NAIK</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>9346210583</v>
+      </c>
+      <c r="D250" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E250" t="inlineStr"/>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>02-Mar-2026 12:59:37</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr"/>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>eight thousand six hundred fifty</t>
+        </is>
+      </c>
+      <c r="L250" t="n">
+        <v>100000036600</v>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N250" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O250" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P250" t="n">
+        <v>11000352181791</v>
+      </c>
+      <c r="Q250" t="n">
+        <v>1772436554</v>
+      </c>
+      <c r="R250" t="n">
+        <v>102107278836</v>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V250" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W250" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X250" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y250" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z250" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA250" t="inlineStr"/>
+      <c r="AB250" t="inlineStr"/>
+      <c r="AC250" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD250" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE250" t="inlineStr"/>
+      <c r="AF250" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG250" t="inlineStr"/>
+      <c r="AH250" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI250" t="n">
+        <v>19024</v>
+      </c>
+      <c r="AJ250" t="inlineStr">
+        <is>
+          <t>268411</t>
+        </is>
+      </c>
+      <c r="AK250" t="inlineStr">
+        <is>
+          <t>2059</t>
+        </is>
+      </c>
+      <c r="AL250" t="inlineStr">
         <is>
           <t>UPI INTENT</t>
         </is>

</xml_diff>

<commit_message>
Normalize student names and class codes
Standardize fee-reporting data across output and source files: cleaned StudentName formatting and normalized class/section codes in daywise_fees_collection (and year-specific/online variants), updated atom_report_cleaned.xlsx and atom_report.xlsx, refreshed fees and concession reports and merged_fee_collection, updated Power BI dashboard and notebook, and renamed a postgres backup file. These changes ensure consistent formatting for reporting and dashboarding.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL298"/>
+  <dimension ref="A1:AL299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32934,8 +32934,16 @@
       <c r="A235" t="n">
         <v>17219</v>
       </c>
-      <c r="B235" t="inlineStr"/>
-      <c r="C235" t="inlineStr"/>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>V****** K*****</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>83****9788</t>
+        </is>
+      </c>
       <c r="D235" t="n">
         <v>7750</v>
       </c>
@@ -32970,7 +32978,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L235" t="inlineStr"/>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M235" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -33026,7 +33038,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z235" t="inlineStr"/>
+      <c r="Z235" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA235" t="n">
         <v>5</v>
       </c>
@@ -33076,8 +33092,16 @@
       <c r="A236" t="n">
         <v>16797</v>
       </c>
-      <c r="B236" t="inlineStr"/>
-      <c r="C236" t="inlineStr"/>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Y******** R**** G****</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>99****5552</t>
+        </is>
+      </c>
       <c r="D236" t="n">
         <v>8350</v>
       </c>
@@ -33112,7 +33136,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L236" t="inlineStr"/>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M236" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -33168,7 +33196,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z236" t="inlineStr"/>
+      <c r="Z236" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA236" t="n">
         <v>5</v>
       </c>
@@ -33218,8 +33250,16 @@
       <c r="A237" t="n">
         <v>16796</v>
       </c>
-      <c r="B237" t="inlineStr"/>
-      <c r="C237" t="inlineStr"/>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>M******* R**** G****</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>99****5552</t>
+        </is>
+      </c>
       <c r="D237" t="n">
         <v>8650</v>
       </c>
@@ -33250,7 +33290,11 @@
           <t>eight thousand six hundred fifty</t>
         </is>
       </c>
-      <c r="L237" t="inlineStr"/>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M237" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -33306,7 +33350,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z237" t="inlineStr"/>
+      <c r="Z237" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA237" t="n">
         <v>5</v>
       </c>
@@ -33356,8 +33404,16 @@
       <c r="A238" t="n">
         <v>16020</v>
       </c>
-      <c r="B238" t="inlineStr"/>
-      <c r="C238" t="inlineStr"/>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>D**** M**********</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>95****7535</t>
+        </is>
+      </c>
       <c r="D238" t="n">
         <v>8050</v>
       </c>
@@ -33392,7 +33448,11 @@
           <t>eight thousand fifty</t>
         </is>
       </c>
-      <c r="L238" t="inlineStr"/>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M238" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -33448,7 +33508,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z238" t="inlineStr"/>
+      <c r="Z238" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA238" t="n">
         <v>5</v>
       </c>
@@ -33498,8 +33562,16 @@
       <c r="A239" t="n">
         <v>16036</v>
       </c>
-      <c r="B239" t="inlineStr"/>
-      <c r="C239" t="inlineStr"/>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>D**** B******* S** S**</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>95****7535</t>
+        </is>
+      </c>
       <c r="D239" t="n">
         <v>8350</v>
       </c>
@@ -33534,7 +33606,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L239" t="inlineStr"/>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M239" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -33590,7 +33666,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z239" t="inlineStr"/>
+      <c r="Z239" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA239" t="n">
         <v>5</v>
       </c>
@@ -33640,8 +33720,16 @@
       <c r="A240" t="n">
         <v>16020</v>
       </c>
-      <c r="B240" t="inlineStr"/>
-      <c r="C240" t="inlineStr"/>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>D**** M**********</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>95****7535</t>
+        </is>
+      </c>
       <c r="D240" t="n">
         <v>8050</v>
       </c>
@@ -33676,7 +33764,11 @@
           <t>eight thousand fifty</t>
         </is>
       </c>
-      <c r="L240" t="inlineStr"/>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M240" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -33732,7 +33824,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z240" t="inlineStr"/>
+      <c r="Z240" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA240" t="n">
         <v>5</v>
       </c>
@@ -33782,8 +33878,16 @@
       <c r="A241" t="n">
         <v>16914</v>
       </c>
-      <c r="B241" t="inlineStr"/>
-      <c r="C241" t="inlineStr"/>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>S** S***** P*******</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>73****2112</t>
+        </is>
+      </c>
       <c r="D241" t="n">
         <v>6750</v>
       </c>
@@ -33818,7 +33922,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L241" t="inlineStr"/>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M241" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -33874,7 +33982,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z241" t="inlineStr"/>
+      <c r="Z241" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA241" t="n">
         <v>5</v>
       </c>
@@ -33920,8 +34032,16 @@
       <c r="A242" t="n">
         <v>15863</v>
       </c>
-      <c r="B242" t="inlineStr"/>
-      <c r="C242" t="inlineStr"/>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>B****** B*** S**** B*****</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>63****5193</t>
+        </is>
+      </c>
       <c r="D242" t="n">
         <v>16100</v>
       </c>
@@ -33956,7 +34076,11 @@
           <t>sixteen thousand one hundred</t>
         </is>
       </c>
-      <c r="L242" t="inlineStr"/>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M242" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -34012,7 +34136,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z242" t="inlineStr"/>
+      <c r="Z242" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA242" t="n">
         <v>5</v>
       </c>
@@ -34058,8 +34186,16 @@
       <c r="A243" t="n">
         <v>17358</v>
       </c>
-      <c r="B243" t="inlineStr"/>
-      <c r="C243" t="inlineStr"/>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>S***** S****</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>83****6856</t>
+        </is>
+      </c>
       <c r="D243" t="n">
         <v>7750</v>
       </c>
@@ -34094,7 +34230,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L243" t="inlineStr"/>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M243" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -34150,7 +34290,11 @@
           <t>DC</t>
         </is>
       </c>
-      <c r="Z243" t="inlineStr"/>
+      <c r="Z243" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA243" t="n">
         <v>5</v>
       </c>
@@ -34196,8 +34340,16 @@
       <c r="A244" t="n">
         <v>16031</v>
       </c>
-      <c r="B244" t="inlineStr"/>
-      <c r="C244" t="inlineStr"/>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>M**** V****** S**</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>92****1340</t>
+        </is>
+      </c>
       <c r="D244" t="n">
         <v>8350</v>
       </c>
@@ -34232,7 +34384,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L244" t="inlineStr"/>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M244" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -34288,7 +34444,11 @@
           <t>QR_UPI</t>
         </is>
       </c>
-      <c r="Z244" t="inlineStr"/>
+      <c r="Z244" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA244" t="n">
         <v>5</v>
       </c>
@@ -34338,8 +34498,16 @@
       <c r="A245" t="n">
         <v>17177</v>
       </c>
-      <c r="B245" t="inlineStr"/>
-      <c r="C245" t="inlineStr"/>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>T***** H*** C******</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>73****9208</t>
+        </is>
+      </c>
       <c r="D245" t="n">
         <v>6750</v>
       </c>
@@ -34374,7 +34542,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L245" t="inlineStr"/>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M245" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -34430,7 +34602,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z245" t="inlineStr"/>
+      <c r="Z245" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA245" t="n">
         <v>5</v>
       </c>
@@ -34480,8 +34656,16 @@
       <c r="A246" t="n">
         <v>16927</v>
       </c>
-      <c r="B246" t="inlineStr"/>
-      <c r="C246" t="inlineStr"/>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>T***** D********</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>73****9208</t>
+        </is>
+      </c>
       <c r="D246" t="n">
         <v>7750</v>
       </c>
@@ -34516,7 +34700,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L246" t="inlineStr"/>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M246" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -34572,7 +34760,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z246" t="inlineStr"/>
+      <c r="Z246" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA246" t="n">
         <v>5</v>
       </c>
@@ -34622,8 +34814,16 @@
       <c r="A247" t="n">
         <v>16974</v>
       </c>
-      <c r="B247" t="inlineStr"/>
-      <c r="C247" t="inlineStr"/>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>K******* E**** E****</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>98****0099</t>
+        </is>
+      </c>
       <c r="D247" t="n">
         <v>7750</v>
       </c>
@@ -34658,7 +34858,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L247" t="inlineStr"/>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M247" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -34714,7 +34918,11 @@
           <t>QR_UPI</t>
         </is>
       </c>
-      <c r="Z247" t="inlineStr"/>
+      <c r="Z247" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA247" t="n">
         <v>5</v>
       </c>
@@ -34764,8 +34972,16 @@
       <c r="A248" t="n">
         <v>17147</v>
       </c>
-      <c r="B248" t="inlineStr"/>
-      <c r="C248" t="inlineStr"/>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>R****** Y**** V****** R*****</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>77****0192</t>
+        </is>
+      </c>
       <c r="D248" t="n">
         <v>8050</v>
       </c>
@@ -34800,7 +35016,11 @@
           <t>eight thousand fifty</t>
         </is>
       </c>
-      <c r="L248" t="inlineStr"/>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M248" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -34856,7 +35076,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z248" t="inlineStr"/>
+      <c r="Z248" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA248" t="n">
         <v>5</v>
       </c>
@@ -34906,8 +35130,16 @@
       <c r="A249" t="n">
         <v>17146</v>
       </c>
-      <c r="B249" t="inlineStr"/>
-      <c r="C249" t="inlineStr"/>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>R****** J******</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>77****0192</t>
+        </is>
+      </c>
       <c r="D249" t="n">
         <v>6750</v>
       </c>
@@ -34942,7 +35174,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L249" t="inlineStr"/>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M249" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -34998,7 +35234,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z249" t="inlineStr"/>
+      <c r="Z249" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA249" t="n">
         <v>5</v>
       </c>
@@ -35048,8 +35288,16 @@
       <c r="A250" t="n">
         <v>16375</v>
       </c>
-      <c r="B250" t="inlineStr"/>
-      <c r="C250" t="inlineStr"/>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>A***** N***</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>93****0583</t>
+        </is>
+      </c>
       <c r="D250" t="n">
         <v>8650</v>
       </c>
@@ -35080,7 +35328,11 @@
           <t>eight thousand six hundred fifty</t>
         </is>
       </c>
-      <c r="L250" t="inlineStr"/>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M250" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -35136,7 +35388,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z250" t="inlineStr"/>
+      <c r="Z250" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA250" t="n">
         <v>5</v>
       </c>
@@ -35186,8 +35442,16 @@
       <c r="A251" t="n">
         <v>16580</v>
       </c>
-      <c r="B251" t="inlineStr"/>
-      <c r="C251" t="inlineStr"/>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>C******* A************* M*********</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>99****6244</t>
+        </is>
+      </c>
       <c r="D251" t="n">
         <v>8350</v>
       </c>
@@ -35222,7 +35486,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L251" t="inlineStr"/>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M251" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -35278,7 +35546,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z251" t="inlineStr"/>
+      <c r="Z251" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA251" t="n">
         <v>5</v>
       </c>
@@ -35328,8 +35600,16 @@
       <c r="A252" t="n">
         <v>16580</v>
       </c>
-      <c r="B252" t="inlineStr"/>
-      <c r="C252" t="inlineStr"/>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>C******* A************* M*********</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>99****6244</t>
+        </is>
+      </c>
       <c r="D252" t="n">
         <v>8350</v>
       </c>
@@ -35364,7 +35644,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L252" t="inlineStr"/>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M252" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -35420,7 +35704,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z252" t="inlineStr"/>
+      <c r="Z252" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA252" t="n">
         <v>5</v>
       </c>
@@ -35470,8 +35758,16 @@
       <c r="A253" t="n">
         <v>16740</v>
       </c>
-      <c r="B253" t="inlineStr"/>
-      <c r="C253" t="inlineStr"/>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>S**** Y****</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>81****6234</t>
+        </is>
+      </c>
       <c r="D253" t="n">
         <v>7750</v>
       </c>
@@ -35506,7 +35802,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L253" t="inlineStr"/>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M253" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -35562,7 +35862,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z253" t="inlineStr"/>
+      <c r="Z253" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA253" t="n">
         <v>5</v>
       </c>
@@ -35612,8 +35916,16 @@
       <c r="A254" t="n">
         <v>16936</v>
       </c>
-      <c r="B254" t="inlineStr"/>
-      <c r="C254" t="inlineStr"/>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>H******** R*****</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>63****8581</t>
+        </is>
+      </c>
       <c r="D254" t="n">
         <v>7750</v>
       </c>
@@ -35648,7 +35960,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L254" t="inlineStr"/>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M254" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -35704,7 +36020,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z254" t="inlineStr"/>
+      <c r="Z254" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA254" t="n">
         <v>5</v>
       </c>
@@ -35754,8 +36074,16 @@
       <c r="A255" t="n">
         <v>15041</v>
       </c>
-      <c r="B255" t="inlineStr"/>
-      <c r="C255" t="inlineStr"/>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>B**** A****** S***</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>90****9626</t>
+        </is>
+      </c>
       <c r="D255" t="n">
         <v>10750</v>
       </c>
@@ -35786,7 +36114,11 @@
           <t>ten thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L255" t="inlineStr"/>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M255" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -35842,7 +36174,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z255" t="inlineStr"/>
+      <c r="Z255" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA255" t="n">
         <v>5</v>
       </c>
@@ -35892,8 +36228,16 @@
       <c r="A256" t="n">
         <v>16721</v>
       </c>
-      <c r="B256" t="inlineStr"/>
-      <c r="C256" t="inlineStr"/>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>K****** G**********</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>99****1635</t>
+        </is>
+      </c>
       <c r="D256" t="n">
         <v>7750</v>
       </c>
@@ -35928,7 +36272,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L256" t="inlineStr"/>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M256" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -35984,7 +36332,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z256" t="inlineStr"/>
+      <c r="Z256" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA256" t="n">
         <v>5</v>
       </c>
@@ -36034,8 +36386,16 @@
       <c r="A257" t="n">
         <v>15823</v>
       </c>
-      <c r="B257" t="inlineStr"/>
-      <c r="C257" t="inlineStr"/>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>K****** H*****</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>99****1635</t>
+        </is>
+      </c>
       <c r="D257" t="n">
         <v>8350</v>
       </c>
@@ -36070,7 +36430,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L257" t="inlineStr"/>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M257" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -36126,7 +36490,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z257" t="inlineStr"/>
+      <c r="Z257" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA257" t="n">
         <v>5</v>
       </c>
@@ -36176,8 +36544,16 @@
       <c r="A258" t="n">
         <v>15536</v>
       </c>
-      <c r="B258" t="inlineStr"/>
-      <c r="C258" t="inlineStr"/>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>K**** M*********</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>97****1309</t>
+        </is>
+      </c>
       <c r="D258" t="n">
         <v>8350</v>
       </c>
@@ -36212,7 +36588,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L258" t="inlineStr"/>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M258" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -36268,7 +36648,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z258" t="inlineStr"/>
+      <c r="Z258" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA258" t="n">
         <v>5</v>
       </c>
@@ -36318,8 +36702,16 @@
       <c r="A259" t="n">
         <v>15541</v>
       </c>
-      <c r="B259" t="inlineStr"/>
-      <c r="C259" t="inlineStr"/>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>R****** V***********</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>98****9449</t>
+        </is>
+      </c>
       <c r="D259" t="n">
         <v>8350</v>
       </c>
@@ -36354,7 +36746,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L259" t="inlineStr"/>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M259" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -36410,7 +36806,11 @@
           <t>QR_UPI</t>
         </is>
       </c>
-      <c r="Z259" t="inlineStr"/>
+      <c r="Z259" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA259" t="n">
         <v>5</v>
       </c>
@@ -36460,8 +36860,16 @@
       <c r="A260" t="n">
         <v>17163</v>
       </c>
-      <c r="B260" t="inlineStr"/>
-      <c r="C260" t="inlineStr"/>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>M******* Z*** K***</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>82****8795</t>
+        </is>
+      </c>
       <c r="D260" t="n">
         <v>6750</v>
       </c>
@@ -36496,7 +36904,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L260" t="inlineStr"/>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M260" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -36552,7 +36964,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z260" t="inlineStr"/>
+      <c r="Z260" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA260" t="n">
         <v>5</v>
       </c>
@@ -36602,8 +37018,16 @@
       <c r="A261" t="n">
         <v>15746</v>
       </c>
-      <c r="B261" t="inlineStr"/>
-      <c r="C261" t="inlineStr"/>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Y**** Y******* N****</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>94****1196</t>
+        </is>
+      </c>
       <c r="D261" t="n">
         <v>16700</v>
       </c>
@@ -36638,7 +37062,11 @@
           <t>sixteen thousand seven hundred</t>
         </is>
       </c>
-      <c r="L261" t="inlineStr"/>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M261" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -36694,7 +37122,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z261" t="inlineStr"/>
+      <c r="Z261" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA261" t="n">
         <v>5</v>
       </c>
@@ -36744,8 +37176,16 @@
       <c r="A262" t="n">
         <v>14949</v>
       </c>
-      <c r="B262" t="inlineStr"/>
-      <c r="C262" t="inlineStr"/>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>M***** S******* L****** S** M** R**</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>80****0739</t>
+        </is>
+      </c>
       <c r="D262" t="n">
         <v>10750</v>
       </c>
@@ -36776,7 +37216,11 @@
           <t>ten thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L262" t="inlineStr"/>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M262" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -36832,7 +37276,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z262" t="inlineStr"/>
+      <c r="Z262" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA262" t="n">
         <v>5</v>
       </c>
@@ -36882,8 +37330,16 @@
       <c r="A263" t="n">
         <v>16894</v>
       </c>
-      <c r="B263" t="inlineStr"/>
-      <c r="C263" t="inlineStr"/>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>S**** V****** S** V***** V******</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>85****3683</t>
+        </is>
+      </c>
       <c r="D263" t="n">
         <v>8650</v>
       </c>
@@ -36914,7 +37370,11 @@
           <t>eight thousand six hundred fifty</t>
         </is>
       </c>
-      <c r="L263" t="inlineStr"/>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M263" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -36970,7 +37430,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z263" t="inlineStr"/>
+      <c r="Z263" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA263" t="n">
         <v>5</v>
       </c>
@@ -37020,8 +37484,16 @@
       <c r="A264" t="n">
         <v>17103</v>
       </c>
-      <c r="B264" t="inlineStr"/>
-      <c r="C264" t="inlineStr"/>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>P******** B******* S**</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>63****9629</t>
+        </is>
+      </c>
       <c r="D264" t="n">
         <v>6750</v>
       </c>
@@ -37056,7 +37528,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L264" t="inlineStr"/>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M264" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -37112,7 +37588,11 @@
           <t>QR_UPI</t>
         </is>
       </c>
-      <c r="Z264" t="inlineStr"/>
+      <c r="Z264" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA264" t="n">
         <v>5</v>
       </c>
@@ -37162,8 +37642,16 @@
       <c r="A265" t="n">
         <v>17093</v>
       </c>
-      <c r="B265" t="inlineStr"/>
-      <c r="C265" t="inlineStr"/>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>S**** A******</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>98****7290</t>
+        </is>
+      </c>
       <c r="D265" t="n">
         <v>6750</v>
       </c>
@@ -37198,7 +37686,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L265" t="inlineStr"/>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M265" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -37254,7 +37746,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z265" t="inlineStr"/>
+      <c r="Z265" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA265" t="n">
         <v>5</v>
       </c>
@@ -37304,8 +37800,16 @@
       <c r="A266" t="n">
         <v>16167</v>
       </c>
-      <c r="B266" t="inlineStr"/>
-      <c r="C266" t="inlineStr"/>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>V******* L********</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>88****9151</t>
+        </is>
+      </c>
       <c r="D266" t="n">
         <v>8350</v>
       </c>
@@ -37340,7 +37844,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L266" t="inlineStr"/>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M266" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -37396,7 +37904,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z266" t="inlineStr"/>
+      <c r="Z266" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA266" t="n">
         <v>5</v>
       </c>
@@ -37446,8 +37958,16 @@
       <c r="A267" t="n">
         <v>16353</v>
       </c>
-      <c r="B267" t="inlineStr"/>
-      <c r="C267" t="inlineStr"/>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>R***** H********* V*****</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>93****3084</t>
+        </is>
+      </c>
       <c r="D267" t="n">
         <v>8050</v>
       </c>
@@ -37482,7 +38002,11 @@
           <t>eight thousand fifty</t>
         </is>
       </c>
-      <c r="L267" t="inlineStr"/>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M267" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -37538,7 +38062,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z267" t="inlineStr"/>
+      <c r="Z267" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA267" t="n">
         <v>5</v>
       </c>
@@ -37588,8 +38116,16 @@
       <c r="A268" t="n">
         <v>17277</v>
       </c>
-      <c r="B268" t="inlineStr"/>
-      <c r="C268" t="inlineStr"/>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>E******* M*******</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>96****1662</t>
+        </is>
+      </c>
       <c r="D268" t="n">
         <v>6750</v>
       </c>
@@ -37624,7 +38160,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L268" t="inlineStr"/>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M268" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -37680,7 +38220,11 @@
           <t>QR_UPI</t>
         </is>
       </c>
-      <c r="Z268" t="inlineStr"/>
+      <c r="Z268" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA268" t="n">
         <v>5</v>
       </c>
@@ -37730,8 +38274,16 @@
       <c r="A269" t="n">
         <v>17138</v>
       </c>
-      <c r="B269" t="inlineStr"/>
-      <c r="C269" t="inlineStr"/>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>S**** B******</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>79****8688</t>
+        </is>
+      </c>
       <c r="D269" t="n">
         <v>7750</v>
       </c>
@@ -37766,7 +38318,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L269" t="inlineStr"/>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M269" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -37822,7 +38378,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z269" t="inlineStr"/>
+      <c r="Z269" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA269" t="n">
         <v>5</v>
       </c>
@@ -37872,8 +38432,16 @@
       <c r="A270" t="n">
         <v>17139</v>
       </c>
-      <c r="B270" t="inlineStr"/>
-      <c r="C270" t="inlineStr"/>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>S**** B********* S**</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>79****8688</t>
+        </is>
+      </c>
       <c r="D270" t="n">
         <v>8350</v>
       </c>
@@ -37908,7 +38476,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L270" t="inlineStr"/>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M270" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -37964,7 +38536,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z270" t="inlineStr"/>
+      <c r="Z270" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA270" t="n">
         <v>5</v>
       </c>
@@ -38014,8 +38590,16 @@
       <c r="A271" t="n">
         <v>16043</v>
       </c>
-      <c r="B271" t="inlineStr"/>
-      <c r="C271" t="inlineStr"/>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>V****** V******* M****</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>76****5088</t>
+        </is>
+      </c>
       <c r="D271" t="n">
         <v>8050</v>
       </c>
@@ -38050,7 +38634,11 @@
           <t>eight thousand fifty</t>
         </is>
       </c>
-      <c r="L271" t="inlineStr"/>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M271" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -38106,7 +38694,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z271" t="inlineStr"/>
+      <c r="Z271" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA271" t="n">
         <v>5</v>
       </c>
@@ -38156,8 +38748,16 @@
       <c r="A272" t="n">
         <v>16548</v>
       </c>
-      <c r="B272" t="inlineStr"/>
-      <c r="C272" t="inlineStr"/>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>P******* C****** R******</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>90****9830</t>
+        </is>
+      </c>
       <c r="D272" t="n">
         <v>8350</v>
       </c>
@@ -38192,7 +38792,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L272" t="inlineStr"/>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M272" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -38248,7 +38852,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z272" t="inlineStr"/>
+      <c r="Z272" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA272" t="n">
         <v>5</v>
       </c>
@@ -38298,8 +38906,16 @@
       <c r="A273" t="n">
         <v>16761</v>
       </c>
-      <c r="B273" t="inlineStr"/>
-      <c r="C273" t="inlineStr"/>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>T**** T*** K****</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>97****8884</t>
+        </is>
+      </c>
       <c r="D273" t="n">
         <v>8650</v>
       </c>
@@ -38330,7 +38946,11 @@
           <t>eight thousand six hundred fifty</t>
         </is>
       </c>
-      <c r="L273" t="inlineStr"/>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M273" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -38386,7 +39006,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z273" t="inlineStr"/>
+      <c r="Z273" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA273" t="n">
         <v>5</v>
       </c>
@@ -38436,8 +39060,16 @@
       <c r="A274" t="n">
         <v>17305</v>
       </c>
-      <c r="B274" t="inlineStr"/>
-      <c r="C274" t="inlineStr"/>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>T******* D** C******</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>90****6332</t>
+        </is>
+      </c>
       <c r="D274" t="n">
         <v>6750</v>
       </c>
@@ -38472,7 +39104,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L274" t="inlineStr"/>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M274" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -38528,7 +39164,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z274" t="inlineStr"/>
+      <c r="Z274" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA274" t="n">
         <v>5</v>
       </c>
@@ -38578,8 +39218,16 @@
       <c r="A275" t="n">
         <v>16492</v>
       </c>
-      <c r="B275" t="inlineStr"/>
-      <c r="C275" t="inlineStr"/>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>A****** A****** M*********</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>99****6244</t>
+        </is>
+      </c>
       <c r="D275" t="n">
         <v>8050</v>
       </c>
@@ -38614,7 +39262,11 @@
           <t>eight thousand fifty</t>
         </is>
       </c>
-      <c r="L275" t="inlineStr"/>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M275" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -38670,7 +39322,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z275" t="inlineStr"/>
+      <c r="Z275" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA275" t="n">
         <v>5</v>
       </c>
@@ -38720,8 +39376,16 @@
       <c r="A276" t="n">
         <v>16492</v>
       </c>
-      <c r="B276" t="inlineStr"/>
-      <c r="C276" t="inlineStr"/>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>A****** A****** M*********</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>99****6244</t>
+        </is>
+      </c>
       <c r="D276" t="n">
         <v>8050</v>
       </c>
@@ -38756,7 +39420,11 @@
           <t>eight thousand fifty</t>
         </is>
       </c>
-      <c r="L276" t="inlineStr"/>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M276" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -38812,7 +39480,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z276" t="inlineStr"/>
+      <c r="Z276" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA276" t="n">
         <v>5</v>
       </c>
@@ -38862,8 +39534,16 @@
       <c r="A277" t="n">
         <v>16966</v>
       </c>
-      <c r="B277" t="inlineStr"/>
-      <c r="C277" t="inlineStr"/>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>G******* J***** A***** A******</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>82****6967</t>
+        </is>
+      </c>
       <c r="D277" t="n">
         <v>6750</v>
       </c>
@@ -38898,7 +39578,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L277" t="inlineStr"/>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M277" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -38954,7 +39638,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z277" t="inlineStr"/>
+      <c r="Z277" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA277" t="n">
         <v>5</v>
       </c>
@@ -39004,8 +39692,16 @@
       <c r="A278" t="n">
         <v>16211</v>
       </c>
-      <c r="B278" t="inlineStr"/>
-      <c r="C278" t="inlineStr"/>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>P******* J*******</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>95****0840</t>
+        </is>
+      </c>
       <c r="D278" t="n">
         <v>8350</v>
       </c>
@@ -39040,7 +39736,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L278" t="inlineStr"/>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M278" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -39096,7 +39796,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z278" t="inlineStr"/>
+      <c r="Z278" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA278" t="n">
         <v>5</v>
       </c>
@@ -39146,8 +39850,16 @@
       <c r="A279" t="n">
         <v>15234</v>
       </c>
-      <c r="B279" t="inlineStr"/>
-      <c r="C279" t="inlineStr"/>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>M****** P*****</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>99****3424</t>
+        </is>
+      </c>
       <c r="D279" t="n">
         <v>8650</v>
       </c>
@@ -39178,7 +39890,11 @@
           <t>eight thousand six hundred fifty</t>
         </is>
       </c>
-      <c r="L279" t="inlineStr"/>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M279" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -39234,7 +39950,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z279" t="inlineStr"/>
+      <c r="Z279" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA279" t="n">
         <v>5</v>
       </c>
@@ -39284,8 +40004,16 @@
       <c r="A280" t="n">
         <v>16710</v>
       </c>
-      <c r="B280" t="inlineStr"/>
-      <c r="C280" t="inlineStr"/>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>B********** H*********</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>98****7129</t>
+        </is>
+      </c>
       <c r="D280" t="n">
         <v>7750</v>
       </c>
@@ -39320,7 +40048,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L280" t="inlineStr"/>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M280" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -39376,7 +40108,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z280" t="inlineStr"/>
+      <c r="Z280" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA280" t="n">
         <v>5</v>
       </c>
@@ -39426,8 +40162,16 @@
       <c r="A281" t="n">
         <v>15544</v>
       </c>
-      <c r="B281" t="inlineStr"/>
-      <c r="C281" t="inlineStr"/>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>B********** J** A******** S**** S*****</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>98****7129</t>
+        </is>
+      </c>
       <c r="D281" t="n">
         <v>8350</v>
       </c>
@@ -39462,7 +40206,11 @@
           <t>eight thousand three hundred fifty</t>
         </is>
       </c>
-      <c r="L281" t="inlineStr"/>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M281" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -39518,7 +40266,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z281" t="inlineStr"/>
+      <c r="Z281" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA281" t="n">
         <v>5</v>
       </c>
@@ -39568,8 +40320,16 @@
       <c r="A282" t="n">
         <v>15009</v>
       </c>
-      <c r="B282" t="inlineStr"/>
-      <c r="C282" t="inlineStr"/>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>G******* G**********</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>93****3464</t>
+        </is>
+      </c>
       <c r="D282" t="n">
         <v>8650</v>
       </c>
@@ -39600,7 +40360,11 @@
           <t>eight thousand six hundred fifty</t>
         </is>
       </c>
-      <c r="L282" t="inlineStr"/>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M282" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -39656,7 +40420,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z282" t="inlineStr"/>
+      <c r="Z282" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA282" t="n">
         <v>5</v>
       </c>
@@ -39706,8 +40474,16 @@
       <c r="A283" t="n">
         <v>15824</v>
       </c>
-      <c r="B283" t="inlineStr"/>
-      <c r="C283" t="inlineStr"/>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>G******* R***** N******</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>93****3464</t>
+        </is>
+      </c>
       <c r="D283" t="n">
         <v>8050</v>
       </c>
@@ -39742,7 +40518,11 @@
           <t>eight thousand fifty</t>
         </is>
       </c>
-      <c r="L283" t="inlineStr"/>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M283" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -39798,7 +40578,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z283" t="inlineStr"/>
+      <c r="Z283" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA283" t="n">
         <v>5</v>
       </c>
@@ -39848,8 +40632,16 @@
       <c r="A284" t="n">
         <v>16885</v>
       </c>
-      <c r="B284" t="inlineStr"/>
-      <c r="C284" t="inlineStr"/>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>J**** C*****</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>81****3759</t>
+        </is>
+      </c>
       <c r="D284" t="n">
         <v>7750</v>
       </c>
@@ -39884,7 +40676,11 @@
           <t>seven thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L284" t="inlineStr"/>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M284" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -39940,7 +40736,11 @@
           <t>QR_UPI</t>
         </is>
       </c>
-      <c r="Z284" t="inlineStr"/>
+      <c r="Z284" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA284" t="n">
         <v>5</v>
       </c>
@@ -39990,8 +40790,16 @@
       <c r="A285" t="n">
         <v>17215</v>
       </c>
-      <c r="B285" t="inlineStr"/>
-      <c r="C285" t="inlineStr"/>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>S********** S*****</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>95****8421</t>
+        </is>
+      </c>
       <c r="D285" t="n">
         <v>6750</v>
       </c>
@@ -40026,7 +40834,11 @@
           <t>six thousand seven hundred fifty</t>
         </is>
       </c>
-      <c r="L285" t="inlineStr"/>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
       <c r="M285" t="inlineStr">
         <is>
           <t>SALESIAN EDUCATION SOCIETY</t>
@@ -40082,7 +40894,11 @@
           <t>UPI</t>
         </is>
       </c>
-      <c r="Z285" t="inlineStr"/>
+      <c r="Z285" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
       <c r="AA285" t="n">
         <v>5</v>
       </c>
@@ -42158,6 +42974,164 @@
         </is>
       </c>
     </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>17187</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>C****** V********</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>88****8971</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E299" t="n">
+        <v>6750</v>
+      </c>
+      <c r="F299" s="1" t="n">
+        <v>46119.49782407407</v>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>08-Apr-2026 17:44:13</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>six thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N299" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O299" t="n">
+        <v>1234</v>
+      </c>
+      <c r="P299" t="n">
+        <v>11000357637359</v>
+      </c>
+      <c r="Q299" t="n">
+        <v>1775543193</v>
+      </c>
+      <c r="R299" t="n">
+        <v>115726878456</v>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V299" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W299" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X299" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y299" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z299" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA299" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB299" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC299" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD299" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE299" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF299" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG299" t="inlineStr"/>
+      <c r="AH299" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI299" t="n">
+        <v>19901</v>
+      </c>
+      <c r="AJ299" t="inlineStr">
+        <is>
+          <t>266636</t>
+        </is>
+      </c>
+      <c r="AK299" t="inlineStr">
+        <is>
+          <t>2055</t>
+        </is>
+      </c>
+      <c r="AL299" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Support 2026-27 data & improve ETL
Add support for the 2026-27 academic year across student and fee pipelines; include new GOOGLE env vars and sheet paths and merge df_2026 into merges. Improve Atom transaction downloader (driver setup, robust date setting, split_ranges, safer download wait) and move file paths to BASE_DIR. Change DB inserts from replace to append in multiple places, map academic_year_id for 3 years, and normalize phone/account columns to TEXT. Fix output paths for various helper CSVs and add small debugging prints. Data files updated: atom_report_cleaned*, daywise_fees_collection*, fees_collection* and merged_fee_collection with new payments (adm 16353, 17455). Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL436"/>
+  <dimension ref="A1:AL438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68796,6 +68796,294 @@
         </is>
       </c>
     </row>
+    <row r="437">
+      <c r="A437" t="n">
+        <v>16353</v>
+      </c>
+      <c r="B437" t="inlineStr"/>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>93****3084</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E437" t="inlineStr"/>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>06-Jul-2026 20:56:28</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr"/>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>*8469</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N437" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O437" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P437" t="n">
+        <v>11000371165679</v>
+      </c>
+      <c r="Q437" t="n">
+        <v>1783351470900</v>
+      </c>
+      <c r="R437" t="n">
+        <v>618726080298</v>
+      </c>
+      <c r="S437" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T437" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U437" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V437" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W437" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X437" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y437" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z437" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA437" t="inlineStr"/>
+      <c r="AB437" t="inlineStr"/>
+      <c r="AC437" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD437" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE437" t="inlineStr"/>
+      <c r="AF437" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG437" t="inlineStr"/>
+      <c r="AH437" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI437" t="n">
+        <v>18469</v>
+      </c>
+      <c r="AJ437" t="inlineStr">
+        <is>
+          <t>272507</t>
+        </is>
+      </c>
+      <c r="AK437" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>17455</v>
+      </c>
+      <c r="B438" t="inlineStr"/>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>73****9369</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E438" t="inlineStr"/>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>06-Jul-2026 21:58:43</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr"/>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>*0450</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N438" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O438" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P438" t="n">
+        <v>11000371178055</v>
+      </c>
+      <c r="Q438" t="n">
+        <v>1783355277549</v>
+      </c>
+      <c r="R438" t="n">
+        <v>298937086055</v>
+      </c>
+      <c r="S438" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T438" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U438" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V438" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W438" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X438" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y438" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z438" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA438" t="inlineStr"/>
+      <c r="AB438" t="inlineStr"/>
+      <c r="AC438" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD438" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE438" t="inlineStr"/>
+      <c r="AF438" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG438" t="inlineStr"/>
+      <c r="AH438" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI438" t="n">
+        <v>20450</v>
+      </c>
+      <c r="AJ438" t="inlineStr">
+        <is>
+          <t>277544</t>
+        </is>
+      </c>
+      <c r="AK438" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL438" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record online fee payments for two students
Add two successful online transactions dated 09-Jul-2026 for AdmissionNo 17001 (₹8,400) and 16567 (₹8,700). Updated atom_report (source and cleaned), daywise_fees_collection (including 2026-27 and online variants), fees_collection (both copies), and merged_fee_collection so Total_Fee_Paid and Total_Due reflect the new payments and reports include the new rows.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL449"/>
+  <dimension ref="A1:AL451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70874,6 +70874,290 @@
         </is>
       </c>
     </row>
+    <row r="450">
+      <c r="A450" t="n">
+        <v>17001</v>
+      </c>
+      <c r="B450" t="inlineStr"/>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>79****8806</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E450" t="inlineStr"/>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>09-Jul-2026 00:30:51</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr"/>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>*8090</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N450" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O450" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P450" t="n">
+        <v>11000371625455</v>
+      </c>
+      <c r="Q450" t="n">
+        <v>1783537186850</v>
+      </c>
+      <c r="R450" t="n">
+        <v>619021000861</v>
+      </c>
+      <c r="S450" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T450" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U450" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V450" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W450" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X450" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y450" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z450" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA450" t="inlineStr"/>
+      <c r="AB450" t="inlineStr"/>
+      <c r="AC450" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD450" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE450" t="inlineStr"/>
+      <c r="AF450" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG450" t="inlineStr"/>
+      <c r="AH450" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI450" t="n">
+        <v>18090</v>
+      </c>
+      <c r="AJ450" t="inlineStr">
+        <is>
+          <t>271343</t>
+        </is>
+      </c>
+      <c r="AK450" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL450" t="inlineStr"/>
+    </row>
+    <row r="451">
+      <c r="A451" t="n">
+        <v>16567</v>
+      </c>
+      <c r="B451" t="inlineStr"/>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>90****7436</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E451" t="inlineStr"/>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>09-Jul-2026 00:28:29</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr"/>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>*8277</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N451" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O451" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P451" t="n">
+        <v>11000371626441</v>
+      </c>
+      <c r="Q451" t="n">
+        <v>1783537025732</v>
+      </c>
+      <c r="R451" t="n">
+        <v>619041000858</v>
+      </c>
+      <c r="S451" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T451" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U451" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V451" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W451" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X451" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y451" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z451" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA451" t="inlineStr"/>
+      <c r="AB451" t="inlineStr"/>
+      <c r="AC451" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD451" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE451" t="inlineStr"/>
+      <c r="AF451" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG451" t="inlineStr"/>
+      <c r="AH451" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI451" t="n">
+        <v>18277</v>
+      </c>
+      <c r="AJ451" t="inlineStr">
+        <is>
+          <t>272327</t>
+        </is>
+      </c>
+      <c r="AK451" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL451" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 11-Jul-2026 fee transactions and update balances
Add new payment rows from 11-Jul-2026 to atom_report_cleaned (CSV/XLSX) and update daywise_fees_collection (regular, online, 2026-27). Reflect corresponding payments in fees_collection, fees_collection_2026_27_1 and merged_fee_collection (several admissions like 17277,15321,16209,14582,15541,15823,16721,16475,16476,15587,17459 etc. updated with paid amounts and reduced dues). Correct fee statuses in fees_report (several '3 Terms' entries changed to 'Total Paid'). Also update source_data/atom_report.xlsx to match. These changes record online/UPI/CC payments received on 11-Jul-2026.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL461"/>
+  <dimension ref="A1:AL472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72694,6 +72694,1616 @@
       </c>
       <c r="AL461" t="inlineStr"/>
     </row>
+    <row r="462">
+      <c r="A462" t="n">
+        <v>17277</v>
+      </c>
+      <c r="B462" t="inlineStr"/>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>96****1662</t>
+        </is>
+      </c>
+      <c r="D462" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E462" t="inlineStr"/>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 07:00:18</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr"/>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K462" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>*9988</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N462" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O462" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P462" t="n">
+        <v>11000372059838</v>
+      </c>
+      <c r="Q462" t="n">
+        <v>1783733404541</v>
+      </c>
+      <c r="R462" t="n">
+        <v>302708764437</v>
+      </c>
+      <c r="S462" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T462" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U462" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V462" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W462" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X462" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y462" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z462" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA462" t="inlineStr"/>
+      <c r="AB462" t="inlineStr"/>
+      <c r="AC462" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD462" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE462" t="inlineStr"/>
+      <c r="AF462" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG462" t="inlineStr"/>
+      <c r="AH462" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI462" t="n">
+        <v>19988</v>
+      </c>
+      <c r="AJ462" t="inlineStr">
+        <is>
+          <t>270330,271405</t>
+        </is>
+      </c>
+      <c r="AK462" t="inlineStr">
+        <is>
+          <t>2067,2076</t>
+        </is>
+      </c>
+      <c r="AL462" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="n">
+        <v>15321</v>
+      </c>
+      <c r="B463" t="inlineStr"/>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>90****6416</t>
+        </is>
+      </c>
+      <c r="D463" t="n">
+        <v>12200</v>
+      </c>
+      <c r="E463" t="inlineStr"/>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 07:10:05</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr"/>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>*8997</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N463" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O463" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P463" t="n">
+        <v>11000372063015</v>
+      </c>
+      <c r="Q463" t="n">
+        <v>1783733983603</v>
+      </c>
+      <c r="R463" t="n">
+        <v>76530301623</v>
+      </c>
+      <c r="S463" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T463" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U463" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V463" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W463" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X463" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y463" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z463" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA463" t="inlineStr"/>
+      <c r="AB463" t="inlineStr"/>
+      <c r="AC463" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD463" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE463" t="inlineStr"/>
+      <c r="AF463" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG463" t="inlineStr"/>
+      <c r="AH463" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI463" t="n">
+        <v>18997</v>
+      </c>
+      <c r="AJ463" t="inlineStr">
+        <is>
+          <t>270911,275393</t>
+        </is>
+      </c>
+      <c r="AK463" t="inlineStr">
+        <is>
+          <t>2075,2092</t>
+        </is>
+      </c>
+      <c r="AL463" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="n">
+        <v>16209</v>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>V********** N**** S**</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>81****1333</t>
+        </is>
+      </c>
+      <c r="D464" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E464" t="inlineStr"/>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 08:21:46</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr"/>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nine thousand </t>
+        </is>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N464" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O464" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="P464" t="n">
+        <v>11000372067768</v>
+      </c>
+      <c r="Q464" t="n">
+        <v>1783738279</v>
+      </c>
+      <c r="R464" t="n">
+        <v>105959969580</v>
+      </c>
+      <c r="S464" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T464" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U464" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V464" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W464" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X464" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y464" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z464" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA464" t="inlineStr"/>
+      <c r="AB464" t="inlineStr"/>
+      <c r="AC464" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD464" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE464" t="inlineStr"/>
+      <c r="AF464" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG464" t="inlineStr"/>
+      <c r="AH464" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI464" t="n">
+        <v>18690</v>
+      </c>
+      <c r="AJ464" t="inlineStr">
+        <is>
+          <t>273722</t>
+        </is>
+      </c>
+      <c r="AK464" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL464" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="n">
+        <v>14582</v>
+      </c>
+      <c r="B465" t="inlineStr"/>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>93****9606</t>
+        </is>
+      </c>
+      <c r="D465" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E465" t="inlineStr"/>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 12:34:57</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr"/>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>*9354</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N465" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O465" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P465" t="n">
+        <v>11000372113886</v>
+      </c>
+      <c r="Q465" t="n">
+        <v>1783753406583</v>
+      </c>
+      <c r="R465" t="n">
+        <v>724009638591</v>
+      </c>
+      <c r="S465" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T465" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U465" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V465" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W465" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X465" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y465" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z465" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA465" t="inlineStr"/>
+      <c r="AB465" t="inlineStr"/>
+      <c r="AC465" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD465" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE465" t="inlineStr"/>
+      <c r="AF465" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG465" t="inlineStr"/>
+      <c r="AH465" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI465" t="n">
+        <v>19354</v>
+      </c>
+      <c r="AJ465" t="inlineStr">
+        <is>
+          <t>276079</t>
+        </is>
+      </c>
+      <c r="AK465" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL465" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="n">
+        <v>15541</v>
+      </c>
+      <c r="B466" t="inlineStr"/>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>98****9449</t>
+        </is>
+      </c>
+      <c r="D466" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E466" t="inlineStr"/>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 12:35:19</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr"/>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>*8766</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N466" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O466" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P466" t="n">
+        <v>11000372114900</v>
+      </c>
+      <c r="Q466" t="n">
+        <v>1783753512275</v>
+      </c>
+      <c r="R466" t="n">
+        <v>429700282239</v>
+      </c>
+      <c r="S466" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T466" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U466" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V466" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W466" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X466" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y466" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z466" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA466" t="inlineStr"/>
+      <c r="AB466" t="inlineStr"/>
+      <c r="AC466" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD466" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE466" t="inlineStr"/>
+      <c r="AF466" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG466" t="inlineStr"/>
+      <c r="AH466" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI466" t="n">
+        <v>18766</v>
+      </c>
+      <c r="AJ466" t="inlineStr">
+        <is>
+          <t>273735</t>
+        </is>
+      </c>
+      <c r="AK466" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL466" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="n">
+        <v>15587</v>
+      </c>
+      <c r="B467" t="inlineStr"/>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>93****9606</t>
+        </is>
+      </c>
+      <c r="D467" t="n">
+        <v>9400</v>
+      </c>
+      <c r="E467" t="inlineStr"/>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 12:48:58</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr"/>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>*8856</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N467" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O467" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P467" t="n">
+        <v>11000372117902</v>
+      </c>
+      <c r="Q467" t="n">
+        <v>1783754283667</v>
+      </c>
+      <c r="R467" t="n">
+        <v>999343787537</v>
+      </c>
+      <c r="S467" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T467" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U467" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V467" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W467" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X467" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y467" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z467" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA467" t="inlineStr"/>
+      <c r="AB467" t="inlineStr"/>
+      <c r="AC467" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD467" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE467" t="inlineStr"/>
+      <c r="AF467" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG467" t="inlineStr"/>
+      <c r="AH467" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI467" t="n">
+        <v>18856</v>
+      </c>
+      <c r="AJ467" t="inlineStr">
+        <is>
+          <t>274809</t>
+        </is>
+      </c>
+      <c r="AK467" t="inlineStr">
+        <is>
+          <t>2088</t>
+        </is>
+      </c>
+      <c r="AL467" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>17459</v>
+      </c>
+      <c r="B468" t="inlineStr"/>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>91****3633</t>
+        </is>
+      </c>
+      <c r="D468" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E468" t="inlineStr"/>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 13:49:46</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>*0171</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N468" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O468" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P468" t="n">
+        <v>11000372131404</v>
+      </c>
+      <c r="Q468" t="n">
+        <v>1783757872189</v>
+      </c>
+      <c r="R468" t="n">
+        <v>655863582381</v>
+      </c>
+      <c r="S468" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T468" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U468" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V468" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W468" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X468" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y468" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z468" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA468" t="inlineStr"/>
+      <c r="AB468" t="inlineStr"/>
+      <c r="AC468" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD468" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE468" t="inlineStr"/>
+      <c r="AF468" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG468" t="inlineStr"/>
+      <c r="AH468" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI468" t="n">
+        <v>20171</v>
+      </c>
+      <c r="AJ468" t="inlineStr">
+        <is>
+          <t>271165</t>
+        </is>
+      </c>
+      <c r="AK468" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL468" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>15823</v>
+      </c>
+      <c r="B469" t="inlineStr"/>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>99****1635</t>
+        </is>
+      </c>
+      <c r="D469" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E469" t="inlineStr"/>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 15:25:36</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr"/>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>*8720</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N469" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O469" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P469" t="n">
+        <v>11000372145896</v>
+      </c>
+      <c r="Q469" t="n">
+        <v>1783763721706</v>
+      </c>
+      <c r="R469" t="n">
+        <v>673975146257</v>
+      </c>
+      <c r="S469" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T469" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U469" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V469" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W469" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X469" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y469" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z469" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA469" t="inlineStr"/>
+      <c r="AB469" t="inlineStr"/>
+      <c r="AC469" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD469" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE469" t="inlineStr"/>
+      <c r="AF469" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG469" t="inlineStr"/>
+      <c r="AH469" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI469" t="n">
+        <v>18720</v>
+      </c>
+      <c r="AJ469" t="inlineStr">
+        <is>
+          <t>273694</t>
+        </is>
+      </c>
+      <c r="AK469" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL469" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>16721</v>
+      </c>
+      <c r="B470" t="inlineStr"/>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>99****1635</t>
+        </is>
+      </c>
+      <c r="D470" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E470" t="inlineStr"/>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 15:20:17</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr"/>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>*8114</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N470" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O470" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P470" t="n">
+        <v>11000372146568</v>
+      </c>
+      <c r="Q470" t="n">
+        <v>1783763397059</v>
+      </c>
+      <c r="R470" t="n">
+        <v>482482929627</v>
+      </c>
+      <c r="S470" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T470" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U470" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V470" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W470" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X470" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y470" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z470" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA470" t="inlineStr"/>
+      <c r="AB470" t="inlineStr"/>
+      <c r="AC470" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD470" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE470" t="inlineStr"/>
+      <c r="AF470" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG470" t="inlineStr"/>
+      <c r="AH470" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI470" t="n">
+        <v>18114</v>
+      </c>
+      <c r="AJ470" t="inlineStr">
+        <is>
+          <t>271206</t>
+        </is>
+      </c>
+      <c r="AK470" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL470" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>16476</v>
+      </c>
+      <c r="B471" t="inlineStr"/>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>99****3153</t>
+        </is>
+      </c>
+      <c r="D471" t="n">
+        <v>9400</v>
+      </c>
+      <c r="E471" t="inlineStr"/>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 19:44:08</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr"/>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>*8969</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N471" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O471" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P471" t="n">
+        <v>11000372181653</v>
+      </c>
+      <c r="Q471" t="n">
+        <v>1783779230077</v>
+      </c>
+      <c r="R471" t="n">
+        <v>663341327002</v>
+      </c>
+      <c r="S471" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T471" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U471" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V471" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W471" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X471" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y471" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z471" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA471" t="inlineStr"/>
+      <c r="AB471" t="inlineStr"/>
+      <c r="AC471" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD471" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE471" t="inlineStr"/>
+      <c r="AF471" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG471" t="inlineStr"/>
+      <c r="AH471" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI471" t="n">
+        <v>18969</v>
+      </c>
+      <c r="AJ471" t="inlineStr">
+        <is>
+          <t>274865</t>
+        </is>
+      </c>
+      <c r="AK471" t="inlineStr">
+        <is>
+          <t>2088</t>
+        </is>
+      </c>
+      <c r="AL471" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>16475</v>
+      </c>
+      <c r="B472" t="inlineStr"/>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>99****3153</t>
+        </is>
+      </c>
+      <c r="D472" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E472" t="inlineStr"/>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>11-Jul-2026 19:46:59</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr"/>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>*8788</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N472" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O472" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P472" t="n">
+        <v>11000372182083</v>
+      </c>
+      <c r="Q472" t="n">
+        <v>1783779407447</v>
+      </c>
+      <c r="R472" t="n">
+        <v>381430784071</v>
+      </c>
+      <c r="S472" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T472" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U472" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V472" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W472" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X472" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y472" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z472" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA472" t="inlineStr"/>
+      <c r="AB472" t="inlineStr"/>
+      <c r="AC472" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD472" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE472" t="inlineStr"/>
+      <c r="AF472" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG472" t="inlineStr"/>
+      <c r="AH472" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI472" t="n">
+        <v>18788</v>
+      </c>
+      <c r="AJ472" t="inlineStr">
+        <is>
+          <t>273686</t>
+        </is>
+      </c>
+      <c r="AK472" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL472" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add payment for admission 17219 and update reports
Insert a new UPI transaction for KUMARI VARTIKA (AdmissionNo 17219) — ₹8,400 on 12-Jul-2026 — into the Atom report and cleaned exports. Propagated the change to daywise_fees_collection (including 2026-27 and online CSVs), fees_collection (Total_Fee_Paid set to 8400 and Total_Due adjusted) and merged_fee_collection. Updated source_data/atom_report.xlsx and regenerated atom_report_cleaned.*. Also committed executed outputs for source_code/KOTAK_DB.ipynb (execution counts and run outputs captured).
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL472"/>
+  <dimension ref="A1:AL473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74304,6 +74304,152 @@
         </is>
       </c>
     </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>17219</v>
+      </c>
+      <c r="B473" t="inlineStr"/>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>83****9788</t>
+        </is>
+      </c>
+      <c r="D473" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E473" t="inlineStr"/>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>12-Jul-2026 13:25:18</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr"/>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K473" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>*9931</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N473" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O473" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P473" t="n">
+        <v>11000372261199</v>
+      </c>
+      <c r="Q473" t="n">
+        <v>1783842905483</v>
+      </c>
+      <c r="R473" t="n">
+        <v>136649511585</v>
+      </c>
+      <c r="S473" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T473" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U473" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V473" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W473" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X473" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y473" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z473" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA473" t="inlineStr"/>
+      <c r="AB473" t="inlineStr"/>
+      <c r="AC473" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD473" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE473" t="inlineStr"/>
+      <c r="AF473" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG473" t="inlineStr"/>
+      <c r="AH473" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI473" t="n">
+        <v>19931</v>
+      </c>
+      <c r="AJ473" t="inlineStr">
+        <is>
+          <t>271238</t>
+        </is>
+      </c>
+      <c r="AK473" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL473" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update fees collection and student data
Refresh output data files with latest fees transactions and student records. Update includes:
- Atom transaction report with settled payments and corrected amounts
- Daywise fees collection data with new payment records
- Student contact information corrections
- Clear Jupyter notebook cell outputs
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL473"/>
+  <dimension ref="A1:AL488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71693,7 +71693,9 @@
       <c r="D455" t="n">
         <v>12300</v>
       </c>
-      <c r="E455" t="inlineStr"/>
+      <c r="E455" t="n">
+        <v>12300</v>
+      </c>
       <c r="F455" t="inlineStr">
         <is>
           <t>10-Jul-2026 07:02:55</t>
@@ -71764,7 +71766,7 @@
       </c>
       <c r="V455" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W455" t="inlineStr">
@@ -71787,15 +71789,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA455" t="inlineStr"/>
-      <c r="AB455" t="inlineStr"/>
+      <c r="AA455" t="n">
+        <v>166.05</v>
+      </c>
+      <c r="AB455" t="n">
+        <v>29.89</v>
+      </c>
       <c r="AC455" t="n">
         <v>0</v>
       </c>
       <c r="AD455" t="n">
         <v>0</v>
       </c>
-      <c r="AE455" t="inlineStr"/>
+      <c r="AE455" t="n">
+        <v>195.94</v>
+      </c>
       <c r="AF455" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -71835,13 +71843,19 @@
       <c r="D456" t="n">
         <v>8400</v>
       </c>
-      <c r="E456" t="inlineStr"/>
+      <c r="E456" t="n">
+        <v>8400</v>
+      </c>
       <c r="F456" t="inlineStr">
         <is>
           <t>10-Jul-2026 15:32:30</t>
         </is>
       </c>
-      <c r="G456" t="inlineStr"/>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H456" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -71906,7 +71920,7 @@
       </c>
       <c r="V456" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W456" t="inlineStr">
@@ -71929,15 +71943,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA456" t="inlineStr"/>
-      <c r="AB456" t="inlineStr"/>
+      <c r="AA456" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB456" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC456" t="n">
         <v>0</v>
       </c>
       <c r="AD456" t="n">
         <v>0</v>
       </c>
-      <c r="AE456" t="inlineStr"/>
+      <c r="AE456" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF456" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -71981,13 +72001,19 @@
       <c r="D457" t="n">
         <v>7250</v>
       </c>
-      <c r="E457" t="inlineStr"/>
+      <c r="E457" t="n">
+        <v>7250</v>
+      </c>
       <c r="F457" t="inlineStr">
         <is>
           <t>10-Jul-2026 15:36:18</t>
         </is>
       </c>
-      <c r="G457" t="inlineStr"/>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H457" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -72052,7 +72078,7 @@
       </c>
       <c r="V457" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W457" t="inlineStr">
@@ -72075,15 +72101,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA457" t="inlineStr"/>
-      <c r="AB457" t="inlineStr"/>
+      <c r="AA457" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB457" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC457" t="n">
         <v>0</v>
       </c>
       <c r="AD457" t="n">
         <v>0</v>
       </c>
-      <c r="AE457" t="inlineStr"/>
+      <c r="AE457" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF457" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
@@ -72127,13 +72159,19 @@
       <c r="D458" t="n">
         <v>8400</v>
       </c>
-      <c r="E458" t="inlineStr"/>
+      <c r="E458" t="n">
+        <v>8400</v>
+      </c>
       <c r="F458" t="inlineStr">
         <is>
           <t>10-Jul-2026 16:20:33</t>
         </is>
       </c>
-      <c r="G458" t="inlineStr"/>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H458" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -72198,7 +72236,7 @@
       </c>
       <c r="V458" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W458" t="inlineStr">
@@ -72221,15 +72259,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA458" t="inlineStr"/>
-      <c r="AB458" t="inlineStr"/>
+      <c r="AA458" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB458" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC458" t="n">
         <v>0</v>
       </c>
       <c r="AD458" t="n">
         <v>0</v>
       </c>
-      <c r="AE458" t="inlineStr"/>
+      <c r="AE458" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF458" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -72273,13 +72317,19 @@
       <c r="D459" t="n">
         <v>9000</v>
       </c>
-      <c r="E459" t="inlineStr"/>
+      <c r="E459" t="n">
+        <v>9000</v>
+      </c>
       <c r="F459" t="inlineStr">
         <is>
           <t>10-Jul-2026 16:21:27</t>
         </is>
       </c>
-      <c r="G459" t="inlineStr"/>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H459" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -72344,7 +72394,7 @@
       </c>
       <c r="V459" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W459" t="inlineStr">
@@ -72367,15 +72417,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA459" t="inlineStr"/>
-      <c r="AB459" t="inlineStr"/>
+      <c r="AA459" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB459" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC459" t="n">
         <v>0</v>
       </c>
       <c r="AD459" t="n">
         <v>0</v>
       </c>
-      <c r="AE459" t="inlineStr"/>
+      <c r="AE459" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF459" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -72419,13 +72475,19 @@
       <c r="D460" t="n">
         <v>7250</v>
       </c>
-      <c r="E460" t="inlineStr"/>
+      <c r="E460" t="n">
+        <v>7250</v>
+      </c>
       <c r="F460" t="inlineStr">
         <is>
           <t>10-Jul-2026 17:45:46</t>
         </is>
       </c>
-      <c r="G460" t="inlineStr"/>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H460" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -72490,7 +72552,7 @@
       </c>
       <c r="V460" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W460" t="inlineStr">
@@ -72513,15 +72575,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA460" t="inlineStr"/>
-      <c r="AB460" t="inlineStr"/>
+      <c r="AA460" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB460" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC460" t="n">
         <v>0</v>
       </c>
       <c r="AD460" t="n">
         <v>0</v>
       </c>
-      <c r="AE460" t="inlineStr"/>
+      <c r="AE460" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF460" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
@@ -72565,7 +72633,9 @@
       <c r="D461" t="n">
         <v>12300</v>
       </c>
-      <c r="E461" t="inlineStr"/>
+      <c r="E461" t="n">
+        <v>12300</v>
+      </c>
       <c r="F461" t="inlineStr">
         <is>
           <t>11-Jul-2026 00:12:30</t>
@@ -72636,7 +72706,7 @@
       </c>
       <c r="V461" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W461" t="inlineStr">
@@ -72659,15 +72729,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA461" t="inlineStr"/>
-      <c r="AB461" t="inlineStr"/>
+      <c r="AA461" t="n">
+        <v>147.6</v>
+      </c>
+      <c r="AB461" t="n">
+        <v>26.57</v>
+      </c>
       <c r="AC461" t="n">
         <v>0</v>
       </c>
       <c r="AD461" t="n">
         <v>0</v>
       </c>
-      <c r="AE461" t="inlineStr"/>
+      <c r="AE461" t="n">
+        <v>174.17</v>
+      </c>
       <c r="AF461" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -72707,13 +72783,19 @@
       <c r="D462" t="n">
         <v>9000</v>
       </c>
-      <c r="E462" t="inlineStr"/>
+      <c r="E462" t="n">
+        <v>9000</v>
+      </c>
       <c r="F462" t="inlineStr">
         <is>
           <t>11-Jul-2026 07:00:18</t>
         </is>
       </c>
-      <c r="G462" t="inlineStr"/>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H462" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -72778,7 +72860,7 @@
       </c>
       <c r="V462" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W462" t="inlineStr">
@@ -72801,15 +72883,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA462" t="inlineStr"/>
-      <c r="AB462" t="inlineStr"/>
+      <c r="AA462" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB462" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC462" t="n">
         <v>0</v>
       </c>
       <c r="AD462" t="n">
         <v>0</v>
       </c>
-      <c r="AE462" t="inlineStr"/>
+      <c r="AE462" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF462" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -72853,7 +72941,9 @@
       <c r="D463" t="n">
         <v>12200</v>
       </c>
-      <c r="E463" t="inlineStr"/>
+      <c r="E463" t="n">
+        <v>12200</v>
+      </c>
       <c r="F463" t="inlineStr">
         <is>
           <t>11-Jul-2026 07:10:05</t>
@@ -72924,7 +73014,7 @@
       </c>
       <c r="V463" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W463" t="inlineStr">
@@ -72947,15 +73037,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA463" t="inlineStr"/>
-      <c r="AB463" t="inlineStr"/>
+      <c r="AA463" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB463" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC463" t="n">
         <v>0</v>
       </c>
       <c r="AD463" t="n">
         <v>0</v>
       </c>
-      <c r="AE463" t="inlineStr"/>
+      <c r="AE463" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF463" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -73003,13 +73099,19 @@
       <c r="D464" t="n">
         <v>9000</v>
       </c>
-      <c r="E464" t="inlineStr"/>
+      <c r="E464" t="n">
+        <v>9000</v>
+      </c>
       <c r="F464" t="inlineStr">
         <is>
           <t>11-Jul-2026 08:21:46</t>
         </is>
       </c>
-      <c r="G464" t="inlineStr"/>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H464" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -73074,7 +73176,7 @@
       </c>
       <c r="V464" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W464" t="inlineStr">
@@ -73097,15 +73199,21 @@
           <t>k*************@gmail.com</t>
         </is>
       </c>
-      <c r="AA464" t="inlineStr"/>
-      <c r="AB464" t="inlineStr"/>
+      <c r="AA464" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB464" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC464" t="n">
         <v>0</v>
       </c>
       <c r="AD464" t="n">
         <v>0</v>
       </c>
-      <c r="AE464" t="inlineStr"/>
+      <c r="AE464" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF464" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -73149,7 +73257,9 @@
       <c r="D465" t="n">
         <v>12300</v>
       </c>
-      <c r="E465" t="inlineStr"/>
+      <c r="E465" t="n">
+        <v>12300</v>
+      </c>
       <c r="F465" t="inlineStr">
         <is>
           <t>11-Jul-2026 12:34:57</t>
@@ -73220,7 +73330,7 @@
       </c>
       <c r="V465" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W465" t="inlineStr">
@@ -73243,15 +73353,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA465" t="inlineStr"/>
-      <c r="AB465" t="inlineStr"/>
+      <c r="AA465" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB465" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC465" t="n">
         <v>0</v>
       </c>
       <c r="AD465" t="n">
         <v>0</v>
       </c>
-      <c r="AE465" t="inlineStr"/>
+      <c r="AE465" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF465" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -73295,13 +73411,19 @@
       <c r="D466" t="n">
         <v>9000</v>
       </c>
-      <c r="E466" t="inlineStr"/>
+      <c r="E466" t="n">
+        <v>9000</v>
+      </c>
       <c r="F466" t="inlineStr">
         <is>
           <t>11-Jul-2026 12:35:19</t>
         </is>
       </c>
-      <c r="G466" t="inlineStr"/>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H466" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -73366,7 +73488,7 @@
       </c>
       <c r="V466" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W466" t="inlineStr">
@@ -73389,15 +73511,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA466" t="inlineStr"/>
-      <c r="AB466" t="inlineStr"/>
+      <c r="AA466" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB466" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC466" t="n">
         <v>0</v>
       </c>
       <c r="AD466" t="n">
         <v>0</v>
       </c>
-      <c r="AE466" t="inlineStr"/>
+      <c r="AE466" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF466" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -73441,7 +73569,9 @@
       <c r="D467" t="n">
         <v>9400</v>
       </c>
-      <c r="E467" t="inlineStr"/>
+      <c r="E467" t="n">
+        <v>9400</v>
+      </c>
       <c r="F467" t="inlineStr">
         <is>
           <t>11-Jul-2026 12:48:58</t>
@@ -73512,7 +73642,7 @@
       </c>
       <c r="V467" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W467" t="inlineStr">
@@ -73535,15 +73665,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA467" t="inlineStr"/>
-      <c r="AB467" t="inlineStr"/>
+      <c r="AA467" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB467" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC467" t="n">
         <v>0</v>
       </c>
       <c r="AD467" t="n">
         <v>0</v>
       </c>
-      <c r="AE467" t="inlineStr"/>
+      <c r="AE467" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF467" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
@@ -73587,13 +73723,19 @@
       <c r="D468" t="n">
         <v>8400</v>
       </c>
-      <c r="E468" t="inlineStr"/>
+      <c r="E468" t="n">
+        <v>8400</v>
+      </c>
       <c r="F468" t="inlineStr">
         <is>
           <t>11-Jul-2026 13:49:46</t>
         </is>
       </c>
-      <c r="G468" t="inlineStr"/>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H468" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -73658,7 +73800,7 @@
       </c>
       <c r="V468" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W468" t="inlineStr">
@@ -73681,15 +73823,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA468" t="inlineStr"/>
-      <c r="AB468" t="inlineStr"/>
+      <c r="AA468" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB468" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC468" t="n">
         <v>0</v>
       </c>
       <c r="AD468" t="n">
         <v>0</v>
       </c>
-      <c r="AE468" t="inlineStr"/>
+      <c r="AE468" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF468" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -73733,13 +73881,19 @@
       <c r="D469" t="n">
         <v>9000</v>
       </c>
-      <c r="E469" t="inlineStr"/>
+      <c r="E469" t="n">
+        <v>9000</v>
+      </c>
       <c r="F469" t="inlineStr">
         <is>
           <t>11-Jul-2026 15:25:36</t>
         </is>
       </c>
-      <c r="G469" t="inlineStr"/>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H469" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -73804,7 +73958,7 @@
       </c>
       <c r="V469" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W469" t="inlineStr">
@@ -73827,15 +73981,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA469" t="inlineStr"/>
-      <c r="AB469" t="inlineStr"/>
+      <c r="AA469" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB469" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC469" t="n">
         <v>0</v>
       </c>
       <c r="AD469" t="n">
         <v>0</v>
       </c>
-      <c r="AE469" t="inlineStr"/>
+      <c r="AE469" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF469" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -73879,13 +74039,19 @@
       <c r="D470" t="n">
         <v>8400</v>
       </c>
-      <c r="E470" t="inlineStr"/>
+      <c r="E470" t="n">
+        <v>8400</v>
+      </c>
       <c r="F470" t="inlineStr">
         <is>
           <t>11-Jul-2026 15:20:17</t>
         </is>
       </c>
-      <c r="G470" t="inlineStr"/>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H470" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -73950,7 +74116,7 @@
       </c>
       <c r="V470" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W470" t="inlineStr">
@@ -73973,15 +74139,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA470" t="inlineStr"/>
-      <c r="AB470" t="inlineStr"/>
+      <c r="AA470" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB470" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC470" t="n">
         <v>0</v>
       </c>
       <c r="AD470" t="n">
         <v>0</v>
       </c>
-      <c r="AE470" t="inlineStr"/>
+      <c r="AE470" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF470" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -74025,7 +74197,9 @@
       <c r="D471" t="n">
         <v>9400</v>
       </c>
-      <c r="E471" t="inlineStr"/>
+      <c r="E471" t="n">
+        <v>9400</v>
+      </c>
       <c r="F471" t="inlineStr">
         <is>
           <t>11-Jul-2026 19:44:08</t>
@@ -74096,7 +74270,7 @@
       </c>
       <c r="V471" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W471" t="inlineStr">
@@ -74119,15 +74293,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA471" t="inlineStr"/>
-      <c r="AB471" t="inlineStr"/>
+      <c r="AA471" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB471" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC471" t="n">
         <v>0</v>
       </c>
       <c r="AD471" t="n">
         <v>0</v>
       </c>
-      <c r="AE471" t="inlineStr"/>
+      <c r="AE471" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF471" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
@@ -74171,13 +74351,19 @@
       <c r="D472" t="n">
         <v>9000</v>
       </c>
-      <c r="E472" t="inlineStr"/>
+      <c r="E472" t="n">
+        <v>9000</v>
+      </c>
       <c r="F472" t="inlineStr">
         <is>
           <t>11-Jul-2026 19:46:59</t>
         </is>
       </c>
-      <c r="G472" t="inlineStr"/>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H472" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -74242,7 +74428,7 @@
       </c>
       <c r="V472" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W472" t="inlineStr">
@@ -74265,15 +74451,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA472" t="inlineStr"/>
-      <c r="AB472" t="inlineStr"/>
+      <c r="AA472" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB472" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC472" t="n">
         <v>0</v>
       </c>
       <c r="AD472" t="n">
         <v>0</v>
       </c>
-      <c r="AE472" t="inlineStr"/>
+      <c r="AE472" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF472" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -74317,13 +74509,19 @@
       <c r="D473" t="n">
         <v>8400</v>
       </c>
-      <c r="E473" t="inlineStr"/>
+      <c r="E473" t="n">
+        <v>8400</v>
+      </c>
       <c r="F473" t="inlineStr">
         <is>
           <t>12-Jul-2026 13:25:18</t>
         </is>
       </c>
-      <c r="G473" t="inlineStr"/>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
       <c r="H473" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -74388,7 +74586,7 @@
       </c>
       <c r="V473" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W473" t="inlineStr">
@@ -74411,15 +74609,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA473" t="inlineStr"/>
-      <c r="AB473" t="inlineStr"/>
+      <c r="AA473" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB473" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC473" t="n">
         <v>0</v>
       </c>
       <c r="AD473" t="n">
         <v>0</v>
       </c>
-      <c r="AE473" t="inlineStr"/>
+      <c r="AE473" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF473" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -74449,6 +74653,2240 @@
           <t>UPI INTENT</t>
         </is>
       </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="n">
+        <v>16552</v>
+      </c>
+      <c r="B474" t="inlineStr"/>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>98****7189</t>
+        </is>
+      </c>
+      <c r="D474" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E474" t="n">
+        <v>8700</v>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>12-Jul-2026 14:46:57</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>*8375</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N474" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O474" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P474" t="n">
+        <v>11000372271363</v>
+      </c>
+      <c r="Q474" t="n">
+        <v>1783847740793</v>
+      </c>
+      <c r="R474" t="n">
+        <v>900975042052</v>
+      </c>
+      <c r="S474" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T474" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U474" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V474" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W474" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X474" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y474" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z474" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA474" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB474" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC474" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD474" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE474" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF474" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG474" t="inlineStr"/>
+      <c r="AH474" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI474" t="n">
+        <v>18375</v>
+      </c>
+      <c r="AJ474" t="inlineStr">
+        <is>
+          <t>272434</t>
+        </is>
+      </c>
+      <c r="AK474" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL474" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="n">
+        <v>17417</v>
+      </c>
+      <c r="B475" t="inlineStr"/>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>83****4561</t>
+        </is>
+      </c>
+      <c r="D475" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E475" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>12-Jul-2026 15:28:40</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>*0447</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N475" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O475" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P475" t="n">
+        <v>11000372274677</v>
+      </c>
+      <c r="Q475" t="n">
+        <v>1783850310406</v>
+      </c>
+      <c r="R475" t="n">
+        <v>199681789218</v>
+      </c>
+      <c r="S475" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T475" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U475" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V475" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W475" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X475" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y475" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z475" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA475" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB475" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC475" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD475" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE475" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF475" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG475" t="inlineStr"/>
+      <c r="AH475" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI475" t="n">
+        <v>20447</v>
+      </c>
+      <c r="AJ475" t="inlineStr">
+        <is>
+          <t>277531</t>
+        </is>
+      </c>
+      <c r="AK475" t="inlineStr">
+        <is>
+          <t>2065</t>
+        </is>
+      </c>
+      <c r="AL475" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="n">
+        <v>15915</v>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>K******* J*****</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>81****8482</t>
+        </is>
+      </c>
+      <c r="D476" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E476" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>12-Jul-2026 15:36:35</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nine thousand </t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N476" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O476" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="P476" t="n">
+        <v>11000372274949</v>
+      </c>
+      <c r="Q476" t="n">
+        <v>1783850726</v>
+      </c>
+      <c r="R476" t="n">
+        <v>619341050138</v>
+      </c>
+      <c r="S476" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T476" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U476" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V476" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W476" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X476" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y476" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="Z476" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA476" t="n">
+        <v>81</v>
+      </c>
+      <c r="AB476" t="n">
+        <v>14.58</v>
+      </c>
+      <c r="AC476" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD476" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE476" t="n">
+        <v>95.58</v>
+      </c>
+      <c r="AF476" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG476" t="inlineStr"/>
+      <c r="AH476" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI476" t="n">
+        <v>18704</v>
+      </c>
+      <c r="AJ476" t="inlineStr">
+        <is>
+          <t>273773</t>
+        </is>
+      </c>
+      <c r="AK476" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL476" t="inlineStr"/>
+    </row>
+    <row r="477">
+      <c r="A477" t="n">
+        <v>17477</v>
+      </c>
+      <c r="B477" t="inlineStr"/>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>92****7887</t>
+        </is>
+      </c>
+      <c r="D477" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E477" t="n">
+        <v>7250</v>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>12-Jul-2026 18:44:55</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>*0151</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N477" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O477" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P477" t="n">
+        <v>11000372295469</v>
+      </c>
+      <c r="Q477" t="n">
+        <v>1783862052004</v>
+      </c>
+      <c r="R477" t="n">
+        <v>619302536692</v>
+      </c>
+      <c r="S477" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T477" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U477" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V477" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W477" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X477" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y477" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z477" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA477" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB477" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC477" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD477" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE477" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="AF477" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG477" t="inlineStr"/>
+      <c r="AH477" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI477" t="n">
+        <v>20151</v>
+      </c>
+      <c r="AJ477" t="inlineStr">
+        <is>
+          <t>269266</t>
+        </is>
+      </c>
+      <c r="AK477" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="AL477" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="n">
+        <v>17476</v>
+      </c>
+      <c r="B478" t="inlineStr"/>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>92****7887</t>
+        </is>
+      </c>
+      <c r="D478" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E478" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>12-Jul-2026 18:55:19</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:11:05</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>*0193</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N478" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O478" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P478" t="n">
+        <v>11000372295995</v>
+      </c>
+      <c r="Q478" t="n">
+        <v>1783862507456</v>
+      </c>
+      <c r="R478" t="n">
+        <v>619323086570</v>
+      </c>
+      <c r="S478" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T478" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U478" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V478" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="W478" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X478" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y478" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z478" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA478" t="n">
+        <v>108</v>
+      </c>
+      <c r="AB478" t="n">
+        <v>19.44</v>
+      </c>
+      <c r="AC478" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD478" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE478" t="n">
+        <v>127.44</v>
+      </c>
+      <c r="AF478" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG478" t="inlineStr"/>
+      <c r="AH478" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI478" t="n">
+        <v>20193</v>
+      </c>
+      <c r="AJ478" t="inlineStr">
+        <is>
+          <t>273486</t>
+        </is>
+      </c>
+      <c r="AK478" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL478" t="inlineStr"/>
+    </row>
+    <row r="479">
+      <c r="A479" t="n">
+        <v>14988</v>
+      </c>
+      <c r="B479" t="inlineStr"/>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>99****1686</t>
+        </is>
+      </c>
+      <c r="D479" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E479" t="inlineStr"/>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 08:43:44</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr"/>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>*9209</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N479" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O479" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P479" t="n">
+        <v>11000372366091</v>
+      </c>
+      <c r="Q479" t="n">
+        <v>1783912411054</v>
+      </c>
+      <c r="R479" t="n">
+        <v>534781613024</v>
+      </c>
+      <c r="S479" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T479" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U479" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V479" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W479" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X479" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y479" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z479" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA479" t="inlineStr"/>
+      <c r="AB479" t="inlineStr"/>
+      <c r="AC479" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD479" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE479" t="inlineStr"/>
+      <c r="AF479" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG479" t="inlineStr"/>
+      <c r="AH479" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI479" t="n">
+        <v>19209</v>
+      </c>
+      <c r="AJ479" t="inlineStr">
+        <is>
+          <t>275933</t>
+        </is>
+      </c>
+      <c r="AK479" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL479" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="n">
+        <v>17645</v>
+      </c>
+      <c r="B480" t="inlineStr"/>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>85****2836</t>
+        </is>
+      </c>
+      <c r="D480" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E480" t="inlineStr"/>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 08:50:31</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr"/>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>*0410</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N480" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O480" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P480" t="n">
+        <v>11000372367339</v>
+      </c>
+      <c r="Q480" t="n">
+        <v>1783912802746</v>
+      </c>
+      <c r="R480" t="n">
+        <v>927027233779</v>
+      </c>
+      <c r="S480" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T480" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U480" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V480" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W480" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X480" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y480" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z480" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA480" t="inlineStr"/>
+      <c r="AB480" t="inlineStr"/>
+      <c r="AC480" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD480" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE480" t="inlineStr"/>
+      <c r="AF480" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG480" t="inlineStr"/>
+      <c r="AH480" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI480" t="n">
+        <v>20410</v>
+      </c>
+      <c r="AJ480" t="inlineStr">
+        <is>
+          <t>277380</t>
+        </is>
+      </c>
+      <c r="AK480" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL480" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="n">
+        <v>14944</v>
+      </c>
+      <c r="B481" t="inlineStr"/>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>97****3320</t>
+        </is>
+      </c>
+      <c r="D481" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E481" t="inlineStr"/>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 09:46:23</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr"/>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>*9236</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N481" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O481" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P481" t="n">
+        <v>11000372375804</v>
+      </c>
+      <c r="Q481" t="n">
+        <v>1783916164452</v>
+      </c>
+      <c r="R481" t="n">
+        <v>815132583286</v>
+      </c>
+      <c r="S481" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T481" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U481" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V481" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W481" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X481" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y481" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z481" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA481" t="inlineStr"/>
+      <c r="AB481" t="inlineStr"/>
+      <c r="AC481" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD481" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE481" t="inlineStr"/>
+      <c r="AF481" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG481" t="inlineStr"/>
+      <c r="AH481" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI481" t="n">
+        <v>19236</v>
+      </c>
+      <c r="AJ481" t="inlineStr">
+        <is>
+          <t>276015</t>
+        </is>
+      </c>
+      <c r="AK481" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL481" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>17413</v>
+      </c>
+      <c r="B482" t="inlineStr"/>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>90****4050</t>
+        </is>
+      </c>
+      <c r="D482" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E482" t="inlineStr"/>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 13:15:08</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr"/>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>*0153</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N482" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O482" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P482" t="n">
+        <v>11000372439451</v>
+      </c>
+      <c r="Q482" t="n">
+        <v>1783928695480</v>
+      </c>
+      <c r="R482" t="n">
+        <v>628026794280</v>
+      </c>
+      <c r="S482" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T482" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U482" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V482" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W482" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X482" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y482" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z482" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA482" t="inlineStr"/>
+      <c r="AB482" t="inlineStr"/>
+      <c r="AC482" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD482" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE482" t="inlineStr"/>
+      <c r="AF482" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG482" t="inlineStr"/>
+      <c r="AH482" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI482" t="n">
+        <v>20153</v>
+      </c>
+      <c r="AJ482" t="inlineStr">
+        <is>
+          <t>269268</t>
+        </is>
+      </c>
+      <c r="AK482" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="AL482" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>16211</v>
+      </c>
+      <c r="B483" t="inlineStr"/>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>95****0840</t>
+        </is>
+      </c>
+      <c r="D483" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E483" t="inlineStr"/>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 15:50:31</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr"/>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>*8814</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N483" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O483" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P483" t="n">
+        <v>11000372485711</v>
+      </c>
+      <c r="Q483" t="n">
+        <v>1783938007306</v>
+      </c>
+      <c r="R483" t="n">
+        <v>523129640767</v>
+      </c>
+      <c r="S483" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T483" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U483" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V483" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W483" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X483" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y483" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z483" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA483" t="inlineStr"/>
+      <c r="AB483" t="inlineStr"/>
+      <c r="AC483" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD483" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE483" t="inlineStr"/>
+      <c r="AF483" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG483" t="inlineStr"/>
+      <c r="AH483" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI483" t="n">
+        <v>18814</v>
+      </c>
+      <c r="AJ483" t="inlineStr">
+        <is>
+          <t>273774</t>
+        </is>
+      </c>
+      <c r="AK483" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL483" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>15367</v>
+      </c>
+      <c r="B484" t="inlineStr"/>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>97****8094</t>
+        </is>
+      </c>
+      <c r="D484" t="n">
+        <v>11600</v>
+      </c>
+      <c r="E484" t="inlineStr"/>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 16:43:37</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr"/>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>*9001</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N484" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O484" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P484" t="n">
+        <v>11000372496635</v>
+      </c>
+      <c r="Q484" t="n">
+        <v>1783941124068</v>
+      </c>
+      <c r="R484" t="n">
+        <v>619444062662</v>
+      </c>
+      <c r="S484" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T484" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U484" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V484" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W484" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X484" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y484" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z484" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA484" t="inlineStr"/>
+      <c r="AB484" t="inlineStr"/>
+      <c r="AC484" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD484" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE484" t="inlineStr"/>
+      <c r="AF484" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG484" t="inlineStr"/>
+      <c r="AH484" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI484" t="n">
+        <v>19001</v>
+      </c>
+      <c r="AJ484" t="inlineStr">
+        <is>
+          <t>275417</t>
+        </is>
+      </c>
+      <c r="AK484" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="AL484" t="inlineStr"/>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>14949</v>
+      </c>
+      <c r="B485" t="inlineStr"/>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>98****7093</t>
+        </is>
+      </c>
+      <c r="D485" t="n">
+        <v>12900</v>
+      </c>
+      <c r="E485" t="inlineStr"/>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 17:06:10</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr"/>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>*9326</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N485" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O485" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P485" t="n">
+        <v>11000372499979</v>
+      </c>
+      <c r="Q485" t="n">
+        <v>1783942555328</v>
+      </c>
+      <c r="R485" t="n">
+        <v>998912050238</v>
+      </c>
+      <c r="S485" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T485" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U485" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V485" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W485" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X485" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y485" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z485" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA485" t="inlineStr"/>
+      <c r="AB485" t="inlineStr"/>
+      <c r="AC485" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD485" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE485" t="inlineStr"/>
+      <c r="AF485" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG485" t="inlineStr"/>
+      <c r="AH485" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI485" t="n">
+        <v>19326</v>
+      </c>
+      <c r="AJ485" t="inlineStr">
+        <is>
+          <t>271103,276017</t>
+        </is>
+      </c>
+      <c r="AK485" t="inlineStr">
+        <is>
+          <t>2075,2096</t>
+        </is>
+      </c>
+      <c r="AL485" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>14576</v>
+      </c>
+      <c r="B486" t="inlineStr"/>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>98****7093</t>
+        </is>
+      </c>
+      <c r="D486" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E486" t="inlineStr"/>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 17:09:58</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr"/>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>*9456</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N486" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O486" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P486" t="n">
+        <v>11000372503211</v>
+      </c>
+      <c r="Q486" t="n">
+        <v>1783942788406</v>
+      </c>
+      <c r="R486" t="n">
+        <v>907449229278</v>
+      </c>
+      <c r="S486" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T486" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U486" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V486" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W486" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X486" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y486" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z486" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA486" t="inlineStr"/>
+      <c r="AB486" t="inlineStr"/>
+      <c r="AC486" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD486" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE486" t="inlineStr"/>
+      <c r="AF486" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG486" t="inlineStr"/>
+      <c r="AH486" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI486" t="n">
+        <v>19456</v>
+      </c>
+      <c r="AJ486" t="inlineStr">
+        <is>
+          <t>276151</t>
+        </is>
+      </c>
+      <c r="AK486" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL486" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>15549</v>
+      </c>
+      <c r="B487" t="inlineStr"/>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>89****0483</t>
+        </is>
+      </c>
+      <c r="D487" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E487" t="inlineStr"/>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 19:47:02</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr"/>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K487" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>*8714</t>
+        </is>
+      </c>
+      <c r="M487" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N487" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O487" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P487" t="n">
+        <v>11000372534162</v>
+      </c>
+      <c r="Q487" t="n">
+        <v>1783952132104</v>
+      </c>
+      <c r="R487" t="n">
+        <v>619435057338</v>
+      </c>
+      <c r="S487" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T487" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U487" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V487" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W487" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X487" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y487" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z487" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA487" t="inlineStr"/>
+      <c r="AB487" t="inlineStr"/>
+      <c r="AC487" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD487" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE487" t="inlineStr"/>
+      <c r="AF487" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG487" t="inlineStr"/>
+      <c r="AH487" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI487" t="n">
+        <v>18714</v>
+      </c>
+      <c r="AJ487" t="inlineStr">
+        <is>
+          <t>273680</t>
+        </is>
+      </c>
+      <c r="AK487" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL487" t="inlineStr"/>
+    </row>
+    <row r="488">
+      <c r="A488" t="n">
+        <v>17678</v>
+      </c>
+      <c r="B488" t="inlineStr"/>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>90****3128</t>
+        </is>
+      </c>
+      <c r="D488" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E488" t="inlineStr"/>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>13-Jul-2026 20:43:31</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr"/>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>*0423</t>
+        </is>
+      </c>
+      <c r="M488" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N488" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O488" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P488" t="n">
+        <v>11000372542814</v>
+      </c>
+      <c r="Q488" t="n">
+        <v>1783955557362</v>
+      </c>
+      <c r="R488" t="n">
+        <v>619433095379</v>
+      </c>
+      <c r="S488" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T488" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U488" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V488" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W488" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X488" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y488" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z488" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA488" t="inlineStr"/>
+      <c r="AB488" t="inlineStr"/>
+      <c r="AC488" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD488" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE488" t="inlineStr"/>
+      <c r="AF488" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG488" t="inlineStr"/>
+      <c r="AH488" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI488" t="n">
+        <v>20423</v>
+      </c>
+      <c r="AJ488" t="inlineStr">
+        <is>
+          <t>277276</t>
+        </is>
+      </c>
+      <c r="AK488" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL488" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Record fee payment for admission 16600
Process online fee payment of ₹8,700 for student admission_no 16600 (RAVI KUMAR RANVITHA PRAYSHITHA SONGA) dated 14-Jul-2026. Updates fee collection records and recalculates outstanding dues from ₹35,400 to ₹26,700.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL488"/>
+  <dimension ref="A1:AL489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76888,6 +76888,152 @@
       </c>
       <c r="AL488" t="inlineStr"/>
     </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>16600</v>
+      </c>
+      <c r="B489" t="inlineStr"/>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>78****9830</t>
+        </is>
+      </c>
+      <c r="D489" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E489" t="inlineStr"/>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 06:24:44</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr"/>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>*8417</t>
+        </is>
+      </c>
+      <c r="M489" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N489" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O489" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P489" t="n">
+        <v>11000372581514</v>
+      </c>
+      <c r="Q489" t="n">
+        <v>1783990473035</v>
+      </c>
+      <c r="R489" t="n">
+        <v>744464417704</v>
+      </c>
+      <c r="S489" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T489" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U489" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V489" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W489" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X489" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y489" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z489" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA489" t="inlineStr"/>
+      <c r="AB489" t="inlineStr"/>
+      <c r="AC489" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD489" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE489" t="inlineStr"/>
+      <c r="AF489" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG489" t="inlineStr"/>
+      <c r="AH489" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI489" t="n">
+        <v>18417</v>
+      </c>
+      <c r="AJ489" t="inlineStr">
+        <is>
+          <t>272464</t>
+        </is>
+      </c>
+      <c r="AK489" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL489" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update fee collection records and payment status
Update fee payment records across multiple data files including atom payment reports, daywise and overall fees collection, and student records. Changes include updating payment amounts, settlement dates for cleared transactions, and correcting student phone numbers where needed. Consolidates fee collection data from July 13-15, 2026.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL489"/>
+  <dimension ref="A1:AL507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75453,7 +75453,9 @@
       <c r="D479" t="n">
         <v>12300</v>
       </c>
-      <c r="E479" t="inlineStr"/>
+      <c r="E479" t="n">
+        <v>12300</v>
+      </c>
       <c r="F479" t="inlineStr">
         <is>
           <t>13-Jul-2026 08:43:44</t>
@@ -75524,7 +75526,7 @@
       </c>
       <c r="V479" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W479" t="inlineStr">
@@ -75547,15 +75549,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA479" t="inlineStr"/>
-      <c r="AB479" t="inlineStr"/>
+      <c r="AA479" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB479" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC479" t="n">
         <v>0</v>
       </c>
       <c r="AD479" t="n">
         <v>0</v>
       </c>
-      <c r="AE479" t="inlineStr"/>
+      <c r="AE479" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF479" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -75599,13 +75607,19 @@
       <c r="D480" t="n">
         <v>9000</v>
       </c>
-      <c r="E480" t="inlineStr"/>
+      <c r="E480" t="n">
+        <v>9000</v>
+      </c>
       <c r="F480" t="inlineStr">
         <is>
           <t>13-Jul-2026 08:50:31</t>
         </is>
       </c>
-      <c r="G480" t="inlineStr"/>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 18:54:43</t>
+        </is>
+      </c>
       <c r="H480" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -75670,7 +75684,7 @@
       </c>
       <c r="V480" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W480" t="inlineStr">
@@ -75693,15 +75707,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA480" t="inlineStr"/>
-      <c r="AB480" t="inlineStr"/>
+      <c r="AA480" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB480" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC480" t="n">
         <v>0</v>
       </c>
       <c r="AD480" t="n">
         <v>0</v>
       </c>
-      <c r="AE480" t="inlineStr"/>
+      <c r="AE480" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF480" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -75745,7 +75765,9 @@
       <c r="D481" t="n">
         <v>12300</v>
       </c>
-      <c r="E481" t="inlineStr"/>
+      <c r="E481" t="n">
+        <v>12300</v>
+      </c>
       <c r="F481" t="inlineStr">
         <is>
           <t>13-Jul-2026 09:46:23</t>
@@ -75816,7 +75838,7 @@
       </c>
       <c r="V481" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W481" t="inlineStr">
@@ -75839,15 +75861,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA481" t="inlineStr"/>
-      <c r="AB481" t="inlineStr"/>
+      <c r="AA481" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB481" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC481" t="n">
         <v>0</v>
       </c>
       <c r="AD481" t="n">
         <v>0</v>
       </c>
-      <c r="AE481" t="inlineStr"/>
+      <c r="AE481" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF481" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -75891,13 +75919,19 @@
       <c r="D482" t="n">
         <v>7250</v>
       </c>
-      <c r="E482" t="inlineStr"/>
+      <c r="E482" t="n">
+        <v>7250</v>
+      </c>
       <c r="F482" t="inlineStr">
         <is>
           <t>13-Jul-2026 13:15:08</t>
         </is>
       </c>
-      <c r="G482" t="inlineStr"/>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 18:54:43</t>
+        </is>
+      </c>
       <c r="H482" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -75962,7 +75996,7 @@
       </c>
       <c r="V482" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W482" t="inlineStr">
@@ -75985,15 +76019,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA482" t="inlineStr"/>
-      <c r="AB482" t="inlineStr"/>
+      <c r="AA482" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB482" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC482" t="n">
         <v>0</v>
       </c>
       <c r="AD482" t="n">
         <v>0</v>
       </c>
-      <c r="AE482" t="inlineStr"/>
+      <c r="AE482" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF482" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
@@ -76037,13 +76077,19 @@
       <c r="D483" t="n">
         <v>9000</v>
       </c>
-      <c r="E483" t="inlineStr"/>
+      <c r="E483" t="n">
+        <v>9000</v>
+      </c>
       <c r="F483" t="inlineStr">
         <is>
           <t>13-Jul-2026 15:50:31</t>
         </is>
       </c>
-      <c r="G483" t="inlineStr"/>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 18:54:43</t>
+        </is>
+      </c>
       <c r="H483" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -76108,7 +76154,7 @@
       </c>
       <c r="V483" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W483" t="inlineStr">
@@ -76131,15 +76177,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA483" t="inlineStr"/>
-      <c r="AB483" t="inlineStr"/>
+      <c r="AA483" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB483" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC483" t="n">
         <v>0</v>
       </c>
       <c r="AD483" t="n">
         <v>0</v>
       </c>
-      <c r="AE483" t="inlineStr"/>
+      <c r="AE483" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF483" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -76183,7 +76235,9 @@
       <c r="D484" t="n">
         <v>11600</v>
       </c>
-      <c r="E484" t="inlineStr"/>
+      <c r="E484" t="n">
+        <v>11600</v>
+      </c>
       <c r="F484" t="inlineStr">
         <is>
           <t>13-Jul-2026 16:43:37</t>
@@ -76254,7 +76308,7 @@
       </c>
       <c r="V484" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W484" t="inlineStr">
@@ -76277,15 +76331,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA484" t="inlineStr"/>
-      <c r="AB484" t="inlineStr"/>
+      <c r="AA484" t="n">
+        <v>139.2</v>
+      </c>
+      <c r="AB484" t="n">
+        <v>25.06</v>
+      </c>
       <c r="AC484" t="n">
         <v>0</v>
       </c>
       <c r="AD484" t="n">
         <v>0</v>
       </c>
-      <c r="AE484" t="inlineStr"/>
+      <c r="AE484" t="n">
+        <v>164.26</v>
+      </c>
       <c r="AF484" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -76325,7 +76385,9 @@
       <c r="D485" t="n">
         <v>12900</v>
       </c>
-      <c r="E485" t="inlineStr"/>
+      <c r="E485" t="n">
+        <v>12900</v>
+      </c>
       <c r="F485" t="inlineStr">
         <is>
           <t>13-Jul-2026 17:06:10</t>
@@ -76396,7 +76458,7 @@
       </c>
       <c r="V485" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W485" t="inlineStr">
@@ -76419,15 +76481,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA485" t="inlineStr"/>
-      <c r="AB485" t="inlineStr"/>
+      <c r="AA485" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB485" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC485" t="n">
         <v>0</v>
       </c>
       <c r="AD485" t="n">
         <v>0</v>
       </c>
-      <c r="AE485" t="inlineStr"/>
+      <c r="AE485" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF485" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -76471,7 +76539,9 @@
       <c r="D486" t="n">
         <v>12300</v>
       </c>
-      <c r="E486" t="inlineStr"/>
+      <c r="E486" t="n">
+        <v>12300</v>
+      </c>
       <c r="F486" t="inlineStr">
         <is>
           <t>13-Jul-2026 17:09:58</t>
@@ -76542,7 +76612,7 @@
       </c>
       <c r="V486" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W486" t="inlineStr">
@@ -76565,15 +76635,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA486" t="inlineStr"/>
-      <c r="AB486" t="inlineStr"/>
+      <c r="AA486" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB486" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC486" t="n">
         <v>0</v>
       </c>
       <c r="AD486" t="n">
         <v>0</v>
       </c>
-      <c r="AE486" t="inlineStr"/>
+      <c r="AE486" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF486" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -76617,13 +76693,19 @@
       <c r="D487" t="n">
         <v>9000</v>
       </c>
-      <c r="E487" t="inlineStr"/>
+      <c r="E487" t="n">
+        <v>9000</v>
+      </c>
       <c r="F487" t="inlineStr">
         <is>
           <t>13-Jul-2026 19:47:02</t>
         </is>
       </c>
-      <c r="G487" t="inlineStr"/>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 18:54:43</t>
+        </is>
+      </c>
       <c r="H487" t="inlineStr">
         <is>
           <t>SUCCESS</t>
@@ -76688,7 +76770,7 @@
       </c>
       <c r="V487" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W487" t="inlineStr">
@@ -76711,15 +76793,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA487" t="inlineStr"/>
-      <c r="AB487" t="inlineStr"/>
+      <c r="AA487" t="n">
+        <v>108</v>
+      </c>
+      <c r="AB487" t="n">
+        <v>19.44</v>
+      </c>
       <c r="AC487" t="n">
         <v>0</v>
       </c>
       <c r="AD487" t="n">
         <v>0</v>
       </c>
-      <c r="AE487" t="inlineStr"/>
+      <c r="AE487" t="n">
+        <v>127.44</v>
+      </c>
       <c r="AF487" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -76759,13 +76847,19 @@
       <c r="D488" t="n">
         <v>8400</v>
       </c>
-      <c r="E488" t="inlineStr"/>
+      <c r="E488" t="n">
+        <v>8400</v>
+      </c>
       <c r="F488" t="inlineStr">
         <is>
           <t>13-Jul-2026 20:43:31</t>
         </is>
       </c>
-      <c r="G488" t="inlineStr"/>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 18:54:43</t>
+        </is>
+      </c>
       <c r="H488" t="inlineStr">
         <is>
           <t>SUCCESS</t>
@@ -76830,7 +76924,7 @@
       </c>
       <c r="V488" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W488" t="inlineStr">
@@ -76853,15 +76947,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA488" t="inlineStr"/>
-      <c r="AB488" t="inlineStr"/>
+      <c r="AA488" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="AB488" t="n">
+        <v>20.41</v>
+      </c>
       <c r="AC488" t="n">
         <v>0</v>
       </c>
       <c r="AD488" t="n">
         <v>0</v>
       </c>
-      <c r="AE488" t="inlineStr"/>
+      <c r="AE488" t="n">
+        <v>133.81</v>
+      </c>
       <c r="AF488" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -77034,6 +77134,2626 @@
         </is>
       </c>
     </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>16210</v>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>V********** H****** K****</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>81****1333</t>
+        </is>
+      </c>
+      <c r="D490" t="n">
+        <v>11600</v>
+      </c>
+      <c r="E490" t="inlineStr"/>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 08:19:45</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr"/>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>eleven thousand six hundred</t>
+        </is>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>********6600</t>
+        </is>
+      </c>
+      <c r="M490" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N490" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O490" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="P490" t="n">
+        <v>11000372592904</v>
+      </c>
+      <c r="Q490" t="n">
+        <v>1783997365</v>
+      </c>
+      <c r="R490" t="n">
+        <v>970216478702</v>
+      </c>
+      <c r="S490" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T490" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U490" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V490" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W490" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X490" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y490" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z490" t="inlineStr">
+        <is>
+          <t>k*************@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA490" t="inlineStr"/>
+      <c r="AB490" t="inlineStr"/>
+      <c r="AC490" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD490" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE490" t="inlineStr"/>
+      <c r="AF490" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG490" t="inlineStr"/>
+      <c r="AH490" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI490" t="n">
+        <v>19051</v>
+      </c>
+      <c r="AJ490" t="inlineStr">
+        <is>
+          <t>275475</t>
+        </is>
+      </c>
+      <c r="AK490" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="AL490" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>16754</v>
+      </c>
+      <c r="B491" t="inlineStr"/>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>79****7118</t>
+        </is>
+      </c>
+      <c r="D491" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E491" t="inlineStr"/>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 08:32:00</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr"/>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K491" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>*8267</t>
+        </is>
+      </c>
+      <c r="M491" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N491" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O491" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P491" t="n">
+        <v>11000372593846</v>
+      </c>
+      <c r="Q491" t="n">
+        <v>1783998111697</v>
+      </c>
+      <c r="R491" t="n">
+        <v>656134982093</v>
+      </c>
+      <c r="S491" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T491" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U491" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V491" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W491" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X491" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y491" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z491" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA491" t="inlineStr"/>
+      <c r="AB491" t="inlineStr"/>
+      <c r="AC491" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD491" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE491" t="inlineStr"/>
+      <c r="AF491" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG491" t="inlineStr"/>
+      <c r="AH491" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI491" t="n">
+        <v>18267</v>
+      </c>
+      <c r="AJ491" t="inlineStr">
+        <is>
+          <t>272264</t>
+        </is>
+      </c>
+      <c r="AK491" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL491" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>17474</v>
+      </c>
+      <c r="B492" t="inlineStr"/>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>95****0855</t>
+        </is>
+      </c>
+      <c r="D492" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E492" t="inlineStr"/>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 08:55:10</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr"/>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>*0440</t>
+        </is>
+      </c>
+      <c r="M492" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N492" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O492" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P492" t="n">
+        <v>11000372597439</v>
+      </c>
+      <c r="Q492" t="n">
+        <v>1783999483660</v>
+      </c>
+      <c r="R492" t="n">
+        <v>163139316836</v>
+      </c>
+      <c r="S492" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T492" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U492" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V492" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W492" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X492" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y492" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z492" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA492" t="inlineStr"/>
+      <c r="AB492" t="inlineStr"/>
+      <c r="AC492" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD492" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE492" t="inlineStr"/>
+      <c r="AF492" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG492" t="inlineStr"/>
+      <c r="AH492" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI492" t="n">
+        <v>20440</v>
+      </c>
+      <c r="AJ492" t="inlineStr">
+        <is>
+          <t>277500</t>
+        </is>
+      </c>
+      <c r="AK492" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL492" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>17635</v>
+      </c>
+      <c r="B493" t="inlineStr"/>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>95****1386</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>9300</v>
+      </c>
+      <c r="E493" t="inlineStr"/>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 09:17:53</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr"/>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>*0439</t>
+        </is>
+      </c>
+      <c r="M493" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N493" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O493" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P493" t="n">
+        <v>11000372602280</v>
+      </c>
+      <c r="Q493" t="n">
+        <v>1784000839883</v>
+      </c>
+      <c r="R493" t="n">
+        <v>586045885504</v>
+      </c>
+      <c r="S493" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T493" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U493" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V493" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W493" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X493" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y493" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z493" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA493" t="inlineStr"/>
+      <c r="AB493" t="inlineStr"/>
+      <c r="AC493" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD493" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE493" t="inlineStr"/>
+      <c r="AF493" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG493" t="inlineStr"/>
+      <c r="AH493" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI493" t="n">
+        <v>20439</v>
+      </c>
+      <c r="AJ493" t="inlineStr">
+        <is>
+          <t>277157,277158</t>
+        </is>
+      </c>
+      <c r="AK493" t="inlineStr">
+        <is>
+          <t>2067,2080</t>
+        </is>
+      </c>
+      <c r="AL493" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>15946</v>
+      </c>
+      <c r="B494" t="inlineStr"/>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>99****3270</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>600</v>
+      </c>
+      <c r="E494" t="inlineStr"/>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 10:38:53</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr"/>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>*8582</t>
+        </is>
+      </c>
+      <c r="M494" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N494" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O494" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P494" t="n">
+        <v>11000372621189</v>
+      </c>
+      <c r="Q494" t="n">
+        <v>1784005658818</v>
+      </c>
+      <c r="R494" t="n">
+        <v>279854132977</v>
+      </c>
+      <c r="S494" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T494" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U494" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V494" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W494" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X494" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y494" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z494" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA494" t="inlineStr"/>
+      <c r="AB494" t="inlineStr"/>
+      <c r="AC494" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD494" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE494" t="inlineStr"/>
+      <c r="AF494" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG494" t="inlineStr"/>
+      <c r="AH494" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI494" t="n">
+        <v>18582</v>
+      </c>
+      <c r="AJ494" t="inlineStr">
+        <is>
+          <t>270376</t>
+        </is>
+      </c>
+      <c r="AK494" t="inlineStr">
+        <is>
+          <t>2067</t>
+        </is>
+      </c>
+      <c r="AL494" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>14595</v>
+      </c>
+      <c r="B495" t="inlineStr"/>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>97****3026</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E495" t="inlineStr"/>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 12:01:07</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr"/>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>*9376</t>
+        </is>
+      </c>
+      <c r="M495" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N495" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O495" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P495" t="n">
+        <v>11000372647475</v>
+      </c>
+      <c r="Q495" t="n">
+        <v>1784010645253</v>
+      </c>
+      <c r="R495" t="n">
+        <v>303738269768</v>
+      </c>
+      <c r="S495" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T495" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U495" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V495" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W495" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X495" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y495" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z495" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA495" t="inlineStr"/>
+      <c r="AB495" t="inlineStr"/>
+      <c r="AC495" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD495" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE495" t="inlineStr"/>
+      <c r="AF495" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG495" t="inlineStr"/>
+      <c r="AH495" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI495" t="n">
+        <v>19376</v>
+      </c>
+      <c r="AJ495" t="inlineStr">
+        <is>
+          <t>276103</t>
+        </is>
+      </c>
+      <c r="AK495" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL495" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>14972</v>
+      </c>
+      <c r="B496" t="inlineStr"/>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>97****3026</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E496" t="inlineStr"/>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 12:07:44</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr"/>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>*9310</t>
+        </is>
+      </c>
+      <c r="M496" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N496" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O496" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P496" t="n">
+        <v>11000372651223</v>
+      </c>
+      <c r="Q496" t="n">
+        <v>1784011047137</v>
+      </c>
+      <c r="R496" t="n">
+        <v>442912257699</v>
+      </c>
+      <c r="S496" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T496" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U496" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V496" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W496" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X496" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y496" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z496" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA496" t="inlineStr"/>
+      <c r="AB496" t="inlineStr"/>
+      <c r="AC496" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD496" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE496" t="inlineStr"/>
+      <c r="AF496" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG496" t="inlineStr"/>
+      <c r="AH496" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI496" t="n">
+        <v>19310</v>
+      </c>
+      <c r="AJ496" t="inlineStr">
+        <is>
+          <t>276056</t>
+        </is>
+      </c>
+      <c r="AK496" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL496" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>16308</v>
+      </c>
+      <c r="B497" t="inlineStr"/>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>88****7880</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E497" t="inlineStr"/>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 15:58:15</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr"/>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>*8443</t>
+        </is>
+      </c>
+      <c r="M497" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N497" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O497" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P497" t="n">
+        <v>11000372709836</v>
+      </c>
+      <c r="Q497" t="n">
+        <v>1784024636491</v>
+      </c>
+      <c r="R497" t="n">
+        <v>619545045871</v>
+      </c>
+      <c r="S497" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T497" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U497" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V497" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W497" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X497" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y497" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z497" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA497" t="inlineStr"/>
+      <c r="AB497" t="inlineStr"/>
+      <c r="AC497" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD497" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE497" t="inlineStr"/>
+      <c r="AF497" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG497" t="inlineStr"/>
+      <c r="AH497" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI497" t="n">
+        <v>18443</v>
+      </c>
+      <c r="AJ497" t="inlineStr">
+        <is>
+          <t>272490</t>
+        </is>
+      </c>
+      <c r="AK497" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL497" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>16636</v>
+      </c>
+      <c r="B498" t="inlineStr"/>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>88****7880</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E498" t="inlineStr"/>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 16:01:05</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr"/>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>*8297</t>
+        </is>
+      </c>
+      <c r="M498" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N498" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O498" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P498" t="n">
+        <v>11000372711014</v>
+      </c>
+      <c r="Q498" t="n">
+        <v>1784024987288</v>
+      </c>
+      <c r="R498" t="n">
+        <v>619533061786</v>
+      </c>
+      <c r="S498" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T498" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U498" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V498" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W498" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X498" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y498" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z498" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA498" t="inlineStr"/>
+      <c r="AB498" t="inlineStr"/>
+      <c r="AC498" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD498" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE498" t="inlineStr"/>
+      <c r="AF498" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG498" t="inlineStr"/>
+      <c r="AH498" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI498" t="n">
+        <v>18297</v>
+      </c>
+      <c r="AJ498" t="inlineStr">
+        <is>
+          <t>272276</t>
+        </is>
+      </c>
+      <c r="AK498" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL498" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" t="n">
+        <v>16946</v>
+      </c>
+      <c r="B499" t="inlineStr"/>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>97****7601</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E499" t="inlineStr"/>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 17:52:35</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr"/>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>*8263</t>
+        </is>
+      </c>
+      <c r="M499" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N499" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O499" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P499" t="n">
+        <v>11000372732102</v>
+      </c>
+      <c r="Q499" t="n">
+        <v>1784031726449</v>
+      </c>
+      <c r="R499" t="n">
+        <v>621816203512</v>
+      </c>
+      <c r="S499" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T499" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U499" t="inlineStr">
+        <is>
+          <t>HDFC BANK UPI</t>
+        </is>
+      </c>
+      <c r="V499" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W499" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X499" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y499" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z499" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA499" t="inlineStr"/>
+      <c r="AB499" t="inlineStr"/>
+      <c r="AC499" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD499" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE499" t="inlineStr"/>
+      <c r="AF499" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG499" t="inlineStr"/>
+      <c r="AH499" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI499" t="n">
+        <v>18263</v>
+      </c>
+      <c r="AJ499" t="inlineStr">
+        <is>
+          <t>272310</t>
+        </is>
+      </c>
+      <c r="AK499" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL499" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="n">
+        <v>17259</v>
+      </c>
+      <c r="B500" t="inlineStr"/>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>63****1566</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E500" t="inlineStr"/>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 18:40:49</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr"/>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>*9971</t>
+        </is>
+      </c>
+      <c r="M500" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N500" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O500" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P500" t="n">
+        <v>11000372738767</v>
+      </c>
+      <c r="Q500" t="n">
+        <v>1784034633473</v>
+      </c>
+      <c r="R500" t="n">
+        <v>619572737176</v>
+      </c>
+      <c r="S500" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T500" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U500" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V500" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W500" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X500" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y500" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z500" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA500" t="inlineStr"/>
+      <c r="AB500" t="inlineStr"/>
+      <c r="AC500" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD500" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE500" t="inlineStr"/>
+      <c r="AF500" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG500" t="inlineStr"/>
+      <c r="AH500" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI500" t="n">
+        <v>19971</v>
+      </c>
+      <c r="AJ500" t="inlineStr">
+        <is>
+          <t>276072</t>
+        </is>
+      </c>
+      <c r="AK500" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL500" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="n">
+        <v>17260</v>
+      </c>
+      <c r="B501" t="inlineStr"/>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>63****1566</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E501" t="inlineStr"/>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 18:43:00</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr"/>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>*9972</t>
+        </is>
+      </c>
+      <c r="M501" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N501" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O501" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P501" t="n">
+        <v>11000372739801</v>
+      </c>
+      <c r="Q501" t="n">
+        <v>1784034760455</v>
+      </c>
+      <c r="R501" t="n">
+        <v>619535244605</v>
+      </c>
+      <c r="S501" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T501" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U501" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V501" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W501" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X501" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y501" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z501" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA501" t="inlineStr"/>
+      <c r="AB501" t="inlineStr"/>
+      <c r="AC501" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD501" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE501" t="inlineStr"/>
+      <c r="AF501" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG501" t="inlineStr"/>
+      <c r="AH501" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI501" t="n">
+        <v>19972</v>
+      </c>
+      <c r="AJ501" t="inlineStr">
+        <is>
+          <t>273787</t>
+        </is>
+      </c>
+      <c r="AK501" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL501" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="n">
+        <v>17305</v>
+      </c>
+      <c r="B502" t="inlineStr"/>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>70****3690</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E502" t="inlineStr"/>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 19:25:25</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr"/>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>*0014</t>
+        </is>
+      </c>
+      <c r="M502" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N502" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O502" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P502" t="n">
+        <v>11000372748134</v>
+      </c>
+      <c r="Q502" t="n">
+        <v>1784037291694</v>
+      </c>
+      <c r="R502" t="n">
+        <v>619523487211</v>
+      </c>
+      <c r="S502" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T502" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U502" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V502" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W502" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X502" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y502" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z502" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA502" t="inlineStr"/>
+      <c r="AB502" t="inlineStr"/>
+      <c r="AC502" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD502" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE502" t="inlineStr"/>
+      <c r="AF502" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG502" t="inlineStr"/>
+      <c r="AH502" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI502" t="n">
+        <v>20014</v>
+      </c>
+      <c r="AJ502" t="inlineStr">
+        <is>
+          <t>269340</t>
+        </is>
+      </c>
+      <c r="AK502" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="AL502" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="n">
+        <v>16184</v>
+      </c>
+      <c r="B503" t="inlineStr"/>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>98****4994</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E503" t="inlineStr"/>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 21:50:45</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr"/>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>*8643</t>
+        </is>
+      </c>
+      <c r="M503" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N503" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O503" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P503" t="n">
+        <v>11000372774187</v>
+      </c>
+      <c r="Q503" t="n">
+        <v>1784045939391</v>
+      </c>
+      <c r="R503" t="n">
+        <v>619526086181</v>
+      </c>
+      <c r="S503" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T503" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U503" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V503" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W503" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X503" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y503" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z503" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA503" t="inlineStr"/>
+      <c r="AB503" t="inlineStr"/>
+      <c r="AC503" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD503" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE503" t="inlineStr"/>
+      <c r="AF503" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG503" t="inlineStr"/>
+      <c r="AH503" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI503" t="n">
+        <v>18643</v>
+      </c>
+      <c r="AJ503" t="inlineStr">
+        <is>
+          <t>273525</t>
+        </is>
+      </c>
+      <c r="AK503" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL503" t="inlineStr"/>
+    </row>
+    <row r="504">
+      <c r="A504" t="n">
+        <v>17139</v>
+      </c>
+      <c r="B504" t="inlineStr"/>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>79****8688</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E504" t="inlineStr"/>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 22:23:39</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr"/>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>*9842</t>
+        </is>
+      </c>
+      <c r="M504" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N504" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O504" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P504" t="n">
+        <v>11000372787749</v>
+      </c>
+      <c r="Q504" t="n">
+        <v>1784047981963</v>
+      </c>
+      <c r="R504" t="n">
+        <v>619566785107</v>
+      </c>
+      <c r="S504" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T504" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U504" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V504" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W504" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X504" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y504" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z504" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA504" t="inlineStr"/>
+      <c r="AB504" t="inlineStr"/>
+      <c r="AC504" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD504" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE504" t="inlineStr"/>
+      <c r="AF504" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG504" t="inlineStr"/>
+      <c r="AH504" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI504" t="n">
+        <v>19842</v>
+      </c>
+      <c r="AJ504" t="inlineStr">
+        <is>
+          <t>273716</t>
+        </is>
+      </c>
+      <c r="AK504" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL504" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="n">
+        <v>17138</v>
+      </c>
+      <c r="B505" t="inlineStr"/>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>79****8688</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E505" t="inlineStr"/>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 22:25:50</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr"/>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESS</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K505" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>*9841</t>
+        </is>
+      </c>
+      <c r="M505" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N505" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O505" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P505" t="n">
+        <v>11000372788739</v>
+      </c>
+      <c r="Q505" t="n">
+        <v>1784048132165</v>
+      </c>
+      <c r="R505" t="n">
+        <v>126301595397</v>
+      </c>
+      <c r="S505" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T505" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U505" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V505" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W505" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X505" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y505" t="inlineStr">
+        <is>
+          <t>QR_UPI</t>
+        </is>
+      </c>
+      <c r="Z505" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA505" t="inlineStr"/>
+      <c r="AB505" t="inlineStr"/>
+      <c r="AC505" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD505" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE505" t="inlineStr"/>
+      <c r="AF505" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG505" t="inlineStr"/>
+      <c r="AH505" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI505" t="n">
+        <v>19841</v>
+      </c>
+      <c r="AJ505" t="inlineStr">
+        <is>
+          <t>272388</t>
+        </is>
+      </c>
+      <c r="AK505" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL505" t="inlineStr">
+        <is>
+          <t>PG QR</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="n">
+        <v>16056</v>
+      </c>
+      <c r="B506" t="inlineStr"/>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>63****9147</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>11600</v>
+      </c>
+      <c r="E506" t="inlineStr"/>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>14-Jul-2026 23:02:15</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr"/>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>*9023</t>
+        </is>
+      </c>
+      <c r="M506" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N506" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O506" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P506" t="n">
+        <v>11000372794165</v>
+      </c>
+      <c r="Q506" t="n">
+        <v>1784050323852</v>
+      </c>
+      <c r="R506" t="n">
+        <v>207509877173</v>
+      </c>
+      <c r="S506" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T506" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U506" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V506" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W506" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X506" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y506" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z506" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA506" t="inlineStr"/>
+      <c r="AB506" t="inlineStr"/>
+      <c r="AC506" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD506" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE506" t="inlineStr"/>
+      <c r="AF506" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG506" t="inlineStr"/>
+      <c r="AH506" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI506" t="n">
+        <v>19023</v>
+      </c>
+      <c r="AJ506" t="inlineStr">
+        <is>
+          <t>275357</t>
+        </is>
+      </c>
+      <c r="AK506" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="AL506" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="n">
+        <v>15011</v>
+      </c>
+      <c r="B507" t="inlineStr"/>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>99****2276</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E507" t="inlineStr"/>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 06:38:13</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr"/>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K507" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>*9283</t>
+        </is>
+      </c>
+      <c r="M507" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N507" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O507" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P507" t="n">
+        <v>11000372803936</v>
+      </c>
+      <c r="Q507" t="n">
+        <v>1784077528625</v>
+      </c>
+      <c r="R507" t="n">
+        <v>82502943802</v>
+      </c>
+      <c r="S507" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T507" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U507" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V507" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W507" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X507" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y507" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z507" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA507" t="inlineStr"/>
+      <c r="AB507" t="inlineStr"/>
+      <c r="AC507" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD507" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE507" t="inlineStr"/>
+      <c r="AF507" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG507" t="inlineStr"/>
+      <c r="AH507" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI507" t="n">
+        <v>19283</v>
+      </c>
+      <c r="AJ507" t="inlineStr">
+        <is>
+          <t>276023</t>
+        </is>
+      </c>
+      <c r="AK507" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL507" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update transaction records and fee collection data
Filled missing settlement dates and net amounts in atom_report_cleaned records. Added ~153 new fee transactions to fee_transcation_atom_report. Updated student fee collection status across multiple date ranges. Corrected student names and father names in student records. Jupyter notebook kernel metadata updated.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL507"/>
+  <dimension ref="A1:AL522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77001,13 +77001,19 @@
       <c r="D489" t="n">
         <v>8700</v>
       </c>
-      <c r="E489" t="inlineStr"/>
+      <c r="E489" t="n">
+        <v>8700</v>
+      </c>
       <c r="F489" t="inlineStr">
         <is>
           <t>14-Jul-2026 06:24:44</t>
         </is>
       </c>
-      <c r="G489" t="inlineStr"/>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H489" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -77072,7 +77078,7 @@
       </c>
       <c r="V489" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W489" t="inlineStr">
@@ -77095,15 +77101,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA489" t="inlineStr"/>
-      <c r="AB489" t="inlineStr"/>
+      <c r="AA489" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB489" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC489" t="n">
         <v>0</v>
       </c>
       <c r="AD489" t="n">
         <v>0</v>
       </c>
-      <c r="AE489" t="inlineStr"/>
+      <c r="AE489" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF489" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -77151,7 +77163,9 @@
       <c r="D490" t="n">
         <v>11600</v>
       </c>
-      <c r="E490" t="inlineStr"/>
+      <c r="E490" t="n">
+        <v>11600</v>
+      </c>
       <c r="F490" t="inlineStr">
         <is>
           <t>14-Jul-2026 08:19:45</t>
@@ -77222,7 +77236,7 @@
       </c>
       <c r="V490" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W490" t="inlineStr">
@@ -77245,15 +77259,21 @@
           <t>k*************@gmail.com</t>
         </is>
       </c>
-      <c r="AA490" t="inlineStr"/>
-      <c r="AB490" t="inlineStr"/>
+      <c r="AA490" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB490" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC490" t="n">
         <v>0</v>
       </c>
       <c r="AD490" t="n">
         <v>0</v>
       </c>
-      <c r="AE490" t="inlineStr"/>
+      <c r="AE490" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF490" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -77297,13 +77317,19 @@
       <c r="D491" t="n">
         <v>8700</v>
       </c>
-      <c r="E491" t="inlineStr"/>
+      <c r="E491" t="n">
+        <v>8700</v>
+      </c>
       <c r="F491" t="inlineStr">
         <is>
           <t>14-Jul-2026 08:32:00</t>
         </is>
       </c>
-      <c r="G491" t="inlineStr"/>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H491" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -77368,7 +77394,7 @@
       </c>
       <c r="V491" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W491" t="inlineStr">
@@ -77391,15 +77417,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA491" t="inlineStr"/>
-      <c r="AB491" t="inlineStr"/>
+      <c r="AA491" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB491" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC491" t="n">
         <v>0</v>
       </c>
       <c r="AD491" t="n">
         <v>0</v>
       </c>
-      <c r="AE491" t="inlineStr"/>
+      <c r="AE491" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF491" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -77443,13 +77475,19 @@
       <c r="D492" t="n">
         <v>9000</v>
       </c>
-      <c r="E492" t="inlineStr"/>
+      <c r="E492" t="n">
+        <v>9000</v>
+      </c>
       <c r="F492" t="inlineStr">
         <is>
           <t>14-Jul-2026 08:55:10</t>
         </is>
       </c>
-      <c r="G492" t="inlineStr"/>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H492" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -77514,7 +77552,7 @@
       </c>
       <c r="V492" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W492" t="inlineStr">
@@ -77537,15 +77575,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA492" t="inlineStr"/>
-      <c r="AB492" t="inlineStr"/>
+      <c r="AA492" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB492" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC492" t="n">
         <v>0</v>
       </c>
       <c r="AD492" t="n">
         <v>0</v>
       </c>
-      <c r="AE492" t="inlineStr"/>
+      <c r="AE492" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF492" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -77589,13 +77633,19 @@
       <c r="D493" t="n">
         <v>9300</v>
       </c>
-      <c r="E493" t="inlineStr"/>
+      <c r="E493" t="n">
+        <v>9300</v>
+      </c>
       <c r="F493" t="inlineStr">
         <is>
           <t>14-Jul-2026 09:17:53</t>
         </is>
       </c>
-      <c r="G493" t="inlineStr"/>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H493" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -77660,7 +77710,7 @@
       </c>
       <c r="V493" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W493" t="inlineStr">
@@ -77683,15 +77733,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA493" t="inlineStr"/>
-      <c r="AB493" t="inlineStr"/>
+      <c r="AA493" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB493" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC493" t="n">
         <v>0</v>
       </c>
       <c r="AD493" t="n">
         <v>0</v>
       </c>
-      <c r="AE493" t="inlineStr"/>
+      <c r="AE493" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF493" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -77735,13 +77791,19 @@
       <c r="D494" t="n">
         <v>600</v>
       </c>
-      <c r="E494" t="inlineStr"/>
+      <c r="E494" t="n">
+        <v>600</v>
+      </c>
       <c r="F494" t="inlineStr">
         <is>
           <t>14-Jul-2026 10:38:53</t>
         </is>
       </c>
-      <c r="G494" t="inlineStr"/>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H494" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -77806,7 +77868,7 @@
       </c>
       <c r="V494" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W494" t="inlineStr">
@@ -77829,15 +77891,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA494" t="inlineStr"/>
-      <c r="AB494" t="inlineStr"/>
+      <c r="AA494" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB494" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC494" t="n">
         <v>0</v>
       </c>
       <c r="AD494" t="n">
         <v>0</v>
       </c>
-      <c r="AE494" t="inlineStr"/>
+      <c r="AE494" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF494" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -77881,7 +77949,9 @@
       <c r="D495" t="n">
         <v>12300</v>
       </c>
-      <c r="E495" t="inlineStr"/>
+      <c r="E495" t="n">
+        <v>12300</v>
+      </c>
       <c r="F495" t="inlineStr">
         <is>
           <t>14-Jul-2026 12:01:07</t>
@@ -77952,7 +78022,7 @@
       </c>
       <c r="V495" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W495" t="inlineStr">
@@ -77975,15 +78045,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA495" t="inlineStr"/>
-      <c r="AB495" t="inlineStr"/>
+      <c r="AA495" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB495" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC495" t="n">
         <v>0</v>
       </c>
       <c r="AD495" t="n">
         <v>0</v>
       </c>
-      <c r="AE495" t="inlineStr"/>
+      <c r="AE495" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF495" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -78027,7 +78103,9 @@
       <c r="D496" t="n">
         <v>12300</v>
       </c>
-      <c r="E496" t="inlineStr"/>
+      <c r="E496" t="n">
+        <v>12300</v>
+      </c>
       <c r="F496" t="inlineStr">
         <is>
           <t>14-Jul-2026 12:07:44</t>
@@ -78098,7 +78176,7 @@
       </c>
       <c r="V496" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W496" t="inlineStr">
@@ -78121,15 +78199,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA496" t="inlineStr"/>
-      <c r="AB496" t="inlineStr"/>
+      <c r="AA496" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB496" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC496" t="n">
         <v>0</v>
       </c>
       <c r="AD496" t="n">
         <v>0</v>
       </c>
-      <c r="AE496" t="inlineStr"/>
+      <c r="AE496" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF496" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -78173,13 +78257,19 @@
       <c r="D497" t="n">
         <v>8700</v>
       </c>
-      <c r="E497" t="inlineStr"/>
+      <c r="E497" t="n">
+        <v>8700</v>
+      </c>
       <c r="F497" t="inlineStr">
         <is>
           <t>14-Jul-2026 15:58:15</t>
         </is>
       </c>
-      <c r="G497" t="inlineStr"/>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H497" t="inlineStr">
         <is>
           <t>SUCCESS</t>
@@ -78244,7 +78334,7 @@
       </c>
       <c r="V497" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W497" t="inlineStr">
@@ -78267,15 +78357,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA497" t="inlineStr"/>
-      <c r="AB497" t="inlineStr"/>
+      <c r="AA497" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="AB497" t="n">
+        <v>18.79</v>
+      </c>
       <c r="AC497" t="n">
         <v>0</v>
       </c>
       <c r="AD497" t="n">
         <v>0</v>
       </c>
-      <c r="AE497" t="inlineStr"/>
+      <c r="AE497" t="n">
+        <v>123.19</v>
+      </c>
       <c r="AF497" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -78315,13 +78411,19 @@
       <c r="D498" t="n">
         <v>8700</v>
       </c>
-      <c r="E498" t="inlineStr"/>
+      <c r="E498" t="n">
+        <v>8700</v>
+      </c>
       <c r="F498" t="inlineStr">
         <is>
           <t>14-Jul-2026 16:01:05</t>
         </is>
       </c>
-      <c r="G498" t="inlineStr"/>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H498" t="inlineStr">
         <is>
           <t>SUCCESS</t>
@@ -78386,7 +78488,7 @@
       </c>
       <c r="V498" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W498" t="inlineStr">
@@ -78409,15 +78511,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA498" t="inlineStr"/>
-      <c r="AB498" t="inlineStr"/>
+      <c r="AA498" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="AB498" t="n">
+        <v>18.79</v>
+      </c>
       <c r="AC498" t="n">
         <v>0</v>
       </c>
       <c r="AD498" t="n">
         <v>0</v>
       </c>
-      <c r="AE498" t="inlineStr"/>
+      <c r="AE498" t="n">
+        <v>123.19</v>
+      </c>
       <c r="AF498" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -78457,13 +78565,19 @@
       <c r="D499" t="n">
         <v>8700</v>
       </c>
-      <c r="E499" t="inlineStr"/>
+      <c r="E499" t="n">
+        <v>8700</v>
+      </c>
       <c r="F499" t="inlineStr">
         <is>
           <t>14-Jul-2026 17:52:35</t>
         </is>
       </c>
-      <c r="G499" t="inlineStr"/>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H499" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -78528,7 +78642,7 @@
       </c>
       <c r="V499" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W499" t="inlineStr">
@@ -78551,15 +78665,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA499" t="inlineStr"/>
-      <c r="AB499" t="inlineStr"/>
+      <c r="AA499" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB499" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC499" t="n">
         <v>0</v>
       </c>
       <c r="AD499" t="n">
         <v>0</v>
       </c>
-      <c r="AE499" t="inlineStr"/>
+      <c r="AE499" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF499" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -78603,7 +78723,9 @@
       <c r="D500" t="n">
         <v>12300</v>
       </c>
-      <c r="E500" t="inlineStr"/>
+      <c r="E500" t="n">
+        <v>12300</v>
+      </c>
       <c r="F500" t="inlineStr">
         <is>
           <t>14-Jul-2026 18:40:49</t>
@@ -78674,7 +78796,7 @@
       </c>
       <c r="V500" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W500" t="inlineStr">
@@ -78697,15 +78819,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA500" t="inlineStr"/>
-      <c r="AB500" t="inlineStr"/>
+      <c r="AA500" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB500" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC500" t="n">
         <v>0</v>
       </c>
       <c r="AD500" t="n">
         <v>0</v>
       </c>
-      <c r="AE500" t="inlineStr"/>
+      <c r="AE500" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF500" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -78749,13 +78877,19 @@
       <c r="D501" t="n">
         <v>9000</v>
       </c>
-      <c r="E501" t="inlineStr"/>
+      <c r="E501" t="n">
+        <v>9000</v>
+      </c>
       <c r="F501" t="inlineStr">
         <is>
           <t>14-Jul-2026 18:43:00</t>
         </is>
       </c>
-      <c r="G501" t="inlineStr"/>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H501" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -78820,7 +78954,7 @@
       </c>
       <c r="V501" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W501" t="inlineStr">
@@ -78843,15 +78977,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA501" t="inlineStr"/>
-      <c r="AB501" t="inlineStr"/>
+      <c r="AA501" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB501" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC501" t="n">
         <v>0</v>
       </c>
       <c r="AD501" t="n">
         <v>0</v>
       </c>
-      <c r="AE501" t="inlineStr"/>
+      <c r="AE501" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF501" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -78895,13 +79035,19 @@
       <c r="D502" t="n">
         <v>7250</v>
       </c>
-      <c r="E502" t="inlineStr"/>
+      <c r="E502" t="n">
+        <v>7250</v>
+      </c>
       <c r="F502" t="inlineStr">
         <is>
           <t>14-Jul-2026 19:25:25</t>
         </is>
       </c>
-      <c r="G502" t="inlineStr"/>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H502" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -78966,7 +79112,7 @@
       </c>
       <c r="V502" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W502" t="inlineStr">
@@ -78989,15 +79135,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA502" t="inlineStr"/>
-      <c r="AB502" t="inlineStr"/>
+      <c r="AA502" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB502" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC502" t="n">
         <v>0</v>
       </c>
       <c r="AD502" t="n">
         <v>0</v>
       </c>
-      <c r="AE502" t="inlineStr"/>
+      <c r="AE502" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF502" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
@@ -79041,13 +79193,19 @@
       <c r="D503" t="n">
         <v>9000</v>
       </c>
-      <c r="E503" t="inlineStr"/>
+      <c r="E503" t="n">
+        <v>9000</v>
+      </c>
       <c r="F503" t="inlineStr">
         <is>
           <t>14-Jul-2026 21:50:45</t>
         </is>
       </c>
-      <c r="G503" t="inlineStr"/>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H503" t="inlineStr">
         <is>
           <t>SUCCESS</t>
@@ -79112,7 +79270,7 @@
       </c>
       <c r="V503" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W503" t="inlineStr">
@@ -79135,15 +79293,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA503" t="inlineStr"/>
-      <c r="AB503" t="inlineStr"/>
+      <c r="AA503" t="n">
+        <v>108</v>
+      </c>
+      <c r="AB503" t="n">
+        <v>19.44</v>
+      </c>
       <c r="AC503" t="n">
         <v>0</v>
       </c>
       <c r="AD503" t="n">
         <v>0</v>
       </c>
-      <c r="AE503" t="inlineStr"/>
+      <c r="AE503" t="n">
+        <v>127.44</v>
+      </c>
       <c r="AF503" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -79183,13 +79347,19 @@
       <c r="D504" t="n">
         <v>9000</v>
       </c>
-      <c r="E504" t="inlineStr"/>
+      <c r="E504" t="n">
+        <v>9000</v>
+      </c>
       <c r="F504" t="inlineStr">
         <is>
           <t>14-Jul-2026 22:23:39</t>
         </is>
       </c>
-      <c r="G504" t="inlineStr"/>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H504" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESS</t>
@@ -79254,7 +79424,7 @@
       </c>
       <c r="V504" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W504" t="inlineStr">
@@ -79277,15 +79447,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA504" t="inlineStr"/>
-      <c r="AB504" t="inlineStr"/>
+      <c r="AA504" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB504" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC504" t="n">
         <v>0</v>
       </c>
       <c r="AD504" t="n">
         <v>0</v>
       </c>
-      <c r="AE504" t="inlineStr"/>
+      <c r="AE504" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF504" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -79329,13 +79505,19 @@
       <c r="D505" t="n">
         <v>8700</v>
       </c>
-      <c r="E505" t="inlineStr"/>
+      <c r="E505" t="n">
+        <v>8700</v>
+      </c>
       <c r="F505" t="inlineStr">
         <is>
           <t>14-Jul-2026 22:25:50</t>
         </is>
       </c>
-      <c r="G505" t="inlineStr"/>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 17:54:32</t>
+        </is>
+      </c>
       <c r="H505" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESS</t>
@@ -79400,7 +79582,7 @@
       </c>
       <c r="V505" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W505" t="inlineStr">
@@ -79423,15 +79605,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA505" t="inlineStr"/>
-      <c r="AB505" t="inlineStr"/>
+      <c r="AA505" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB505" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC505" t="n">
         <v>0</v>
       </c>
       <c r="AD505" t="n">
         <v>0</v>
       </c>
-      <c r="AE505" t="inlineStr"/>
+      <c r="AE505" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF505" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -79475,7 +79663,9 @@
       <c r="D506" t="n">
         <v>11600</v>
       </c>
-      <c r="E506" t="inlineStr"/>
+      <c r="E506" t="n">
+        <v>11600</v>
+      </c>
       <c r="F506" t="inlineStr">
         <is>
           <t>14-Jul-2026 23:02:15</t>
@@ -79546,7 +79736,7 @@
       </c>
       <c r="V506" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W506" t="inlineStr">
@@ -79569,15 +79759,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA506" t="inlineStr"/>
-      <c r="AB506" t="inlineStr"/>
+      <c r="AA506" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB506" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC506" t="n">
         <v>0</v>
       </c>
       <c r="AD506" t="n">
         <v>0</v>
       </c>
-      <c r="AE506" t="inlineStr"/>
+      <c r="AE506" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF506" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
@@ -79753,6 +79949,2192 @@
           <t>UPI INTENT</t>
         </is>
       </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="n">
+        <v>17595</v>
+      </c>
+      <c r="B508" t="inlineStr"/>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>83****2419</t>
+        </is>
+      </c>
+      <c r="D508" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E508" t="inlineStr"/>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 07:06:53</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr"/>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K508" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>*0314</t>
+        </is>
+      </c>
+      <c r="M508" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N508" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O508" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P508" t="n">
+        <v>11000372806721</v>
+      </c>
+      <c r="Q508" t="n">
+        <v>1784079402320</v>
+      </c>
+      <c r="R508" t="n">
+        <v>109042362519</v>
+      </c>
+      <c r="S508" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T508" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U508" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V508" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W508" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X508" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y508" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z508" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA508" t="inlineStr"/>
+      <c r="AB508" t="inlineStr"/>
+      <c r="AC508" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD508" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE508" t="inlineStr"/>
+      <c r="AF508" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG508" t="inlineStr"/>
+      <c r="AH508" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI508" t="n">
+        <v>20314</v>
+      </c>
+      <c r="AJ508" t="inlineStr">
+        <is>
+          <t>273655</t>
+        </is>
+      </c>
+      <c r="AK508" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL508" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="n">
+        <v>17596</v>
+      </c>
+      <c r="B509" t="inlineStr"/>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>83****2419</t>
+        </is>
+      </c>
+      <c r="D509" t="n">
+        <v>9400</v>
+      </c>
+      <c r="E509" t="inlineStr"/>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 07:08:31</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr"/>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K509" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>*0315</t>
+        </is>
+      </c>
+      <c r="M509" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N509" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O509" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P509" t="n">
+        <v>11000372806821</v>
+      </c>
+      <c r="Q509" t="n">
+        <v>1784079502710</v>
+      </c>
+      <c r="R509" t="n">
+        <v>501835994354</v>
+      </c>
+      <c r="S509" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T509" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U509" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V509" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W509" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X509" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y509" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z509" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA509" t="inlineStr"/>
+      <c r="AB509" t="inlineStr"/>
+      <c r="AC509" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD509" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE509" t="inlineStr"/>
+      <c r="AF509" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG509" t="inlineStr"/>
+      <c r="AH509" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI509" t="n">
+        <v>20315</v>
+      </c>
+      <c r="AJ509" t="inlineStr">
+        <is>
+          <t>274742</t>
+        </is>
+      </c>
+      <c r="AK509" t="inlineStr">
+        <is>
+          <t>2088</t>
+        </is>
+      </c>
+      <c r="AL509" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="n">
+        <v>16782</v>
+      </c>
+      <c r="B510" t="inlineStr"/>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>63****2843</t>
+        </is>
+      </c>
+      <c r="D510" t="n">
+        <v>11600</v>
+      </c>
+      <c r="E510" t="inlineStr"/>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 07:35:47</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr"/>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K510" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>*9079</t>
+        </is>
+      </c>
+      <c r="M510" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N510" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O510" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P510" t="n">
+        <v>11000372811593</v>
+      </c>
+      <c r="Q510" t="n">
+        <v>1784081129004</v>
+      </c>
+      <c r="R510" t="n">
+        <v>619641890897</v>
+      </c>
+      <c r="S510" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T510" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U510" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V510" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W510" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X510" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y510" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z510" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA510" t="inlineStr"/>
+      <c r="AB510" t="inlineStr"/>
+      <c r="AC510" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD510" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE510" t="inlineStr"/>
+      <c r="AF510" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG510" t="inlineStr"/>
+      <c r="AH510" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI510" t="n">
+        <v>19079</v>
+      </c>
+      <c r="AJ510" t="inlineStr">
+        <is>
+          <t>275413</t>
+        </is>
+      </c>
+      <c r="AK510" t="inlineStr">
+        <is>
+          <t>2092</t>
+        </is>
+      </c>
+      <c r="AL510" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="n">
+        <v>16783</v>
+      </c>
+      <c r="B511" t="inlineStr"/>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>63****2843</t>
+        </is>
+      </c>
+      <c r="D511" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E511" t="inlineStr"/>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 07:37:12</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr"/>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K511" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>*8559</t>
+        </is>
+      </c>
+      <c r="M511" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N511" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O511" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P511" t="n">
+        <v>11000372811793</v>
+      </c>
+      <c r="Q511" t="n">
+        <v>1784081222752</v>
+      </c>
+      <c r="R511" t="n">
+        <v>619636383557</v>
+      </c>
+      <c r="S511" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T511" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U511" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V511" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W511" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X511" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y511" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z511" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA511" t="inlineStr"/>
+      <c r="AB511" t="inlineStr"/>
+      <c r="AC511" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD511" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE511" t="inlineStr"/>
+      <c r="AF511" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG511" t="inlineStr"/>
+      <c r="AH511" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI511" t="n">
+        <v>18559</v>
+      </c>
+      <c r="AJ511" t="inlineStr">
+        <is>
+          <t>273564</t>
+        </is>
+      </c>
+      <c r="AK511" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL511" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="n">
+        <v>16934</v>
+      </c>
+      <c r="B512" t="inlineStr"/>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>73****0623</t>
+        </is>
+      </c>
+      <c r="D512" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E512" t="inlineStr"/>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 09:13:39</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr"/>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K512" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>*8063</t>
+        </is>
+      </c>
+      <c r="M512" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N512" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O512" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P512" t="n">
+        <v>11000372831197</v>
+      </c>
+      <c r="Q512" t="n">
+        <v>1784086996179</v>
+      </c>
+      <c r="R512" t="n">
+        <v>122321756433</v>
+      </c>
+      <c r="S512" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T512" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U512" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V512" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W512" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X512" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y512" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z512" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA512" t="inlineStr"/>
+      <c r="AB512" t="inlineStr"/>
+      <c r="AC512" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD512" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE512" t="inlineStr"/>
+      <c r="AF512" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG512" t="inlineStr"/>
+      <c r="AH512" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI512" t="n">
+        <v>18063</v>
+      </c>
+      <c r="AJ512" t="inlineStr">
+        <is>
+          <t>271403</t>
+        </is>
+      </c>
+      <c r="AK512" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL512" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="n">
+        <v>17051</v>
+      </c>
+      <c r="B513" t="inlineStr"/>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>73****0623</t>
+        </is>
+      </c>
+      <c r="D513" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E513" t="inlineStr"/>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 09:18:21</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr"/>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K513" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>*8700</t>
+        </is>
+      </c>
+      <c r="M513" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N513" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O513" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P513" t="n">
+        <v>11000372832257</v>
+      </c>
+      <c r="Q513" t="n">
+        <v>1784087211347</v>
+      </c>
+      <c r="R513" t="n">
+        <v>943665380156</v>
+      </c>
+      <c r="S513" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T513" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U513" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V513" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W513" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X513" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y513" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z513" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA513" t="inlineStr"/>
+      <c r="AB513" t="inlineStr"/>
+      <c r="AC513" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD513" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE513" t="inlineStr"/>
+      <c r="AF513" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG513" t="inlineStr"/>
+      <c r="AH513" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI513" t="n">
+        <v>18700</v>
+      </c>
+      <c r="AJ513" t="inlineStr">
+        <is>
+          <t>273733</t>
+        </is>
+      </c>
+      <c r="AK513" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL513" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="n">
+        <v>16572</v>
+      </c>
+      <c r="B514" t="inlineStr"/>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>99****9977</t>
+        </is>
+      </c>
+      <c r="D514" t="n">
+        <v>9400</v>
+      </c>
+      <c r="E514" t="inlineStr"/>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 10:42:37</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr"/>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K514" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>*8977</t>
+        </is>
+      </c>
+      <c r="M514" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N514" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O514" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P514" t="n">
+        <v>11000372853210</v>
+      </c>
+      <c r="Q514" t="n">
+        <v>1784092322989</v>
+      </c>
+      <c r="R514" t="n">
+        <v>204571823197</v>
+      </c>
+      <c r="S514" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T514" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U514" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V514" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W514" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X514" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y514" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z514" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA514" t="inlineStr"/>
+      <c r="AB514" t="inlineStr"/>
+      <c r="AC514" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD514" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE514" t="inlineStr"/>
+      <c r="AF514" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG514" t="inlineStr"/>
+      <c r="AH514" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI514" t="n">
+        <v>18977</v>
+      </c>
+      <c r="AJ514" t="inlineStr">
+        <is>
+          <t>274858</t>
+        </is>
+      </c>
+      <c r="AK514" t="inlineStr">
+        <is>
+          <t>2088</t>
+        </is>
+      </c>
+      <c r="AL514" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="n">
+        <v>16571</v>
+      </c>
+      <c r="B515" t="inlineStr"/>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>99****9977</t>
+        </is>
+      </c>
+      <c r="D515" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E515" t="inlineStr"/>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 10:44:51</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr"/>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K515" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>*9204</t>
+        </is>
+      </c>
+      <c r="M515" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N515" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O515" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P515" t="n">
+        <v>11000372854188</v>
+      </c>
+      <c r="Q515" t="n">
+        <v>1784092481421</v>
+      </c>
+      <c r="R515" t="n">
+        <v>27098224180</v>
+      </c>
+      <c r="S515" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T515" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U515" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V515" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W515" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X515" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y515" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z515" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA515" t="inlineStr"/>
+      <c r="AB515" t="inlineStr"/>
+      <c r="AC515" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD515" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE515" t="inlineStr"/>
+      <c r="AF515" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG515" t="inlineStr"/>
+      <c r="AH515" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI515" t="n">
+        <v>19204</v>
+      </c>
+      <c r="AJ515" t="inlineStr">
+        <is>
+          <t>275975</t>
+        </is>
+      </c>
+      <c r="AK515" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL515" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="n">
+        <v>17577</v>
+      </c>
+      <c r="B516" t="inlineStr"/>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>95****1640</t>
+        </is>
+      </c>
+      <c r="D516" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E516" t="inlineStr"/>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 13:35:56</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr"/>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K516" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>*0296</t>
+        </is>
+      </c>
+      <c r="M516" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N516" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O516" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P516" t="n">
+        <v>11000372928457</v>
+      </c>
+      <c r="Q516" t="n">
+        <v>1784102716449</v>
+      </c>
+      <c r="R516" t="n">
+        <v>743878369192</v>
+      </c>
+      <c r="S516" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T516" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U516" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V516" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W516" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X516" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y516" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z516" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA516" t="inlineStr"/>
+      <c r="AB516" t="inlineStr"/>
+      <c r="AC516" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD516" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE516" t="inlineStr"/>
+      <c r="AF516" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG516" t="inlineStr"/>
+      <c r="AH516" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI516" t="n">
+        <v>20296</v>
+      </c>
+      <c r="AJ516" t="inlineStr">
+        <is>
+          <t>273652</t>
+        </is>
+      </c>
+      <c r="AK516" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL516" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="n">
+        <v>17576</v>
+      </c>
+      <c r="B517" t="inlineStr"/>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>95****1640</t>
+        </is>
+      </c>
+      <c r="D517" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E517" t="inlineStr"/>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 13:34:37</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr"/>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K517" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>*0295</t>
+        </is>
+      </c>
+      <c r="M517" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N517" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O517" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P517" t="n">
+        <v>11000372929322</v>
+      </c>
+      <c r="Q517" t="n">
+        <v>1784102668153</v>
+      </c>
+      <c r="R517" t="n">
+        <v>310715703195</v>
+      </c>
+      <c r="S517" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T517" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U517" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V517" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W517" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X517" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y517" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z517" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA517" t="inlineStr"/>
+      <c r="AB517" t="inlineStr"/>
+      <c r="AC517" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD517" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE517" t="inlineStr"/>
+      <c r="AF517" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG517" t="inlineStr"/>
+      <c r="AH517" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI517" t="n">
+        <v>20295</v>
+      </c>
+      <c r="AJ517" t="inlineStr">
+        <is>
+          <t>272416</t>
+        </is>
+      </c>
+      <c r="AK517" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL517" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="n">
+        <v>15866</v>
+      </c>
+      <c r="B518" t="inlineStr"/>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>83****1596</t>
+        </is>
+      </c>
+      <c r="D518" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E518" t="inlineStr"/>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 14:52:10</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr"/>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K518" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>*8617</t>
+        </is>
+      </c>
+      <c r="M518" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N518" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O518" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P518" t="n">
+        <v>11000372954049</v>
+      </c>
+      <c r="Q518" t="n">
+        <v>1784107318823</v>
+      </c>
+      <c r="R518" t="n">
+        <v>959857018282</v>
+      </c>
+      <c r="S518" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T518" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U518" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V518" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W518" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X518" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y518" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z518" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA518" t="inlineStr"/>
+      <c r="AB518" t="inlineStr"/>
+      <c r="AC518" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD518" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE518" t="inlineStr"/>
+      <c r="AF518" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG518" t="inlineStr"/>
+      <c r="AH518" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI518" t="n">
+        <v>18617</v>
+      </c>
+      <c r="AJ518" t="inlineStr">
+        <is>
+          <t>273586</t>
+        </is>
+      </c>
+      <c r="AK518" t="inlineStr">
+        <is>
+          <t>2084</t>
+        </is>
+      </c>
+      <c r="AL518" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="n">
+        <v>17315</v>
+      </c>
+      <c r="B519" t="inlineStr"/>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>83****2524</t>
+        </is>
+      </c>
+      <c r="D519" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E519" t="inlineStr"/>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 15:36:05</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr"/>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K519" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>*0023</t>
+        </is>
+      </c>
+      <c r="M519" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N519" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O519" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P519" t="n">
+        <v>11000372961520</v>
+      </c>
+      <c r="Q519" t="n">
+        <v>1784111204911</v>
+      </c>
+      <c r="R519" t="n">
+        <v>550381119890</v>
+      </c>
+      <c r="S519" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T519" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U519" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V519" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W519" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X519" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y519" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z519" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA519" t="inlineStr"/>
+      <c r="AB519" t="inlineStr"/>
+      <c r="AC519" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD519" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE519" t="inlineStr"/>
+      <c r="AF519" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG519" t="inlineStr"/>
+      <c r="AH519" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI519" t="n">
+        <v>20023</v>
+      </c>
+      <c r="AJ519" t="inlineStr">
+        <is>
+          <t>271428</t>
+        </is>
+      </c>
+      <c r="AK519" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL519" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="n">
+        <v>17597</v>
+      </c>
+      <c r="B520" t="inlineStr"/>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>83****2524</t>
+        </is>
+      </c>
+      <c r="D520" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E520" t="inlineStr"/>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 15:41:19</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr"/>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K520" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>*0316</t>
+        </is>
+      </c>
+      <c r="M520" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N520" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O520" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P520" t="n">
+        <v>11000372961777</v>
+      </c>
+      <c r="Q520" t="n">
+        <v>1784111565572</v>
+      </c>
+      <c r="R520" t="n">
+        <v>807149121170</v>
+      </c>
+      <c r="S520" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T520" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U520" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V520" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W520" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X520" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y520" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z520" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA520" t="inlineStr"/>
+      <c r="AB520" t="inlineStr"/>
+      <c r="AC520" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD520" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE520" t="inlineStr"/>
+      <c r="AF520" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG520" t="inlineStr"/>
+      <c r="AH520" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI520" t="n">
+        <v>20316</v>
+      </c>
+      <c r="AJ520" t="inlineStr">
+        <is>
+          <t>269214</t>
+        </is>
+      </c>
+      <c r="AK520" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="AL520" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="n">
+        <v>17661</v>
+      </c>
+      <c r="B521" t="inlineStr"/>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>70****0341</t>
+        </is>
+      </c>
+      <c r="D521" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E521" t="inlineStr"/>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 18:21:38</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr"/>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K521" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>*0383</t>
+        </is>
+      </c>
+      <c r="M521" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N521" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O521" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P521" t="n">
+        <v>11000372996670</v>
+      </c>
+      <c r="Q521" t="n">
+        <v>1784119874839</v>
+      </c>
+      <c r="R521" t="n">
+        <v>377647234780</v>
+      </c>
+      <c r="S521" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T521" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U521" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V521" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W521" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X521" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y521" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z521" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA521" t="inlineStr"/>
+      <c r="AB521" t="inlineStr"/>
+      <c r="AC521" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD521" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE521" t="inlineStr"/>
+      <c r="AF521" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG521" t="inlineStr"/>
+      <c r="AH521" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI521" t="n">
+        <v>20383</v>
+      </c>
+      <c r="AJ521" t="inlineStr">
+        <is>
+          <t>277204</t>
+        </is>
+      </c>
+      <c r="AK521" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="AL521" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="n">
+        <v>17523</v>
+      </c>
+      <c r="B522" t="inlineStr"/>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>77****9882</t>
+        </is>
+      </c>
+      <c r="D522" t="n">
+        <v>18600</v>
+      </c>
+      <c r="E522" t="inlineStr"/>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>15-Jul-2026 19:46:28</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr"/>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K522" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>*0242</t>
+        </is>
+      </c>
+      <c r="M522" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N522" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O522" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P522" t="n">
+        <v>11000373011586</v>
+      </c>
+      <c r="Q522" t="n">
+        <v>1784124848978</v>
+      </c>
+      <c r="R522" t="n">
+        <v>619631055262</v>
+      </c>
+      <c r="S522" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T522" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U522" t="inlineStr">
+        <is>
+          <t>HDFC Bank FSS PG</t>
+        </is>
+      </c>
+      <c r="V522" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W522" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X522" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y522" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="Z522" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA522" t="inlineStr"/>
+      <c r="AB522" t="inlineStr"/>
+      <c r="AC522" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD522" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE522" t="inlineStr"/>
+      <c r="AF522" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG522" t="inlineStr"/>
+      <c r="AH522" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI522" t="n">
+        <v>20242</v>
+      </c>
+      <c r="AJ522" t="inlineStr">
+        <is>
+          <t>273497,269878,273810</t>
+        </is>
+      </c>
+      <c r="AK522" t="inlineStr">
+        <is>
+          <t>2084,2067,2085</t>
+        </is>
+      </c>
+      <c r="AL522" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update fee collection records and payment data
Correct and update student fee payment records across multiple reports. Changes include:

- Fix transaction records in atom payment report with corrected net amounts and settlement details
- Reorder and add missing daywise fee collection entries with updated student payment records
- Update individual student fee payment amounts in the comprehensive fees collection report
- Add new fee concession records for students making additional payments on July 17
- Consolidate and correct payment status across related fee collection data files

These updates reflect recent fee payments received and corrections to previously incomplete transaction records.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL527"/>
+  <dimension ref="A1:AL528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82321,7 +82321,9 @@
       <c r="D523" t="n">
         <v>8700</v>
       </c>
-      <c r="E523" t="inlineStr"/>
+      <c r="E523" t="n">
+        <v>8700</v>
+      </c>
       <c r="F523" t="inlineStr">
         <is>
           <t>16-Jul-2026 09:10:49</t>
@@ -82392,7 +82394,7 @@
       </c>
       <c r="V523" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W523" t="inlineStr">
@@ -82415,15 +82417,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA523" t="inlineStr"/>
-      <c r="AB523" t="inlineStr"/>
+      <c r="AA523" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB523" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC523" t="n">
         <v>0</v>
       </c>
       <c r="AD523" t="n">
         <v>0</v>
       </c>
-      <c r="AE523" t="inlineStr"/>
+      <c r="AE523" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF523" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -82467,7 +82475,9 @@
       <c r="D524" t="n">
         <v>9000</v>
       </c>
-      <c r="E524" t="inlineStr"/>
+      <c r="E524" t="n">
+        <v>9000</v>
+      </c>
       <c r="F524" t="inlineStr">
         <is>
           <t>16-Jul-2026 11:23:39</t>
@@ -82538,7 +82548,7 @@
       </c>
       <c r="V524" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W524" t="inlineStr">
@@ -82561,15 +82571,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA524" t="inlineStr"/>
-      <c r="AB524" t="inlineStr"/>
+      <c r="AA524" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC524" t="n">
         <v>0</v>
       </c>
       <c r="AD524" t="n">
         <v>0</v>
       </c>
-      <c r="AE524" t="inlineStr"/>
+      <c r="AE524" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF524" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -82613,7 +82629,9 @@
       <c r="D525" t="n">
         <v>9000</v>
       </c>
-      <c r="E525" t="inlineStr"/>
+      <c r="E525" t="n">
+        <v>9000</v>
+      </c>
       <c r="F525" t="inlineStr">
         <is>
           <t>16-Jul-2026 11:53:37</t>
@@ -82684,7 +82702,7 @@
       </c>
       <c r="V525" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W525" t="inlineStr">
@@ -82707,15 +82725,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA525" t="inlineStr"/>
-      <c r="AB525" t="inlineStr"/>
+      <c r="AA525" t="n">
+        <v>108</v>
+      </c>
+      <c r="AB525" t="n">
+        <v>19.44</v>
+      </c>
       <c r="AC525" t="n">
         <v>0</v>
       </c>
       <c r="AD525" t="n">
         <v>0</v>
       </c>
-      <c r="AE525" t="inlineStr"/>
+      <c r="AE525" t="n">
+        <v>127.44</v>
+      </c>
       <c r="AF525" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -82755,7 +82779,9 @@
       <c r="D526" t="n">
         <v>7250</v>
       </c>
-      <c r="E526" t="inlineStr"/>
+      <c r="E526" t="n">
+        <v>7250</v>
+      </c>
       <c r="F526" t="inlineStr">
         <is>
           <t>16-Jul-2026 12:07:38</t>
@@ -82826,7 +82852,7 @@
       </c>
       <c r="V526" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W526" t="inlineStr">
@@ -82849,15 +82875,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA526" t="inlineStr"/>
-      <c r="AB526" t="inlineStr"/>
+      <c r="AA526" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB526" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC526" t="n">
         <v>0</v>
       </c>
       <c r="AD526" t="n">
         <v>0</v>
       </c>
-      <c r="AE526" t="inlineStr"/>
+      <c r="AE526" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF526" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
@@ -82897,7 +82929,9 @@
       <c r="D527" t="n">
         <v>8400</v>
       </c>
-      <c r="E527" t="inlineStr"/>
+      <c r="E527" t="n">
+        <v>8400</v>
+      </c>
       <c r="F527" t="inlineStr">
         <is>
           <t>16-Jul-2026 14:35:35</t>
@@ -82968,7 +83002,7 @@
       </c>
       <c r="V527" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="W527" t="inlineStr">
@@ -82991,15 +83025,21 @@
           <t>m**********@gmail.com</t>
         </is>
       </c>
-      <c r="AA527" t="inlineStr"/>
-      <c r="AB527" t="inlineStr"/>
+      <c r="AA527" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB527" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AC527" t="n">
         <v>0</v>
       </c>
       <c r="AD527" t="n">
         <v>0</v>
       </c>
-      <c r="AE527" t="inlineStr"/>
+      <c r="AE527" t="n">
+        <v>5.9</v>
+      </c>
       <c r="AF527" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
@@ -83025,6 +83065,152 @@
         </is>
       </c>
       <c r="AL527" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="n">
+        <v>17633</v>
+      </c>
+      <c r="B528" t="inlineStr"/>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>73****3777</t>
+        </is>
+      </c>
+      <c r="D528" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E528" t="inlineStr"/>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>17-Jul-2026 17:16:04</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr"/>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K528" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>*0377</t>
+        </is>
+      </c>
+      <c r="M528" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N528" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O528" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P528" t="n">
+        <v>11000373484907</v>
+      </c>
+      <c r="Q528" t="n">
+        <v>1784288751850</v>
+      </c>
+      <c r="R528" t="n">
+        <v>760702566589</v>
+      </c>
+      <c r="S528" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T528" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U528" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V528" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W528" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X528" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y528" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z528" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA528" t="inlineStr"/>
+      <c r="AB528" t="inlineStr"/>
+      <c r="AC528" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD528" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE528" t="inlineStr"/>
+      <c r="AF528" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG528" t="inlineStr"/>
+      <c r="AH528" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI528" t="n">
+        <v>20377</v>
+      </c>
+      <c r="AJ528" t="inlineStr">
+        <is>
+          <t>277205</t>
+        </is>
+      </c>
+      <c r="AK528" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="AL528" t="inlineStr">
         <is>
           <t>UPI INTENT</t>
         </is>

</xml_diff>

<commit_message>
Record two online fee payments and update collections
Add two UPI payment records (AdmissionNo 17163: MUHAMMAD ZAYN KHAN, 7250; AdmissionNo 15974: VARSHINI PRIYA UMMIDI, 12300) to atom_report_cleaned (CSV/XLSX) and daywise CSVs (daywise_fees_collection, daywise_fees_collection_2026-27, daywise_fees_collection_online). Update aggregated totals in fees_collection.csv, fees_collection_2026_27_1.csv and merged_fee_collection to reflect the payments (Total_Fee_Paid adjusted and Total_Due reduced). source_data/atom_report.xlsx (binary) was also updated.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL530"/>
+  <dimension ref="A1:AL532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83540,6 +83540,298 @@
         </is>
       </c>
     </row>
+    <row r="531">
+      <c r="A531" t="n">
+        <v>17163</v>
+      </c>
+      <c r="B531" t="inlineStr"/>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>82****8795</t>
+        </is>
+      </c>
+      <c r="D531" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E531" t="inlineStr"/>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>18-Jul-2026 23:36:28</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr"/>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K531" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L531" t="inlineStr">
+        <is>
+          <t>*9878</t>
+        </is>
+      </c>
+      <c r="M531" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N531" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O531" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P531" t="n">
+        <v>11000373792011</v>
+      </c>
+      <c r="Q531" t="n">
+        <v>1784397874065</v>
+      </c>
+      <c r="R531" t="n">
+        <v>656573924792</v>
+      </c>
+      <c r="S531" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T531" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U531" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V531" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W531" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X531" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y531" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z531" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA531" t="inlineStr"/>
+      <c r="AB531" t="inlineStr"/>
+      <c r="AC531" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD531" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE531" t="inlineStr"/>
+      <c r="AF531" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG531" t="inlineStr"/>
+      <c r="AH531" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI531" t="n">
+        <v>19878</v>
+      </c>
+      <c r="AJ531" t="inlineStr">
+        <is>
+          <t>269357</t>
+        </is>
+      </c>
+      <c r="AK531" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="AL531" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="n">
+        <v>15974</v>
+      </c>
+      <c r="B532" t="inlineStr"/>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>99****4605</t>
+        </is>
+      </c>
+      <c r="D532" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E532" t="inlineStr"/>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>19-Jul-2026 12:14:18</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr"/>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K532" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L532" t="inlineStr">
+        <is>
+          <t>*9352</t>
+        </is>
+      </c>
+      <c r="M532" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N532" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O532" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P532" t="n">
+        <v>11000373829949</v>
+      </c>
+      <c r="Q532" t="n">
+        <v>1784443438932</v>
+      </c>
+      <c r="R532" t="n">
+        <v>495905674100</v>
+      </c>
+      <c r="S532" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T532" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U532" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V532" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W532" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X532" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y532" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z532" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA532" t="inlineStr"/>
+      <c r="AB532" t="inlineStr"/>
+      <c r="AC532" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD532" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE532" t="inlineStr"/>
+      <c r="AF532" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG532" t="inlineStr"/>
+      <c r="AH532" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI532" t="n">
+        <v>19352</v>
+      </c>
+      <c r="AJ532" t="inlineStr">
+        <is>
+          <t>276141</t>
+        </is>
+      </c>
+      <c r="AK532" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL532" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record fee payment for student 17464
Added online payment transaction of 7250 for student MOURYA UMMIDI (admission no 17464). Updated fee collection records across all output files and source data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL534"/>
+  <dimension ref="A1:AL535"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -84164,6 +84164,152 @@
         </is>
       </c>
     </row>
+    <row r="535">
+      <c r="A535" t="n">
+        <v>17464</v>
+      </c>
+      <c r="B535" t="inlineStr"/>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>81****4454</t>
+        </is>
+      </c>
+      <c r="D535" t="n">
+        <v>7250</v>
+      </c>
+      <c r="E535" t="inlineStr"/>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>20-Jul-2026 21:46:59</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr"/>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K535" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L535" t="inlineStr">
+        <is>
+          <t>*0147</t>
+        </is>
+      </c>
+      <c r="M535" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N535" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O535" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P535" t="n">
+        <v>11000374170898</v>
+      </c>
+      <c r="Q535" t="n">
+        <v>1784564204653</v>
+      </c>
+      <c r="R535" t="n">
+        <v>177810809921</v>
+      </c>
+      <c r="S535" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T535" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U535" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V535" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W535" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X535" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y535" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z535" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA535" t="inlineStr"/>
+      <c r="AB535" t="inlineStr"/>
+      <c r="AC535" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD535" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE535" t="inlineStr"/>
+      <c r="AF535" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG535" t="inlineStr"/>
+      <c r="AH535" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI535" t="n">
+        <v>20147</v>
+      </c>
+      <c r="AJ535" t="inlineStr">
+        <is>
+          <t>269188</t>
+        </is>
+      </c>
+      <c r="AK535" t="inlineStr">
+        <is>
+          <t>2070</t>
+        </is>
+      </c>
+      <c r="AL535" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update atom settlements and fees reports
Apply data fixes across reports and source: fill settlement dates for multiple UPI transactions in atom_report_cleaned (CSV/XLSX); add test/student entry 'mysklc1,praveentesting' to fees_collection and fees_collection_2026_27_1 and matching rows in merged_fee_collection; correct many rows in fees_report.csv (fb_no, term payments, totals and status labels such as '1 Term'/'2 Terms'/'Total Paid'); update source_data/atom_report.xlsx accordingly.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -87811,7 +87811,11 @@
           <t>23-Jul-2026 09:48:54</t>
         </is>
       </c>
-      <c r="G558" t="inlineStr"/>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>24-Jul-2026 18:56:45</t>
+        </is>
+      </c>
       <c r="H558" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -87876,7 +87880,7 @@
       </c>
       <c r="V558" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W558" t="inlineStr">
@@ -87965,7 +87969,11 @@
           <t>23-Jul-2026 12:01:04</t>
         </is>
       </c>
-      <c r="G559" t="inlineStr"/>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>24-Jul-2026 18:56:45</t>
+        </is>
+      </c>
       <c r="H559" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -88030,7 +88038,7 @@
       </c>
       <c r="V559" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W559" t="inlineStr">
@@ -88119,7 +88127,11 @@
           <t>23-Jul-2026 11:59:43</t>
         </is>
       </c>
-      <c r="G560" t="inlineStr"/>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>24-Jul-2026 18:56:45</t>
+        </is>
+      </c>
       <c r="H560" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -88184,7 +88196,7 @@
       </c>
       <c r="V560" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W560" t="inlineStr">
@@ -88273,7 +88285,11 @@
           <t>23-Jul-2026 12:33:37</t>
         </is>
       </c>
-      <c r="G561" t="inlineStr"/>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>24-Jul-2026 18:56:45</t>
+        </is>
+      </c>
       <c r="H561" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -88338,7 +88354,7 @@
       </c>
       <c r="V561" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W561" t="inlineStr">
@@ -88581,7 +88597,11 @@
           <t>23-Jul-2026 12:44:14</t>
         </is>
       </c>
-      <c r="G563" t="inlineStr"/>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>24-Jul-2026 18:56:45</t>
+        </is>
+      </c>
       <c r="H563" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -88646,7 +88666,7 @@
       </c>
       <c r="V563" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W563" t="inlineStr">
@@ -88735,7 +88755,11 @@
           <t>23-Jul-2026 13:22:42</t>
         </is>
       </c>
-      <c r="G564" t="inlineStr"/>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>24-Jul-2026 18:56:45</t>
+        </is>
+      </c>
       <c r="H564" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -88800,7 +88824,7 @@
       </c>
       <c r="V564" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W564" t="inlineStr">
@@ -88889,7 +88913,11 @@
           <t>23-Jul-2026 16:10:13</t>
         </is>
       </c>
-      <c r="G565" t="inlineStr"/>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>24-Jul-2026 18:56:45</t>
+        </is>
+      </c>
       <c r="H565" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -88954,7 +88982,7 @@
       </c>
       <c r="V565" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W565" t="inlineStr">
@@ -89043,7 +89071,11 @@
           <t>23-Jul-2026 18:59:23</t>
         </is>
       </c>
-      <c r="G566" t="inlineStr"/>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>24-Jul-2026 18:56:45</t>
+        </is>
+      </c>
       <c r="H566" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
@@ -89108,7 +89140,7 @@
       </c>
       <c r="V566" t="inlineStr">
         <is>
-          <t>RNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="W566" t="inlineStr">

</xml_diff>

<commit_message>
Update fee collections and fix student data records
Added recent fee collection transactions dated 2026-07-25 from ATOM payment gateway. Updated student fee payment status reflecting new payments received. Corrected student name spellings: 'SIRIVALLI GANAPATI' to 'GANAPATHI', 'KOLLIMALA' to 'KOLLIMALLA'. Updated fee paid amounts for students: DHARSHITH ASURI, SHASHANK GONDLU, REUEL PAUL KAMMARI, YAMINI GUDLA, and INAAYA BEGUM. Also added new payment entries to online and daywise fee collection reports for July 2026.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL566"/>
+  <dimension ref="A1:AL572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89208,6 +89208,882 @@
         </is>
       </c>
     </row>
+    <row r="567">
+      <c r="A567" t="n">
+        <v>17247</v>
+      </c>
+      <c r="B567" t="inlineStr"/>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>98****4144</t>
+        </is>
+      </c>
+      <c r="D567" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E567" t="inlineStr"/>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>25-Jul-2026 08:23:40</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr"/>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>*9959</t>
+        </is>
+      </c>
+      <c r="M567" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N567" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O567" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P567" t="n">
+        <v>11000374898465</v>
+      </c>
+      <c r="Q567" t="n">
+        <v>1784948006490</v>
+      </c>
+      <c r="R567" t="n">
+        <v>3077259763</v>
+      </c>
+      <c r="S567" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T567" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U567" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V567" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W567" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X567" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y567" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z567" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA567" t="inlineStr"/>
+      <c r="AB567" t="inlineStr"/>
+      <c r="AC567" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD567" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE567" t="inlineStr"/>
+      <c r="AF567" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG567" t="inlineStr"/>
+      <c r="AH567" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI567" t="n">
+        <v>19959</v>
+      </c>
+      <c r="AJ567" t="inlineStr">
+        <is>
+          <t>271271</t>
+        </is>
+      </c>
+      <c r="AK567" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL567" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="n">
+        <v>16351</v>
+      </c>
+      <c r="B568" t="inlineStr"/>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>95****4297</t>
+        </is>
+      </c>
+      <c r="D568" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E568" t="inlineStr"/>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>25-Jul-2026 10:20:06</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr"/>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>*8369</t>
+        </is>
+      </c>
+      <c r="M568" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N568" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O568" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P568" t="n">
+        <v>11000374910056</v>
+      </c>
+      <c r="Q568" t="n">
+        <v>1784954977603</v>
+      </c>
+      <c r="R568" t="n">
+        <v>1214918255</v>
+      </c>
+      <c r="S568" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T568" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U568" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V568" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W568" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X568" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y568" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z568" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA568" t="inlineStr"/>
+      <c r="AB568" t="inlineStr"/>
+      <c r="AC568" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD568" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE568" t="inlineStr"/>
+      <c r="AF568" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG568" t="inlineStr"/>
+      <c r="AH568" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI568" t="n">
+        <v>18369</v>
+      </c>
+      <c r="AJ568" t="inlineStr">
+        <is>
+          <t>272342</t>
+        </is>
+      </c>
+      <c r="AK568" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL568" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="n">
+        <v>14152</v>
+      </c>
+      <c r="B569" t="inlineStr"/>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>77****7970</t>
+        </is>
+      </c>
+      <c r="D569" t="n">
+        <v>12300</v>
+      </c>
+      <c r="E569" t="inlineStr"/>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>25-Jul-2026 10:51:44</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr"/>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>*9353</t>
+        </is>
+      </c>
+      <c r="M569" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N569" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O569" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P569" t="n">
+        <v>11000374915744</v>
+      </c>
+      <c r="Q569" t="n">
+        <v>1784956884079</v>
+      </c>
+      <c r="R569" t="n">
+        <v>814665494707</v>
+      </c>
+      <c r="S569" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T569" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U569" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V569" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W569" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X569" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y569" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z569" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA569" t="inlineStr"/>
+      <c r="AB569" t="inlineStr"/>
+      <c r="AC569" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD569" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE569" t="inlineStr"/>
+      <c r="AF569" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="AG569" t="inlineStr"/>
+      <c r="AH569" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI569" t="n">
+        <v>19353</v>
+      </c>
+      <c r="AJ569" t="inlineStr">
+        <is>
+          <t>276105</t>
+        </is>
+      </c>
+      <c r="AK569" t="inlineStr">
+        <is>
+          <t>2096</t>
+        </is>
+      </c>
+      <c r="AL569" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="n">
+        <v>16404</v>
+      </c>
+      <c r="B570" t="inlineStr"/>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>77****6258</t>
+        </is>
+      </c>
+      <c r="D570" t="n">
+        <v>8050</v>
+      </c>
+      <c r="E570" t="inlineStr"/>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>25-Jul-2026 12:29:38</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr"/>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>*8546</t>
+        </is>
+      </c>
+      <c r="M570" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N570" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O570" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P570" t="n">
+        <v>11000374938004</v>
+      </c>
+      <c r="Q570" t="n">
+        <v>1784962754414</v>
+      </c>
+      <c r="R570" t="n">
+        <v>150236443436</v>
+      </c>
+      <c r="S570" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T570" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U570" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V570" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W570" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X570" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y570" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z570" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA570" t="inlineStr"/>
+      <c r="AB570" t="inlineStr"/>
+      <c r="AC570" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD570" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE570" t="inlineStr"/>
+      <c r="AF570" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG570" t="inlineStr"/>
+      <c r="AH570" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI570" t="n">
+        <v>18546</v>
+      </c>
+      <c r="AJ570" t="inlineStr">
+        <is>
+          <t>267319</t>
+        </is>
+      </c>
+      <c r="AK570" t="inlineStr">
+        <is>
+          <t>2057</t>
+        </is>
+      </c>
+      <c r="AL570" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="n">
+        <v>17609</v>
+      </c>
+      <c r="B571" t="inlineStr"/>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>83****2537</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E571" t="inlineStr"/>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>25-Jul-2026 12:56:37</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr"/>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>PREKGUKG</t>
+        </is>
+      </c>
+      <c r="K571" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L571" t="inlineStr">
+        <is>
+          <t>*0328</t>
+        </is>
+      </c>
+      <c r="M571" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N571" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O571" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P571" t="n">
+        <v>11000374944254</v>
+      </c>
+      <c r="Q571" t="n">
+        <v>1784964385508</v>
+      </c>
+      <c r="R571" t="n">
+        <v>198902843986</v>
+      </c>
+      <c r="S571" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T571" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U571" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V571" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W571" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X571" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y571" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z571" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA571" t="inlineStr"/>
+      <c r="AB571" t="inlineStr"/>
+      <c r="AC571" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD571" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE571" t="inlineStr"/>
+      <c r="AF571" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SCHOOL MANAGEMENT ACCOUNT</t>
+        </is>
+      </c>
+      <c r="AG571" t="inlineStr"/>
+      <c r="AH571" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI571" t="n">
+        <v>20328</v>
+      </c>
+      <c r="AJ571" t="inlineStr">
+        <is>
+          <t>277548</t>
+        </is>
+      </c>
+      <c r="AK571" t="inlineStr">
+        <is>
+          <t>2065</t>
+        </is>
+      </c>
+      <c r="AL571" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="n">
+        <v>17524</v>
+      </c>
+      <c r="B572" t="inlineStr"/>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>63****8718</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E572" t="inlineStr"/>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>25-Jul-2026 13:32:31</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr"/>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L572" t="inlineStr">
+        <is>
+          <t>*0243</t>
+        </is>
+      </c>
+      <c r="M572" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N572" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O572" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P572" t="n">
+        <v>11000374952523</v>
+      </c>
+      <c r="Q572" t="n">
+        <v>1784966535315</v>
+      </c>
+      <c r="R572" t="n">
+        <v>441622965891</v>
+      </c>
+      <c r="S572" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T572" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U572" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V572" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W572" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X572" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y572" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z572" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA572" t="inlineStr"/>
+      <c r="AB572" t="inlineStr"/>
+      <c r="AC572" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD572" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE572" t="inlineStr"/>
+      <c r="AF572" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG572" t="inlineStr"/>
+      <c r="AH572" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI572" t="n">
+        <v>20243</v>
+      </c>
+      <c r="AJ572" t="inlineStr">
+        <is>
+          <t>272411</t>
+        </is>
+      </c>
+      <c r="AK572" t="inlineStr">
+        <is>
+          <t>2080</t>
+        </is>
+      </c>
+      <c r="AL572" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update fee collection with new payments
Add two new online payment transactions from 26-Jul-2026 and update fee collection records for students 16673 (PATAN SHAREEF) and 16398 (VINOOTHNA SINGAM). Update fees_collection, daywise_fees_collection, and merged_fee_collection files across all versions.
</commit_message>
<xml_diff>
--- a/output_data/atom_report_cleaned.xlsx
+++ b/output_data/atom_report_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL572"/>
+  <dimension ref="A1:AL574"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -90084,6 +90084,298 @@
         </is>
       </c>
     </row>
+    <row r="573">
+      <c r="A573" t="n">
+        <v>16673</v>
+      </c>
+      <c r="B573" t="inlineStr"/>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>90****3576</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>8400</v>
+      </c>
+      <c r="E573" t="inlineStr"/>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>26-Jul-2026 00:28:26</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr"/>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="K573" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L573" t="inlineStr">
+        <is>
+          <t>*8166</t>
+        </is>
+      </c>
+      <c r="M573" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N573" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O573" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P573" t="n">
+        <v>11000375016744</v>
+      </c>
+      <c r="Q573" t="n">
+        <v>1785005874009</v>
+      </c>
+      <c r="R573" t="n">
+        <v>653353524103</v>
+      </c>
+      <c r="S573" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T573" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U573" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V573" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W573" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X573" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y573" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z573" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA573" t="inlineStr"/>
+      <c r="AB573" t="inlineStr"/>
+      <c r="AC573" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD573" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE573" t="inlineStr"/>
+      <c r="AF573" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="AG573" t="inlineStr"/>
+      <c r="AH573" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI573" t="n">
+        <v>18166</v>
+      </c>
+      <c r="AJ573" t="inlineStr">
+        <is>
+          <t>271281</t>
+        </is>
+      </c>
+      <c r="AK573" t="inlineStr">
+        <is>
+          <t>2076</t>
+        </is>
+      </c>
+      <c r="AL573" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="n">
+        <v>16398</v>
+      </c>
+      <c r="B574" t="inlineStr"/>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>91****2954</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>9400</v>
+      </c>
+      <c r="E574" t="inlineStr"/>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>26-Jul-2026 14:17:35</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr"/>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>Vll</t>
+        </is>
+      </c>
+      <c r="K574" t="inlineStr">
+        <is>
+          <t>Rupees Only...</t>
+        </is>
+      </c>
+      <c r="L574" t="inlineStr">
+        <is>
+          <t>*8886</t>
+        </is>
+      </c>
+      <c r="M574" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="N574" t="n">
+        <v>753702</v>
+      </c>
+      <c r="O574" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="P574" t="n">
+        <v>11000375055101</v>
+      </c>
+      <c r="Q574" t="n">
+        <v>1785055641129</v>
+      </c>
+      <c r="R574" t="n">
+        <v>310058895026</v>
+      </c>
+      <c r="S574" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="T574" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="U574" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="V574" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="W574" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="X574" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="Y574" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="Z574" t="inlineStr">
+        <is>
+          <t>m**********@gmail.com</t>
+        </is>
+      </c>
+      <c r="AA574" t="inlineStr"/>
+      <c r="AB574" t="inlineStr"/>
+      <c r="AC574" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD574" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE574" t="inlineStr"/>
+      <c r="AF574" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN HIGH SCHOOL SSC</t>
+        </is>
+      </c>
+      <c r="AG574" t="inlineStr"/>
+      <c r="AH574" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="AI574" t="n">
+        <v>18886</v>
+      </c>
+      <c r="AJ574" t="inlineStr">
+        <is>
+          <t>274826</t>
+        </is>
+      </c>
+      <c r="AK574" t="inlineStr">
+        <is>
+          <t>2088</t>
+        </is>
+      </c>
+      <c r="AL574" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>